<commit_message>
patients: 5 SDS donors (Machado 2023) + PD54832 (TN-ET); populate can repopulate and prefer an assembly / projects (PD45534)
Trees from ~/Documents/TP53_HSPC_trees with the artificial 'zeros' outgroup dropped:
SDS2 PD43975 (38), SDS4 PD43293 (18), SDS6 PD45887 (27), SDS7 PD44706 (35), SDS8 PD42191 (10),
all GRCh37; PD54832 (49, GRCh37) with the short lo00NN tips renamed to PD54832b_lo00NN.
Placeholder colonies.tsv for each.

PD45534 colonies.tsv mixed 450 GRCh38 + 472 hs37d5 BAMs because populate took the first WGS
release of each colony. hsc_run.sh populate gains REPOPULATE=1 (old file kept as .bak.<ts>),
PREFER_ASSEMBLY (nst_links header path) and PREFER_PROJECTS (iRODS fallback: a tip in several
projects takes the first listed; tips with none of them are reported and left out).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -788,7 +788,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>mixed GRCh38/GRCh37</t>
+          <t>GRCh38 (repopulate)</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
@@ -819,7 +819,7 @@
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>colonies.tsv has 450 GRCh38 + 472 hs37d5 BAMs -&gt; pick one assembly per colony; old-pipeline results in ~/Documents/retrotransposons_sanger/results/PD45534</t>
+          <t>populate took the first WGS release per colony -&gt; 450 GRCh38 (proj 2450) + 472 hs37d5 (proj 2515); farm has 945 GRCh38 BAMs in 2450/3819/3838 -&gt; repopulate preferring GRCh38 (REPOPULATE=1 PREFER_ASSEMBLY / PREFER_PROJECTS). Old-pipeline results in ~/Documents/retrotransposons_sanger/results/PD45534</t>
         </is>
       </c>
     </row>
@@ -1429,13 +1429,21 @@
           <t>C141Y</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>PD43975</t>
+        </is>
+      </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>38 (tree tips)</t>
+        </is>
+      </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
           <t>not run</t>
@@ -1461,7 +1469,7 @@
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>no patients/ folder or tree yet</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv placeholder -&gt; hsc_run.sh populate</t>
         </is>
       </c>
     </row>
@@ -1491,13 +1499,21 @@
           <t>R273L</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>PD43293</t>
+        </is>
+      </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>18 (tree tips)</t>
+        </is>
+      </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
           <t>not run</t>
@@ -1523,7 +1539,7 @@
       </c>
       <c r="T15" s="3" t="inlineStr">
         <is>
-          <t>no patients/ folder or tree yet</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv placeholder -&gt; hsc_run.sh populate</t>
         </is>
       </c>
     </row>
@@ -1693,13 +1709,21 @@
           <t>E258K, G245S, I195F, R175H, V157F</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>PD45887</t>
+        </is>
+      </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>27 (tree tips)</t>
+        </is>
+      </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
           <t>not run</t>
@@ -1725,7 +1749,7 @@
       </c>
       <c r="T18" s="3" t="inlineStr">
         <is>
-          <t>no patients/ folder or tree yet</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv placeholder -&gt; hsc_run.sh populate</t>
         </is>
       </c>
     </row>
@@ -1755,13 +1779,21 @@
           <t>C275Y, V272M, G245S, Y205F, H179Q, V173M</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>PD44706</t>
+        </is>
+      </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>35 (tree tips)</t>
+        </is>
+      </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
           <t>not run</t>
@@ -1787,7 +1819,7 @@
       </c>
       <c r="T19" s="3" t="inlineStr">
         <is>
-          <t>no patients/ folder or tree yet</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv placeholder -&gt; hsc_run.sh populate</t>
         </is>
       </c>
     </row>
@@ -1817,13 +1849,21 @@
           <t>I254F+R248Q biallelic trunk (all 10 col)</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>PD42191</t>
+        </is>
+      </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>10 (tree tips)</t>
+        </is>
+      </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
           <t>not run</t>
@@ -1849,7 +1889,7 @@
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>no patients/ folder or tree yet</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv placeholder -&gt; hsc_run.sh populate</t>
         </is>
       </c>
     </row>
@@ -1969,13 +2009,21 @@
           <t>S215N</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr"/>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>PD54832</t>
+        </is>
+      </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>GRCh38?</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr"/>
+          <t>GRCh37</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>49 (tree tips)</t>
+        </is>
+      </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
           <t>not run</t>
@@ -2001,7 +2049,7 @@
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>no patients/ folder or tree yet; assembly unchecked</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv placeholder -&gt; hsc_run.sh populate; tips renamed lo00NN -&gt; PD54832b_lo00NN; tissue folder (peripheral_blood) not verified</t>
         </is>
       </c>
     </row>
@@ -2597,7 +2645,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-10 04:19</t>
+          <t>refreshed 2026-10-10 05:00</t>
         </is>
       </c>
     </row>
@@ -3037,7 +3085,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>mixed GRCh38/GRCh37</t>
+          <t>GRCh38 (repopulate)</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -3068,7 +3116,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>colonies.tsv has 450 GRCh38 + 472 hs37d5 BAMs -&gt; pick one assembly per colony; old-pipeline results in ~/Documents/retrotransposons_sanger/results/PD45534</t>
+          <t>populate took the first WGS release per colony -&gt; 450 GRCh38 (proj 2450) + 472 hs37d5 (proj 2515); farm has 945 GRCh38 BAMs in 2450/3819/3838 -&gt; repopulate preferring GRCh38 (REPOPULATE=1 PREFER_ASSEMBLY / PREFER_PROJECTS). Old-pipeline results in ~/Documents/retrotransposons_sanger/results/PD45534</t>
         </is>
       </c>
     </row>
@@ -3678,13 +3726,21 @@
           <t>C141Y</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>PD43975</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr">
         <is>
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>38 (tree tips)</t>
+        </is>
+      </c>
       <c r="I14" t="inlineStr">
         <is>
           <t>not run</t>
@@ -3710,7 +3766,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>no patients/ folder or tree yet</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv placeholder -&gt; hsc_run.sh populate</t>
         </is>
       </c>
     </row>
@@ -3740,13 +3796,21 @@
           <t>R273L</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>PD43293</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>18 (tree tips)</t>
+        </is>
+      </c>
       <c r="I15" t="inlineStr">
         <is>
           <t>not run</t>
@@ -3772,7 +3836,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>no patients/ folder or tree yet</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv placeholder -&gt; hsc_run.sh populate</t>
         </is>
       </c>
     </row>
@@ -3942,13 +4006,21 @@
           <t>E258K, G245S, I195F, R175H, V157F</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>PD45887</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr">
         <is>
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>27 (tree tips)</t>
+        </is>
+      </c>
       <c r="I18" t="inlineStr">
         <is>
           <t>not run</t>
@@ -3974,7 +4046,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>no patients/ folder or tree yet</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv placeholder -&gt; hsc_run.sh populate</t>
         </is>
       </c>
     </row>
@@ -4004,13 +4076,21 @@
           <t>C275Y, V272M, G245S, Y205F, H179Q, V173M</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>PD44706</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr">
         <is>
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>35 (tree tips)</t>
+        </is>
+      </c>
       <c r="I19" t="inlineStr">
         <is>
           <t>not run</t>
@@ -4036,7 +4116,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>no patients/ folder or tree yet</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv placeholder -&gt; hsc_run.sh populate</t>
         </is>
       </c>
     </row>
@@ -4066,13 +4146,21 @@
           <t>I254F+R248Q biallelic trunk (all 10 col)</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>PD42191</t>
+        </is>
+      </c>
       <c r="G20" t="inlineStr">
         <is>
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>10 (tree tips)</t>
+        </is>
+      </c>
       <c r="I20" t="inlineStr">
         <is>
           <t>not run</t>
@@ -4098,7 +4186,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>no patients/ folder or tree yet</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv placeholder -&gt; hsc_run.sh populate</t>
         </is>
       </c>
     </row>
@@ -4218,13 +4306,21 @@
           <t>S215N</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>PD54832</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>GRCh38?</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr"/>
+          <t>GRCh37</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>49 (tree tips)</t>
+        </is>
+      </c>
       <c r="I22" t="inlineStr">
         <is>
           <t>not run</t>
@@ -4250,7 +4346,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>no patients/ folder or tree yet; assembly unchecked</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv placeholder -&gt; hsc_run.sh populate; tips renamed lo00NN -&gt; PD54832b_lo00NN; tissue folder (peripheral_blood) not verified</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Transplant pairs are analysed as one unit: hsc_run.sh / pipeline.sh refuse a single PD id of a shared-tree folder; tracker keeps a unit's run columns in sync
hsc_run.sh patient_dir: a PD id that is one half of Pair<N>_<donor>_<recipient> (or
SDS5_PD42190_PD45888) dies naming the unit to submit instead. pipeline.sh submit (per-PD irods
route) refuses the same unless PT_ALLOW_SPLIT=1. run_tracker.py: farm status, run dir, commit,
results dir and sign-off are per run unit -- a hand edit on one row is copied to its partner.
Tracker: PD45534 settled on GRCh38 (922/922), populate results noted.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -521,7 +521,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Run unit</t>
+          <t>Run unit (analysed together)</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>GRCh38 (repopulate)</t>
+          <t>GRCh38</t>
         </is>
       </c>
       <c r="H4" s="2" t="n">
@@ -819,7 +819,7 @@
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>populate took the first WGS release per colony -&gt; 450 GRCh38 (proj 2450) + 472 hs37d5 (proj 2515); farm has 945 GRCh38 BAMs in 2450/3819/3838 -&gt; repopulate preferring GRCh38 (REPOPULATE=1 PREFER_ASSEMBLY / PREFER_PROJECTS). Old-pipeline results in ~/Documents/retrotransposons_sanger/results/PD45534</t>
+          <t>SETTLED 2026-10-10: repopulated preferring GRCh38 -&gt; all 922 colonies GRCh38 (450 proj 2450, 472 proj 3819; old mixed file kept as colonies.tsv.bak.20261010040433). Old-pipeline results in ~/Documents/retrotransposons_sanger/results/PD45534</t>
         </is>
       </c>
     </row>
@@ -1439,10 +1439,8 @@
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>38 (tree tips)</t>
-        </is>
+      <c r="H14" s="2" t="n">
+        <v>38</v>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
@@ -1469,7 +1467,7 @@
       </c>
       <c r="T14" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv placeholder -&gt; hsc_run.sh populate</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips)</t>
         </is>
       </c>
     </row>
@@ -1509,10 +1507,8 @@
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>18 (tree tips)</t>
-        </is>
+      <c r="H15" s="2" t="n">
+        <v>18</v>
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
@@ -1539,7 +1535,7 @@
       </c>
       <c r="T15" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv placeholder -&gt; hsc_run.sh populate</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips)</t>
         </is>
       </c>
     </row>
@@ -1579,10 +1575,8 @@
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>100 (tree tips)</t>
-        </is>
+      <c r="H16" s="2" t="n">
+        <v>48</v>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
@@ -1609,7 +1603,7 @@
       </c>
       <c r="T16" s="3" t="inlineStr">
         <is>
-          <t>one tree with PD45888; colonies.tsv placeholder</t>
+          <t>one tree with PD45888; colonies.tsv populated 2026-10-10 (100/100)</t>
         </is>
       </c>
     </row>
@@ -1649,10 +1643,8 @@
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>100 (tree tips)</t>
-        </is>
+      <c r="H17" s="2" t="n">
+        <v>52</v>
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
@@ -1679,7 +1671,7 @@
       </c>
       <c r="T17" s="3" t="inlineStr">
         <is>
-          <t>one tree with PD42190; colonies.tsv placeholder</t>
+          <t>one tree with PD42190; colonies.tsv populated 2026-10-10 (100/100)</t>
         </is>
       </c>
     </row>
@@ -1719,10 +1711,8 @@
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>27 (tree tips)</t>
-        </is>
+      <c r="H18" s="2" t="n">
+        <v>27</v>
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
@@ -1749,7 +1739,7 @@
       </c>
       <c r="T18" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv placeholder -&gt; hsc_run.sh populate</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips)</t>
         </is>
       </c>
     </row>
@@ -1789,10 +1779,8 @@
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>35 (tree tips)</t>
-        </is>
+      <c r="H19" s="2" t="n">
+        <v>35</v>
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
@@ -1819,7 +1807,7 @@
       </c>
       <c r="T19" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv placeholder -&gt; hsc_run.sh populate</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips)</t>
         </is>
       </c>
     </row>
@@ -1859,10 +1847,8 @@
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>10 (tree tips)</t>
-        </is>
+      <c r="H20" s="2" t="n">
+        <v>10</v>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
@@ -1889,7 +1875,7 @@
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv placeholder -&gt; hsc_run.sh populate</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips)</t>
         </is>
       </c>
     </row>
@@ -2019,10 +2005,8 @@
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>49 (tree tips)</t>
-        </is>
+      <c r="H22" s="2" t="n">
+        <v>49</v>
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
@@ -2049,7 +2033,7 @@
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv placeholder -&gt; hsc_run.sh populate; tips renamed lo00NN -&gt; PD54832b_lo00NN; tissue folder (peripheral_blood) not verified</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); tips renamed lo00NN -&gt; PD54832b_lo00NN; tissue folder (peripheral_blood) not verified</t>
         </is>
       </c>
     </row>
@@ -2085,10 +2069,8 @@
           <t>GRCh38</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>117 (tree tips)</t>
-        </is>
+      <c r="H23" s="2" t="n">
+        <v>117</v>
       </c>
       <c r="I23" s="4" t="inlineStr">
         <is>
@@ -2171,10 +2153,8 @@
           <t>GRCh38</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>83 (tree tips)</t>
-        </is>
+      <c r="H24" s="2" t="n">
+        <v>83</v>
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
@@ -2229,10 +2209,8 @@
           <t>GRCh38</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>81 (tree tips)</t>
-        </is>
+      <c r="H25" s="2" t="n">
+        <v>81</v>
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
@@ -2287,10 +2265,8 @@
           <t>GRCh38</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>123 (tree tips)</t>
-        </is>
+      <c r="H26" s="2" t="n">
+        <v>117</v>
       </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
@@ -2315,7 +2291,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T26" s="3" t="inlineStr"/>
+      <c r="T26" s="3" t="inlineStr">
+        <is>
+          <t>117/123 tips have a BAM: PD51634b (bulk?) and ch_lo0003/0007/0013/0026/0030 missing from the iRODS populate (not found, or in several projects) -- check the populate log before submitting</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2345,10 +2325,8 @@
           <t>GRCh38</t>
         </is>
       </c>
-      <c r="H27" s="2" t="inlineStr">
-        <is>
-          <t>163 (tree tips)</t>
-        </is>
+      <c r="H27" s="2" t="n">
+        <v>163</v>
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
@@ -2403,10 +2381,8 @@
           <t>GRCh38</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>35 (tree tips)</t>
-        </is>
+      <c r="H28" s="2" t="n">
+        <v>35</v>
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
@@ -2461,10 +2437,8 @@
           <t>GRCh38</t>
         </is>
       </c>
-      <c r="H29" s="2" t="inlineStr">
-        <is>
-          <t>75 (tree tips)</t>
-        </is>
+      <c r="H29" s="2" t="n">
+        <v>75</v>
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
@@ -2519,10 +2493,8 @@
           <t>GRCh38</t>
         </is>
       </c>
-      <c r="H30" s="2" t="inlineStr">
-        <is>
-          <t>55 (tree tips)</t>
-        </is>
+      <c r="H30" s="2" t="n">
+        <v>55</v>
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
@@ -2577,10 +2549,8 @@
           <t>GRCh38</t>
         </is>
       </c>
-      <c r="H31" s="2" t="inlineStr">
-        <is>
-          <t>102 (tree tips)</t>
-        </is>
+      <c r="H31" s="2" t="n">
+        <v>102</v>
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
@@ -2627,7 +2597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2645,7 +2615,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-10 05:00</t>
+          <t>refreshed 2026-10-10 05:07</t>
         </is>
       </c>
     </row>
@@ -2713,7 +2683,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>transplant pair</t>
+          <t>transplant pair (people)</t>
         </is>
       </c>
       <c r="B6" t="n">
@@ -2751,26 +2721,33 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Manual columns (edit here, they survive a rebuild): Farm run, Farm run dir, PEAR-TREE commit, Results dir, Review signed off, Notes.</t>
+          <t>Rows with the same Run unit (transplant donor + recipient, SDS5's two time points) are ONE run on one shared tree: Farm run, run dir, commit, results and sign-off are kept identical across them; editing one row updates the others. hsc_run.sh refuses to submit one PD id of a unit alone.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Automatic columns (rebuilt from ~/Documents/hsc_results): Colonies, Data local, Somatic rows, Tiers, Excluded, Reviewed (insertion_review verdicts), Review progress.</t>
+          <t>Manual columns (edit here, they survive a rebuild): Farm run, Farm run dir, PEAR-TREE commit, Results dir, Review signed off, Notes.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>A commit starting with '~' was inferred from dates, not recorded by the run; runs submitted after pipeline.sh started stamping PT_COMMIT into run.env show the real one.</t>
+          <t>Automatic columns (rebuilt from ~/Documents/hsc_results): Colonies, Data local, Somatic rows, Tiers, Excluded, Reviewed (insertion_review verdicts), Review progress.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>A commit starting with '~' was inferred from dates, not recorded by the run; runs submitted after pipeline.sh started stamping PT_COMMIT into run.env show the real one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>Rebuild: python3 cluster/run_tracker.py   (roster: patients/run_tracker.tsv)</t>
         </is>
@@ -2818,7 +2795,7 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Run unit</t>
+          <t>Run unit (analysed together)</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
@@ -3085,7 +3062,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>GRCh38 (repopulate)</t>
+          <t>GRCh38</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -3116,7 +3093,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>populate took the first WGS release per colony -&gt; 450 GRCh38 (proj 2450) + 472 hs37d5 (proj 2515); farm has 945 GRCh38 BAMs in 2450/3819/3838 -&gt; repopulate preferring GRCh38 (REPOPULATE=1 PREFER_ASSEMBLY / PREFER_PROJECTS). Old-pipeline results in ~/Documents/retrotransposons_sanger/results/PD45534</t>
+          <t>SETTLED 2026-10-10: repopulated preferring GRCh38 -&gt; all 922 colonies GRCh38 (450 proj 2450, 472 proj 3819; old mixed file kept as colonies.tsv.bak.20261010040433). Old-pipeline results in ~/Documents/retrotransposons_sanger/results/PD45534</t>
         </is>
       </c>
     </row>
@@ -3736,10 +3713,8 @@
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>38 (tree tips)</t>
-        </is>
+      <c r="H14" t="n">
+        <v>38</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -3766,7 +3741,7 @@
       </c>
       <c r="T14" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv placeholder -&gt; hsc_run.sh populate</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips)</t>
         </is>
       </c>
     </row>
@@ -3806,10 +3781,8 @@
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>18 (tree tips)</t>
-        </is>
+      <c r="H15" t="n">
+        <v>18</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -3836,7 +3809,7 @@
       </c>
       <c r="T15" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv placeholder -&gt; hsc_run.sh populate</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips)</t>
         </is>
       </c>
     </row>
@@ -3876,10 +3849,8 @@
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>100 (tree tips)</t>
-        </is>
+      <c r="H16" t="n">
+        <v>48</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -3906,7 +3877,7 @@
       </c>
       <c r="T16" t="inlineStr">
         <is>
-          <t>one tree with PD45888; colonies.tsv placeholder</t>
+          <t>one tree with PD45888; colonies.tsv populated 2026-10-10 (100/100)</t>
         </is>
       </c>
     </row>
@@ -3946,10 +3917,8 @@
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>100 (tree tips)</t>
-        </is>
+      <c r="H17" t="n">
+        <v>52</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -3976,7 +3945,7 @@
       </c>
       <c r="T17" t="inlineStr">
         <is>
-          <t>one tree with PD42190; colonies.tsv placeholder</t>
+          <t>one tree with PD42190; colonies.tsv populated 2026-10-10 (100/100)</t>
         </is>
       </c>
     </row>
@@ -4016,10 +3985,8 @@
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>27 (tree tips)</t>
-        </is>
+      <c r="H18" t="n">
+        <v>27</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -4046,7 +4013,7 @@
       </c>
       <c r="T18" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv placeholder -&gt; hsc_run.sh populate</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips)</t>
         </is>
       </c>
     </row>
@@ -4086,10 +4053,8 @@
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>35 (tree tips)</t>
-        </is>
+      <c r="H19" t="n">
+        <v>35</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -4116,7 +4081,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv placeholder -&gt; hsc_run.sh populate</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips)</t>
         </is>
       </c>
     </row>
@@ -4156,10 +4121,8 @@
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>10 (tree tips)</t>
-        </is>
+      <c r="H20" t="n">
+        <v>10</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -4186,7 +4149,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv placeholder -&gt; hsc_run.sh populate</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips)</t>
         </is>
       </c>
     </row>
@@ -4316,10 +4279,8 @@
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>49 (tree tips)</t>
-        </is>
+      <c r="H22" t="n">
+        <v>49</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
@@ -4346,7 +4307,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv placeholder -&gt; hsc_run.sh populate; tips renamed lo00NN -&gt; PD54832b_lo00NN; tissue folder (peripheral_blood) not verified</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); tips renamed lo00NN -&gt; PD54832b_lo00NN; tissue folder (peripheral_blood) not verified</t>
         </is>
       </c>
     </row>
@@ -4382,10 +4343,8 @@
           <t>GRCh38</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>117 (tree tips)</t>
-        </is>
+      <c r="H23" t="n">
+        <v>117</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -4468,10 +4427,8 @@
           <t>GRCh38</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>83 (tree tips)</t>
-        </is>
+      <c r="H24" t="n">
+        <v>83</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -4526,10 +4483,8 @@
           <t>GRCh38</t>
         </is>
       </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>81 (tree tips)</t>
-        </is>
+      <c r="H25" t="n">
+        <v>81</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -4584,10 +4539,8 @@
           <t>GRCh38</t>
         </is>
       </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>123 (tree tips)</t>
-        </is>
+      <c r="H26" t="n">
+        <v>117</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -4612,7 +4565,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T26" t="inlineStr"/>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>117/123 tips have a BAM: PD51634b (bulk?) and ch_lo0003/0007/0013/0026/0030 missing from the iRODS populate (not found, or in several projects) -- check the populate log before submitting</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -4642,10 +4599,8 @@
           <t>GRCh38</t>
         </is>
       </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>163 (tree tips)</t>
-        </is>
+      <c r="H27" t="n">
+        <v>163</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -4700,10 +4655,8 @@
           <t>GRCh38</t>
         </is>
       </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>35 (tree tips)</t>
-        </is>
+      <c r="H28" t="n">
+        <v>35</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -4758,10 +4711,8 @@
           <t>GRCh38</t>
         </is>
       </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>75 (tree tips)</t>
-        </is>
+      <c r="H29" t="n">
+        <v>75</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -4816,10 +4767,8 @@
           <t>GRCh38</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>55 (tree tips)</t>
-        </is>
+      <c r="H30" t="n">
+        <v>55</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -4874,10 +4823,8 @@
           <t>GRCh38</t>
         </is>
       </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>102 (tree tips)</t>
-        </is>
+      <c r="H31" t="n">
+        <v>102</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Run tracker: PD45886 now points at the hsc_foldback2 rerun (59f51a9)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -1925,12 +1925,12 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback/PD45886/PD45886</t>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD45886/PD45886</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>~5ed4f32 (inferred, main 2026-10-09, fold-back gate); first run ~59b75b6</t>
+          <t>59f51a9 (combine fold-back strand fix; discovery reused from hsc_foldback ~5ed4f32); first run ~59b75b6</t>
         </is>
       </c>
       <c r="L21" s="4" t="inlineStr">
@@ -1940,19 +1940,19 @@
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>PD45886_foldback/PD45886</t>
+          <t>PD45886_foldback2/PD45886</t>
         </is>
       </c>
       <c r="N21" s="2" t="n">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>7 / 10 / 63</t>
+          <t>7 / 10 / 56</t>
         </is>
       </c>
       <c r="P21" s="2" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="Q21" s="2" t="n">
         <v>0</v>
@@ -1969,7 +1969,7 @@
       </c>
       <c r="T21" s="3" t="inlineStr">
         <is>
-          <t>27 colonies, proj 2045; first run (489 private calls = cruciform artefacts) in ~/Documents/hsc_results/PD45886</t>
+          <t>27 colonies, proj 2045; 73 private calls (B 7, C 10), 2570 germline MEIs; first run (489 = cruciform artefacts) in ~/Documents/hsc_results/PD45886; hsc_foldback lost 217 germline (strand bug)</t>
         </is>
       </c>
     </row>
@@ -2615,7 +2615,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-10 05:07</t>
+          <t>refreshed 2026-10-10 12:19</t>
         </is>
       </c>
     </row>
@@ -4199,12 +4199,12 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback/PD45886/PD45886</t>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD45886/PD45886</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>~5ed4f32 (inferred, main 2026-10-09, fold-back gate); first run ~59b75b6</t>
+          <t>59f51a9 (combine fold-back strand fix; discovery reused from hsc_foldback ~5ed4f32); first run ~59b75b6</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
@@ -4214,19 +4214,19 @@
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>PD45886_foldback/PD45886</t>
+          <t>PD45886_foldback2/PD45886</t>
         </is>
       </c>
       <c r="N21" t="n">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>7 / 10 / 63</t>
+          <t>7 / 10 / 56</t>
         </is>
       </c>
       <c r="P21" t="n">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="Q21" t="n">
         <v>0</v>
@@ -4243,7 +4243,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>27 colonies, proj 2045; first run (489 private calls = cruciform artefacts) in ~/Documents/hsc_results/PD45886</t>
+          <t>27 colonies, proj 2045; 73 private calls (B 7, C 10), 2570 germline MEIs; first run (489 = cruciform artefacts) in ~/Documents/hsc_results/PD45886; hsc_foldback lost 217 germline (strand bug)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Run tracker: PD49229 needs a combine rerun after the dense-filter removal (not scheduled)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tracker" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_generated" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet name="tracker" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="_generated" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'tracker'!$A$1:$T$31</definedName>
@@ -669,11 +669,11 @@
       </c>
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R2" s="5" t="inlineStr">
-        <is>
-          <t>not started</t>
+        <v>6</v>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>30 %</t>
         </is>
       </c>
       <c r="S2" s="5" t="inlineStr">
@@ -1399,7 +1399,7 @@
       </c>
       <c r="T13" s="3" t="inlineStr">
         <is>
-          <t>722 colonies; annotated + joint table copied, no tree_fit / somatic.xlsx yet (annotate OOM at 32 GB -&gt; Rust RTE rerun)</t>
+          <t>NEEDS RERUN (not scheduled): combine predates the dense-region filter removal (2026-10-11), which dropped ~2.4% of germline MEIs here (3381 loci in 733 bins); 722 colonies; annotated + joint table copied, no tree_fit / somatic.xlsx yet (annotate OOM at 32 GB -&gt; Rust RTE rerun)</t>
         </is>
       </c>
     </row>
@@ -1955,11 +1955,11 @@
         <v>43</v>
       </c>
       <c r="Q21" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R21" s="5" t="inlineStr">
-        <is>
-          <t>not started</t>
+        <v>37</v>
+      </c>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>50 %</t>
         </is>
       </c>
       <c r="S21" s="5" t="inlineStr">
@@ -2615,7 +2615,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-10 12:19</t>
+          <t>refreshed 2026-10-11 07:43</t>
         </is>
       </c>
     </row>
@@ -2943,11 +2943,11 @@
       </c>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>30 %</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -3673,7 +3673,7 @@
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>722 colonies; annotated + joint table copied, no tree_fit / somatic.xlsx yet (annotate OOM at 32 GB -&gt; Rust RTE rerun)</t>
+          <t>NEEDS RERUN (not scheduled): combine predates the dense-region filter removal (2026-10-11), which dropped ~2.4% of germline MEIs here (3381 loci in 733 bins); 722 colonies; annotated + joint table copied, no tree_fit / somatic.xlsx yet (annotate OOM at 32 GB -&gt; Rust RTE rerun)</t>
         </is>
       </c>
     </row>
@@ -4229,11 +4229,11 @@
         <v>43</v>
       </c>
       <c r="Q21" t="n">
-        <v>0</v>
+        <v>37</v>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>50 %</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">

</xml_diff>

<commit_message>
Run tracker: PD56961 done on 3bb7d22 (hsc_foldback2); needs a combine rerun (predates dense-filter removal + supp-twin exclusion)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="tracker" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="_generated" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tracker" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="_generated" sheetId="3" state="hidden" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'tracker'!$A$1:$T$31</definedName>
@@ -2328,13 +2328,21 @@
       <c r="H27" s="2" t="n">
         <v>163</v>
       </c>
-      <c r="I27" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr"/>
-      <c r="K27" s="2" t="inlineStr"/>
+      <c r="I27" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD56961/PD56961</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>3bb7d22 (fold-back strand fix in; predates fa616a2 supp-twin exclusion + 9626905 dense-filter removal)</t>
+        </is>
+      </c>
       <c r="L27" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2351,7 +2359,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T27" s="3" t="inlineStr"/>
+      <c r="T27" s="3" t="inlineStr">
+        <is>
+          <t>NEEDS RERUN (not scheduled): combine (2026-10-10) predates the dense-region filter removal (9626905) and the supplementary-clip twin exclusion (fa616a2); 163/163 colonies discovered + genotyped, somatic.xlsx + tree_fit written 2026-10-11 06:37</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2615,7 +2627,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-11 07:43</t>
+          <t>refreshed 2026-10-11 09:14</t>
         </is>
       </c>
     </row>
@@ -2671,7 +2683,7 @@
         <v>9</v>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" t="n">
         <v>1</v>
@@ -2709,7 +2721,7 @@
         <v>30</v>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D7" t="n">
         <v>3</v>
@@ -4604,11 +4616,19 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
+          <t>done</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD56961/PD56961</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>3bb7d22 (fold-back strand fix in; predates fa616a2 supp-twin exclusion + 9626905 dense-filter removal)</t>
+        </is>
+      </c>
       <c r="L27" t="inlineStr">
         <is>
           <t>no</t>
@@ -4625,7 +4645,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T27" t="inlineStr"/>
+      <c r="T27" t="inlineStr">
+        <is>
+          <t>NEEDS RERUN (not scheduled): combine (2026-10-10) predates the dense-region filter removal (9626905) and the supplementary-clip twin exclusion (fa616a2); 163/163 colonies discovered + genotyped, somatic.xlsx + tree_fit written 2026-10-11 06:37</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">

</xml_diff>

<commit_message>
Run tracker: PD56961 results local (20 somatic rows, B/C/D 5/3/12)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -2343,17 +2343,35 @@
           <t>3bb7d22 (fold-back strand fix in; predates fa616a2 supp-twin exclusion + 9626905 dense-filter removal)</t>
         </is>
       </c>
-      <c r="L27" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M27" s="2" t="inlineStr"/>
-      <c r="N27" s="2" t="inlineStr"/>
-      <c r="O27" s="2" t="inlineStr"/>
-      <c r="P27" s="2" t="inlineStr"/>
-      <c r="Q27" s="2" t="inlineStr"/>
-      <c r="R27" s="2" t="inlineStr"/>
+      <c r="L27" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="inlineStr">
+        <is>
+          <t>PD56961</t>
+        </is>
+      </c>
+      <c r="N27" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>5 / 3 / 12</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="Q27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R27" s="5" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S27" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2627,7 +2645,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-11 09:14</t>
+          <t>refreshed 2026-10-11 09:15</t>
         </is>
       </c>
     </row>
@@ -2686,7 +2704,7 @@
         <v>2</v>
       </c>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -2724,7 +2742,7 @@
         <v>4</v>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
@@ -4631,15 +4649,33 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M27" t="inlineStr"/>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
-      <c r="P27" t="inlineStr"/>
-      <c r="Q27" t="inlineStr"/>
-      <c r="R27" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>PD56961</t>
+        </is>
+      </c>
+      <c r="N27" t="n">
+        <v>20</v>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>5 / 3 / 12</t>
+        </is>
+      </c>
+      <c r="P27" t="n">
+        <v>32</v>
+      </c>
+      <c r="Q27" t="n">
+        <v>0</v>
+      </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S27" t="inlineStr">
         <is>
           <t>no</t>

</xml_diff>

<commit_message>
Run tracker: PD51634 submitted on c72e5a6 (hsc_foldback2, jobs 915507-915515)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -2268,13 +2268,21 @@
       <c r="H26" s="2" t="n">
         <v>117</v>
       </c>
-      <c r="I26" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr"/>
-      <c r="K26" s="2" t="inlineStr"/>
+      <c r="I26" s="6" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD51634/PD51634</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>c72e5a6 (dense-filter removal + supp-twin exclusion in)</t>
+        </is>
+      </c>
       <c r="L26" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2293,7 +2301,7 @@
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>117/123 tips have a BAM: PD51634b (bulk?) and ch_lo0003/0007/0013/0026/0030 missing from the iRODS populate (not found, or in several projects) -- check the populate log before submitting</t>
+          <t>submitted 2026-10-11 08:16, LSF jobs 915507-915515, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD51634; 117/123 tips have a BAM: PD51634b (bulk?) and ch_lo0003/0007/0013/0026/0030 missing from the iRODS populate, run without them</t>
         </is>
       </c>
     </row>
@@ -2645,7 +2653,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-11 09:15</t>
+          <t>refreshed 2026-10-11 09:17</t>
         </is>
       </c>
     </row>
@@ -4574,11 +4582,19 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD51634/PD51634</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>c72e5a6 (dense-filter removal + supp-twin exclusion in)</t>
+        </is>
+      </c>
       <c r="L26" t="inlineStr">
         <is>
           <t>no</t>
@@ -4597,7 +4613,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>117/123 tips have a BAM: PD51634b (bulk?) and ch_lo0003/0007/0013/0026/0030 missing from the iRODS populate (not found, or in several projects) -- check the populate log before submitting</t>
+          <t>submitted 2026-10-11 08:16, LSF jobs 915507-915515, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD51634; 117/123 tips have a BAM: PD51634b (bulk?) and ch_lo0003/0007/0013/0026/0030 missing from the iRODS populate, run without them</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Run tracker: PD51634 done on c72e5a6 (hsc_foldback2), results local
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -1373,9 +1373,9 @@
           <t>~7d9e241 (inferred, hsc-deploy 2026-10-07); annotate rerun on 59b75b6 (Rust RTE)</t>
         </is>
       </c>
-      <c r="L13" s="6" t="inlineStr">
-        <is>
-          <t>partial</t>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
@@ -1383,13 +1383,23 @@
           <t>PD49229</t>
         </is>
       </c>
-      <c r="N13" s="2" t="inlineStr"/>
-      <c r="O13" s="2" t="inlineStr"/>
-      <c r="P13" s="2" t="inlineStr"/>
-      <c r="Q13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="n">
+        <v>237</v>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>16 / 188 / 33</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="Q13" s="2" t="n">
+        <v>220</v>
+      </c>
       <c r="R13" s="2" t="inlineStr">
         <is>
-          <t>no somatic table</t>
+          <t>92 %</t>
         </is>
       </c>
       <c r="S13" s="5" t="inlineStr">
@@ -2268,9 +2278,9 @@
       <c r="H26" s="2" t="n">
         <v>117</v>
       </c>
-      <c r="I26" s="6" t="inlineStr">
-        <is>
-          <t>running</t>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
@@ -2283,17 +2293,35 @@
           <t>c72e5a6 (dense-filter removal + supp-twin exclusion in)</t>
         </is>
       </c>
-      <c r="L26" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M26" s="2" t="inlineStr"/>
-      <c r="N26" s="2" t="inlineStr"/>
-      <c r="O26" s="2" t="inlineStr"/>
-      <c r="P26" s="2" t="inlineStr"/>
-      <c r="Q26" s="2" t="inlineStr"/>
-      <c r="R26" s="2" t="inlineStr"/>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>PD51634</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>3 / 4 / 54</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="Q26" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R26" s="5" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S26" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2301,7 +2329,7 @@
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>submitted 2026-10-11 08:16, LSF jobs 915507-915515, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD51634; 117/123 tips have a BAM: PD51634b (bulk?) and ch_lo0003/0007/0013/0026/0030 missing from the iRODS populate, run without them</t>
+          <t>submitted 2026-10-11 08:16, LSF jobs 915507-915515; done, results copied 2026-10-12 to ~/Documents/hsc_results/PD51634 (from /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD51634); 117/123 tips have a BAM: PD51634b (bulk?) and ch_lo0003/0007/0013/0026/0030 missing from the iRODS populate, run without them; tree_fit: 303 private, 2849 informative shared, 8348 germline</t>
         </is>
       </c>
     </row>
@@ -2653,7 +2681,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-11 09:17</t>
+          <t>refreshed 2026-10-12 05:36</t>
         </is>
       </c>
     </row>
@@ -2693,7 +2721,7 @@
         <v>3</v>
       </c>
       <c r="D4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -2709,10 +2737,10 @@
         <v>9</v>
       </c>
       <c r="C5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -2747,10 +2775,10 @@
         <v>30</v>
       </c>
       <c r="C7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
@@ -3687,7 +3715,7 @@
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
@@ -3695,13 +3723,23 @@
           <t>PD49229</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
+      <c r="N13" t="n">
+        <v>237</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>16 / 188 / 33</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>62</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>220</v>
+      </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>no somatic table</t>
+          <t>92 %</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -4582,7 +4620,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
@@ -4597,15 +4635,33 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M26" t="inlineStr"/>
-      <c r="N26" t="inlineStr"/>
-      <c r="O26" t="inlineStr"/>
-      <c r="P26" t="inlineStr"/>
-      <c r="Q26" t="inlineStr"/>
-      <c r="R26" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>PD51634</t>
+        </is>
+      </c>
+      <c r="N26" t="n">
+        <v>61</v>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>3 / 4 / 54</t>
+        </is>
+      </c>
+      <c r="P26" t="n">
+        <v>35</v>
+      </c>
+      <c r="Q26" t="n">
+        <v>0</v>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S26" t="inlineStr">
         <is>
           <t>no</t>
@@ -4613,7 +4669,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>submitted 2026-10-11 08:16, LSF jobs 915507-915515, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD51634; 117/123 tips have a BAM: PD51634b (bulk?) and ch_lo0003/0007/0013/0026/0030 missing from the iRODS populate, run without them</t>
+          <t>submitted 2026-10-11 08:16, LSF jobs 915507-915515; done, results copied 2026-10-12 to ~/Documents/hsc_results/PD51634 (from /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD51634); 117/123 tips have a BAM: PD51634b (bulk?) and ch_lo0003/0007/0013/0026/0030 missing from the iRODS populate, run without them; tree_fit: 303 private, 2849 informative shared, 8348 germline</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Run tracker: PD51632 submitted on 1fcdc92 (hsc_foldback2)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -2166,13 +2166,21 @@
       <c r="H24" s="2" t="n">
         <v>83</v>
       </c>
-      <c r="I24" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr"/>
-      <c r="K24" s="2" t="inlineStr"/>
+      <c r="I24" s="6" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD51632/PD51632</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L24" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2189,7 +2197,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T24" s="3" t="inlineStr"/>
+      <c r="T24" s="3" t="inlineStr">
+        <is>
+          <t>submitted 2026-10-12, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD51632; 83/83 colonies GRCh38</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2681,7 +2693,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-12 05:36</t>
+          <t>refreshed 2026-10-12 05:37</t>
         </is>
       </c>
     </row>
@@ -4508,11 +4520,19 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD51632/PD51632</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L24" t="inlineStr">
         <is>
           <t>no</t>
@@ -4529,7 +4549,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T24" t="inlineStr"/>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>submitted 2026-10-12, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD51632; 83/83 colonies GRCh38</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">

</xml_diff>

<commit_message>
Run tracker: PD51633 submitted on 1fcdc92 (hsc_foldback2, jobs 135445-135468)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -2234,13 +2234,21 @@
       <c r="H25" s="2" t="n">
         <v>81</v>
       </c>
-      <c r="I25" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J25" s="2" t="inlineStr"/>
-      <c r="K25" s="2" t="inlineStr"/>
+      <c r="I25" s="6" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD51633/PD51633</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L25" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2257,7 +2265,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T25" s="3" t="inlineStr"/>
+      <c r="T25" s="3" t="inlineStr">
+        <is>
+          <t>submitted 2026-10-12 19:09 (farm22-head2), LSF jobs 135445-135468, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD51633; 81/81 colonies GRCh38</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2413,11 +2425,11 @@
         <v>32</v>
       </c>
       <c r="Q27" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R27" s="5" t="inlineStr">
-        <is>
-          <t>not started</t>
+        <v>10</v>
+      </c>
+      <c r="R27" s="2" t="inlineStr">
+        <is>
+          <t>50 %</t>
         </is>
       </c>
       <c r="S27" s="5" t="inlineStr">
@@ -2693,7 +2705,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-12 05:37</t>
+          <t>refreshed 2026-10-12 20:10</t>
         </is>
       </c>
     </row>
@@ -4588,11 +4600,19 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr"/>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD51633/PD51633</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L25" t="inlineStr">
         <is>
           <t>no</t>
@@ -4609,7 +4629,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T25" t="inlineStr"/>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>submitted 2026-10-12 19:09 (farm22-head2), LSF jobs 135445-135468, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD51633; 81/81 colonies GRCh38</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -4765,11 +4789,11 @@
         <v>32</v>
       </c>
       <c r="Q27" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>50 %</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">

</xml_diff>

<commit_message>
Run tracker: PD51632 done + local; PD57332 and PD44706 (native GRCh37) submitted on 1fcdc92
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -1792,13 +1792,21 @@
       <c r="H19" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="I19" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr"/>
-      <c r="K19" s="2" t="inlineStr"/>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD44706/PD44706</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L19" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -1817,7 +1825,7 @@
       </c>
       <c r="T19" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips)</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-13 03:47 (farm22-head2), native GRCh37 (hg19.2bit + hs1-&gt;hg19 chain), LSF jobs 245034-245043, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD44706; 35/35 colonies</t>
         </is>
       </c>
     </row>
@@ -2166,9 +2174,9 @@
       <c r="H24" s="2" t="n">
         <v>83</v>
       </c>
-      <c r="I24" s="6" t="inlineStr">
-        <is>
-          <t>running</t>
+      <c r="I24" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
@@ -2181,17 +2189,35 @@
           <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
         </is>
       </c>
-      <c r="L24" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="inlineStr"/>
-      <c r="N24" s="2" t="inlineStr"/>
-      <c r="O24" s="2" t="inlineStr"/>
-      <c r="P24" s="2" t="inlineStr"/>
-      <c r="Q24" s="2" t="inlineStr"/>
-      <c r="R24" s="2" t="inlineStr"/>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>PD51632</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>2 / 1 / 27</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q24" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" s="5" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S24" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2199,7 +2225,7 @@
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>submitted 2026-10-12, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD51632; 83/83 colonies GRCh38</t>
+          <t>submitted 2026-10-12, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD51632; 83/83 colonies GRCh38; done; results copied 2026-10-13 to ~/Documents/hsc_results/PD51632; tree_fit: 222 private, 2035 informative shared, 9028 germline</t>
         </is>
       </c>
     </row>
@@ -2474,13 +2500,21 @@
       <c r="H28" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="I28" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr"/>
+      <c r="I28" s="6" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD57332/PD57332</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L28" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2497,7 +2531,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T28" s="3" t="inlineStr"/>
+      <c r="T28" s="3" t="inlineStr">
+        <is>
+          <t>submitted 2026-10-13 03:46 (farm22-head2), LSF jobs 244897-244907, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57332; 35/35 colonies GRCh38</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2705,7 +2743,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-12 20:10</t>
+          <t>refreshed 2026-10-13 04:48</t>
         </is>
       </c>
     </row>
@@ -2761,10 +2799,10 @@
         <v>9</v>
       </c>
       <c r="C5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -2799,10 +2837,10 @@
         <v>30</v>
       </c>
       <c r="C7" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
@@ -4158,11 +4196,19 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD44706/PD44706</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr">
         <is>
           <t>no</t>
@@ -4181,7 +4227,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips)</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-13 03:47 (farm22-head2), native GRCh37 (hg19.2bit + hs1-&gt;hg19 chain), LSF jobs 245034-245043, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD44706; 35/35 colonies</t>
         </is>
       </c>
     </row>
@@ -4532,7 +4578,7 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
@@ -4547,15 +4593,33 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr"/>
-      <c r="N24" t="inlineStr"/>
-      <c r="O24" t="inlineStr"/>
-      <c r="P24" t="inlineStr"/>
-      <c r="Q24" t="inlineStr"/>
-      <c r="R24" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>PD51632</t>
+        </is>
+      </c>
+      <c r="N24" t="n">
+        <v>30</v>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>2 / 1 / 27</t>
+        </is>
+      </c>
+      <c r="P24" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q24" t="n">
+        <v>0</v>
+      </c>
+      <c r="R24" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S24" t="inlineStr">
         <is>
           <t>no</t>
@@ -4563,7 +4627,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>submitted 2026-10-12, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD51632; 83/83 colonies GRCh38</t>
+          <t>submitted 2026-10-12, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD51632; 83/83 colonies GRCh38; done; results copied 2026-10-13 to ~/Documents/hsc_results/PD51632; tree_fit: 222 private, 2035 informative shared, 9028 germline</t>
         </is>
       </c>
     </row>
@@ -4840,11 +4904,19 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD57332/PD57332</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L28" t="inlineStr">
         <is>
           <t>no</t>
@@ -4861,7 +4933,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T28" t="inlineStr"/>
+      <c r="T28" t="inlineStr">
+        <is>
+          <t>submitted 2026-10-13 03:46 (farm22-head2), LSF jobs 244897-244907, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57332; 35/35 colonies GRCh38</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">

</xml_diff>

<commit_message>
Run tracker: PD51633, PD57332, PD44706 done on 1fcdc92, results local
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -1792,9 +1792,9 @@
       <c r="H19" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="I19" s="6" t="inlineStr">
-        <is>
-          <t>running</t>
+      <c r="I19" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -1807,17 +1807,35 @@
           <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
         </is>
       </c>
-      <c r="L19" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="inlineStr"/>
-      <c r="N19" s="2" t="inlineStr"/>
-      <c r="O19" s="2" t="inlineStr"/>
-      <c r="P19" s="2" t="inlineStr"/>
-      <c r="Q19" s="2" t="inlineStr"/>
-      <c r="R19" s="2" t="inlineStr"/>
+      <c r="L19" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>PD44706</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>4 / 3 / 53</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q19" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" s="5" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S19" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -1825,7 +1843,7 @@
       </c>
       <c r="T19" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-13 03:47 (farm22-head2), native GRCh37 (hg19.2bit + hs1-&gt;hg19 chain), LSF jobs 245034-245043, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD44706; 35/35 colonies</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-13 03:47 (farm22-head2), native GRCh37 (hg19.2bit + hs1-&gt;hg19 chain), LSF jobs 245034-245043, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD44706; 35/35 colonies; done; results copied 2026-10-13 to ~/Documents/hsc_results/PD44706; tree_fit: 119 private, 1063 informative shared, 8550 germline</t>
         </is>
       </c>
     </row>
@@ -2260,9 +2278,9 @@
       <c r="H25" s="2" t="n">
         <v>81</v>
       </c>
-      <c r="I25" s="6" t="inlineStr">
-        <is>
-          <t>running</t>
+      <c r="I25" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
@@ -2275,17 +2293,35 @@
           <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
         </is>
       </c>
-      <c r="L25" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M25" s="2" t="inlineStr"/>
-      <c r="N25" s="2" t="inlineStr"/>
-      <c r="O25" s="2" t="inlineStr"/>
-      <c r="P25" s="2" t="inlineStr"/>
-      <c r="Q25" s="2" t="inlineStr"/>
-      <c r="R25" s="2" t="inlineStr"/>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>PD51633</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>1 / 2 / 20</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q25" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R25" s="5" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S25" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2293,7 +2329,7 @@
       </c>
       <c r="T25" s="3" t="inlineStr">
         <is>
-          <t>submitted 2026-10-12 19:09 (farm22-head2), LSF jobs 135445-135468, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD51633; 81/81 colonies GRCh38</t>
+          <t>submitted 2026-10-12 19:09 (farm22-head2), LSF jobs 135445-135468, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD51633; 81/81 colonies GRCh38; done; results copied 2026-10-13 to ~/Documents/hsc_results/PD51633; tree_fit: 95 private, 2058 informative shared, 6183 germline</t>
         </is>
       </c>
     </row>
@@ -2500,9 +2536,9 @@
       <c r="H28" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="I28" s="6" t="inlineStr">
-        <is>
-          <t>running</t>
+      <c r="I28" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
@@ -2515,17 +2551,35 @@
           <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
         </is>
       </c>
-      <c r="L28" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M28" s="2" t="inlineStr"/>
-      <c r="N28" s="2" t="inlineStr"/>
-      <c r="O28" s="2" t="inlineStr"/>
-      <c r="P28" s="2" t="inlineStr"/>
-      <c r="Q28" s="2" t="inlineStr"/>
-      <c r="R28" s="2" t="inlineStr"/>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="inlineStr">
+        <is>
+          <t>PD57332</t>
+        </is>
+      </c>
+      <c r="N28" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>2 / 2 / 6</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q28" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R28" s="5" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S28" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2533,7 +2587,7 @@
       </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>submitted 2026-10-13 03:46 (farm22-head2), LSF jobs 244897-244907, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57332; 35/35 colonies GRCh38</t>
+          <t>submitted 2026-10-13 03:46 (farm22-head2), LSF jobs 244897-244907, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57332; 35/35 colonies GRCh38; done; results copied 2026-10-13 to ~/Documents/hsc_results/PD57332; tree_fit: 59 private, 1184 informative shared, 5502 germline</t>
         </is>
       </c>
     </row>
@@ -2743,7 +2797,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-13 04:48</t>
+          <t>refreshed 2026-10-13 17:06</t>
         </is>
       </c>
     </row>
@@ -2780,10 +2834,10 @@
         <v>18</v>
       </c>
       <c r="C4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -2799,10 +2853,10 @@
         <v>9</v>
       </c>
       <c r="C5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D5" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -2837,10 +2891,10 @@
         <v>30</v>
       </c>
       <c r="C7" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D7" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
@@ -4196,7 +4250,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -4211,15 +4265,33 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M19" t="inlineStr"/>
-      <c r="N19" t="inlineStr"/>
-      <c r="O19" t="inlineStr"/>
-      <c r="P19" t="inlineStr"/>
-      <c r="Q19" t="inlineStr"/>
-      <c r="R19" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>PD44706</t>
+        </is>
+      </c>
+      <c r="N19" t="n">
+        <v>60</v>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>4 / 3 / 53</t>
+        </is>
+      </c>
+      <c r="P19" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q19" t="n">
+        <v>0</v>
+      </c>
+      <c r="R19" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S19" t="inlineStr">
         <is>
           <t>no</t>
@@ -4227,7 +4299,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-13 03:47 (farm22-head2), native GRCh37 (hg19.2bit + hs1-&gt;hg19 chain), LSF jobs 245034-245043, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD44706; 35/35 colonies</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-13 03:47 (farm22-head2), native GRCh37 (hg19.2bit + hs1-&gt;hg19 chain), LSF jobs 245034-245043, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD44706; 35/35 colonies; done; results copied 2026-10-13 to ~/Documents/hsc_results/PD44706; tree_fit: 119 private, 1063 informative shared, 8550 germline</t>
         </is>
       </c>
     </row>
@@ -4664,7 +4736,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
@@ -4679,15 +4751,33 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M25" t="inlineStr"/>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr"/>
-      <c r="P25" t="inlineStr"/>
-      <c r="Q25" t="inlineStr"/>
-      <c r="R25" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>PD51633</t>
+        </is>
+      </c>
+      <c r="N25" t="n">
+        <v>23</v>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>1 / 2 / 20</t>
+        </is>
+      </c>
+      <c r="P25" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q25" t="n">
+        <v>0</v>
+      </c>
+      <c r="R25" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S25" t="inlineStr">
         <is>
           <t>no</t>
@@ -4695,7 +4785,7 @@
       </c>
       <c r="T25" t="inlineStr">
         <is>
-          <t>submitted 2026-10-12 19:09 (farm22-head2), LSF jobs 135445-135468, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD51633; 81/81 colonies GRCh38</t>
+          <t>submitted 2026-10-12 19:09 (farm22-head2), LSF jobs 135445-135468, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD51633; 81/81 colonies GRCh38; done; results copied 2026-10-13 to ~/Documents/hsc_results/PD51633; tree_fit: 95 private, 2058 informative shared, 6183 germline</t>
         </is>
       </c>
     </row>
@@ -4904,7 +4994,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
@@ -4919,15 +5009,33 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
-      <c r="O28" t="inlineStr"/>
-      <c r="P28" t="inlineStr"/>
-      <c r="Q28" t="inlineStr"/>
-      <c r="R28" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>PD57332</t>
+        </is>
+      </c>
+      <c r="N28" t="n">
+        <v>10</v>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>2 / 2 / 6</t>
+        </is>
+      </c>
+      <c r="P28" t="n">
+        <v>9</v>
+      </c>
+      <c r="Q28" t="n">
+        <v>0</v>
+      </c>
+      <c r="R28" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S28" t="inlineStr">
         <is>
           <t>no</t>
@@ -4935,7 +5043,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>submitted 2026-10-13 03:46 (farm22-head2), LSF jobs 244897-244907, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57332; 35/35 colonies GRCh38</t>
+          <t>submitted 2026-10-13 03:46 (farm22-head2), LSF jobs 244897-244907, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57332; 35/35 colonies GRCh38; done; results copied 2026-10-13 to ~/Documents/hsc_results/PD57332; tree_fit: 59 private, 1184 informative shared, 5502 germline</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Run tracker: PD57333/PD57334 done on 1fcdc92 (not yet local); PD57335 submitted
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -2229,11 +2229,11 @@
         <v>5</v>
       </c>
       <c r="Q24" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R24" s="5" t="inlineStr">
-        <is>
-          <t>not started</t>
+        <v>3</v>
+      </c>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t>10 %</t>
         </is>
       </c>
       <c r="S24" s="5" t="inlineStr">
@@ -2315,11 +2315,11 @@
         <v>13</v>
       </c>
       <c r="Q25" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R25" s="5" t="inlineStr">
-        <is>
-          <t>not started</t>
+        <v>2</v>
+      </c>
+      <c r="R25" s="2" t="inlineStr">
+        <is>
+          <t>8 %</t>
         </is>
       </c>
       <c r="S25" s="5" t="inlineStr">
@@ -2401,11 +2401,11 @@
         <v>35</v>
       </c>
       <c r="Q26" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R26" s="5" t="inlineStr">
-        <is>
-          <t>not started</t>
+        <v>7</v>
+      </c>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>11 %</t>
         </is>
       </c>
       <c r="S26" s="5" t="inlineStr">
@@ -2487,11 +2487,11 @@
         <v>32</v>
       </c>
       <c r="Q27" s="2" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="R27" s="2" t="inlineStr">
         <is>
-          <t>50 %</t>
+          <t>80 %</t>
         </is>
       </c>
       <c r="S27" s="5" t="inlineStr">
@@ -2573,11 +2573,11 @@
         <v>9</v>
       </c>
       <c r="Q28" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R28" s="5" t="inlineStr">
-        <is>
-          <t>not started</t>
+        <v>4</v>
+      </c>
+      <c r="R28" s="2" t="inlineStr">
+        <is>
+          <t>40 %</t>
         </is>
       </c>
       <c r="S28" s="5" t="inlineStr">
@@ -2622,30 +2622,50 @@
       <c r="H29" s="2" t="n">
         <v>75</v>
       </c>
-      <c r="I29" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J29" s="2" t="inlineStr"/>
-      <c r="K29" s="2" t="inlineStr"/>
-      <c r="L29" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>done (results not yet copied)</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD57333/PD57333</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
+      <c r="L29" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="inlineStr">
+        <is>
+          <t>PD57333</t>
+        </is>
+      </c>
       <c r="N29" s="2" t="inlineStr"/>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
       <c r="Q29" s="2" t="inlineStr"/>
-      <c r="R29" s="2" t="inlineStr"/>
+      <c r="R29" s="2" t="inlineStr">
+        <is>
+          <t>no somatic table</t>
+        </is>
+      </c>
       <c r="S29" s="5" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="T29" s="3" t="inlineStr"/>
+      <c r="T29" s="3" t="inlineStr">
+        <is>
+          <t>submitted ~2026-10-13 (job IDs not recorded); done 2026-10-15, results in /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57333; 75/75 colonies GRCh38</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2678,13 +2698,21 @@
       <c r="H30" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="I30" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J30" s="2" t="inlineStr"/>
-      <c r="K30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>done (results not yet copied)</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD57334/PD57334</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L30" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2701,7 +2729,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T30" s="3" t="inlineStr"/>
+      <c r="T30" s="3" t="inlineStr">
+        <is>
+          <t>submitted ~2026-10-13 (job IDs not recorded); done 2026-10-15, results in /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57334; 55/55 colonies GRCh38</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2734,13 +2766,21 @@
       <c r="H31" s="2" t="n">
         <v>102</v>
       </c>
-      <c r="I31" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="inlineStr"/>
-      <c r="K31" s="2" t="inlineStr"/>
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD57335/PD57335</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L31" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2757,7 +2797,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T31" s="3" t="inlineStr"/>
+      <c r="T31" s="3" t="inlineStr">
+        <is>
+          <t>submitted 2026-10-15 (job IDs not recorded), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57335; 102/102 colonies GRCh38</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:T31"/>
@@ -2797,7 +2841,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-13 17:06</t>
+          <t>refreshed 2026-10-15 06:24</t>
         </is>
       </c>
     </row>
@@ -4685,11 +4729,11 @@
         <v>5</v>
       </c>
       <c r="Q24" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>10 %</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -4771,11 +4815,11 @@
         <v>13</v>
       </c>
       <c r="Q25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>8 %</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -4857,11 +4901,11 @@
         <v>35</v>
       </c>
       <c r="Q26" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>11 %</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -4943,11 +4987,11 @@
         <v>32</v>
       </c>
       <c r="Q27" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>50 %</t>
+          <t>80 %</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
@@ -5029,11 +5073,11 @@
         <v>9</v>
       </c>
       <c r="Q28" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>40 %</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -5080,28 +5124,48 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
+          <t>done (results not yet copied)</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD57333/PD57333</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M29" t="inlineStr"/>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>PD57333</t>
+        </is>
+      </c>
       <c r="N29" t="inlineStr"/>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="inlineStr"/>
       <c r="Q29" t="inlineStr"/>
-      <c r="R29" t="inlineStr"/>
+      <c r="R29" t="inlineStr">
+        <is>
+          <t>no somatic table</t>
+        </is>
+      </c>
       <c r="S29" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="T29" t="inlineStr"/>
+      <c r="T29" t="inlineStr">
+        <is>
+          <t>submitted ~2026-10-13 (job IDs not recorded); done 2026-10-15, results in /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57333; 75/75 colonies GRCh38</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -5136,11 +5200,19 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
+          <t>done (results not yet copied)</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD57334/PD57334</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L30" t="inlineStr">
         <is>
           <t>no</t>
@@ -5157,7 +5229,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T30" t="inlineStr"/>
+      <c r="T30" t="inlineStr">
+        <is>
+          <t>submitted ~2026-10-13 (job IDs not recorded); done 2026-10-15, results in /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57334; 55/55 colonies GRCh38</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5192,11 +5268,19 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD57335/PD57335</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L31" t="inlineStr">
         <is>
           <t>no</t>
@@ -5213,7 +5297,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T31" t="inlineStr"/>
+      <c r="T31" t="inlineStr">
+        <is>
+          <t>submitted 2026-10-15 (job IDs not recorded), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57335; 102/102 colonies GRCh38</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Run tracker: PD57335 LSF jobs 699021-699042
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -2799,7 +2799,7 @@
       </c>
       <c r="T31" s="3" t="inlineStr">
         <is>
-          <t>submitted 2026-10-15 (job IDs not recorded), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57335; 102/102 colonies GRCh38</t>
+          <t>submitted 2026-10-15 05:24, LSF jobs 699021-699042, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57335; 102/102 colonies GRCh38</t>
         </is>
       </c>
     </row>
@@ -2841,7 +2841,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-15 06:24</t>
+          <t>refreshed 2026-10-15 06:25</t>
         </is>
       </c>
     </row>
@@ -5299,7 +5299,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>submitted 2026-10-15 (job IDs not recorded), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57335; 102/102 colonies GRCh38</t>
+          <t>submitted 2026-10-15 05:24, LSF jobs 699021-699042, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57335; 102/102 colonies GRCh38</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Run tracker: SDS1/SDS3/SDS9 colonies.tsv populated (GRCh37), ready to submit
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -3129,10 +3129,8 @@
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H39" s="2" t="inlineStr">
-        <is>
-          <t>18 (tree tips)</t>
-        </is>
+      <c r="H39" s="2" t="n">
+        <v>18</v>
       </c>
       <c r="I39" s="5" t="inlineStr">
         <is>
@@ -3159,7 +3157,7 @@
       </c>
       <c r="T39" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv is a PLACEHOLDER: needs hsc_run.sh populate on the farm before submit</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 18/18 tips, all proj 2045; ready to submit</t>
         </is>
       </c>
     </row>
@@ -3195,10 +3193,8 @@
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H40" s="2" t="inlineStr">
-        <is>
-          <t>23 (tree tips)</t>
-        </is>
+      <c r="H40" s="2" t="n">
+        <v>23</v>
       </c>
       <c r="I40" s="5" t="inlineStr">
         <is>
@@ -3225,7 +3221,7 @@
       </c>
       <c r="T40" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv is a PLACEHOLDER: needs hsc_run.sh populate on the farm before submit</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 23/23 tips, all proj 2045; ready to submit</t>
         </is>
       </c>
     </row>
@@ -3261,10 +3257,8 @@
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>27 (tree tips)</t>
-        </is>
+      <c r="H41" s="2" t="n">
+        <v>27</v>
       </c>
       <c r="I41" s="5" t="inlineStr">
         <is>
@@ -3291,7 +3285,7 @@
       </c>
       <c r="T41" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv is a PLACEHOLDER: needs hsc_run.sh populate on the farm before submit</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 27/27 tips, all proj 2045; ready to submit</t>
         </is>
       </c>
     </row>
@@ -3923,9 +3917,9 @@
           <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
         </is>
       </c>
-      <c r="L49" s="6" t="inlineStr">
-        <is>
-          <t>partial</t>
+      <c r="L49" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="M49" s="2" t="inlineStr">
@@ -3933,13 +3927,23 @@
           <t>PD57333</t>
         </is>
       </c>
-      <c r="N49" s="2" t="inlineStr"/>
-      <c r="O49" s="2" t="inlineStr"/>
-      <c r="P49" s="2" t="inlineStr"/>
-      <c r="Q49" s="2" t="inlineStr"/>
-      <c r="R49" s="2" t="inlineStr">
-        <is>
-          <t>no somatic table</t>
+      <c r="N49" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="O49" s="2" t="inlineStr">
+        <is>
+          <t>1 / 2 / 43</t>
+        </is>
+      </c>
+      <c r="P49" s="2" t="n">
+        <v>115</v>
+      </c>
+      <c r="Q49" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R49" s="5" t="inlineStr">
+        <is>
+          <t>not started</t>
         </is>
       </c>
       <c r="S49" s="5" t="inlineStr">
@@ -4145,7 +4149,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-15 06:53</t>
+          <t>refreshed 2026-10-16 04:58</t>
         </is>
       </c>
     </row>
@@ -4204,7 +4208,7 @@
         <v>6</v>
       </c>
       <c r="D5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -4280,7 +4284,7 @@
         <v>9</v>
       </c>
       <c r="D9" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -6971,10 +6975,8 @@
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>18 (tree tips)</t>
-        </is>
+      <c r="H39" t="n">
+        <v>18</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
@@ -7001,7 +7003,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv is a PLACEHOLDER: needs hsc_run.sh populate on the farm before submit</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 18/18 tips, all proj 2045; ready to submit</t>
         </is>
       </c>
     </row>
@@ -7037,10 +7039,8 @@
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>23 (tree tips)</t>
-        </is>
+      <c r="H40" t="n">
+        <v>23</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -7067,7 +7067,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv is a PLACEHOLDER: needs hsc_run.sh populate on the farm before submit</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 23/23 tips, all proj 2045; ready to submit</t>
         </is>
       </c>
     </row>
@@ -7103,10 +7103,8 @@
           <t>GRCh37</t>
         </is>
       </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>27 (tree tips)</t>
-        </is>
+      <c r="H41" t="n">
+        <v>27</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -7133,7 +7131,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv is a PLACEHOLDER: needs hsc_run.sh populate on the farm before submit</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 27/27 tips, all proj 2045; ready to submit</t>
         </is>
       </c>
     </row>
@@ -7767,7 +7765,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
@@ -7775,13 +7773,23 @@
           <t>PD57333</t>
         </is>
       </c>
-      <c r="N49" t="inlineStr"/>
-      <c r="O49" t="inlineStr"/>
-      <c r="P49" t="inlineStr"/>
-      <c r="Q49" t="inlineStr"/>
+      <c r="N49" t="n">
+        <v>46</v>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>1 / 2 / 43</t>
+        </is>
+      </c>
+      <c r="P49" t="n">
+        <v>115</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>0</v>
+      </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>no somatic table</t>
+          <t>not started</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">

</xml_diff>

<commit_message>
Run tracker: PD57333/PD57334 local; PD43975 + PD54832 (native GRCh37) submitted on 1fcdc92
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -2540,13 +2540,21 @@
       <c r="H31" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="I31" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J31" s="2" t="inlineStr"/>
-      <c r="K31" s="2" t="inlineStr"/>
+      <c r="I31" s="6" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD43975/PD43975</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L31" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2565,7 +2573,7 @@
       </c>
       <c r="T31" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips)</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-16 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43975; 38/38 colonies</t>
         </is>
       </c>
     </row>
@@ -3324,13 +3332,21 @@
       <c r="H42" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="I42" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J42" s="2" t="inlineStr"/>
-      <c r="K42" s="2" t="inlineStr"/>
+      <c r="I42" s="6" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD54832/PD54832</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L42" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -3349,7 +3365,7 @@
       </c>
       <c r="T42" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); tips renamed lo00NN -&gt; PD54832b_lo00NN; tissue folder (peripheral_blood) not verified</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); tips renamed lo00NN -&gt; PD54832b_lo00NN; tissue folder (peripheral_blood) not verified; submitted 2026-10-16 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD54832; 49/49 colonies</t>
         </is>
       </c>
     </row>
@@ -3902,9 +3918,9 @@
       <c r="H49" s="2" t="n">
         <v>75</v>
       </c>
-      <c r="I49" s="2" t="inlineStr">
-        <is>
-          <t>done (results not yet copied)</t>
+      <c r="I49" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
@@ -3953,7 +3969,7 @@
       </c>
       <c r="T49" s="3" t="inlineStr">
         <is>
-          <t>submitted ~2026-10-13 (job IDs not recorded); done 2026-10-15, results in /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57333; 75/75 colonies GRCh38</t>
+          <t>submitted ~2026-10-13 (job IDs not recorded); done 2026-10-15, results in /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57333; 75/75 colonies GRCh38; results copied 2026-10-16 to ~/Documents/hsc_results/PD57333; tree_fit: 234 private, 2010 informative shared, 8077 germline</t>
         </is>
       </c>
     </row>
@@ -3988,9 +4004,9 @@
       <c r="H50" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="I50" s="2" t="inlineStr">
-        <is>
-          <t>done (results not yet copied)</t>
+      <c r="I50" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="J50" s="2" t="inlineStr">
@@ -4039,7 +4055,7 @@
       </c>
       <c r="T50" s="3" t="inlineStr">
         <is>
-          <t>submitted ~2026-10-13 (job IDs not recorded); done 2026-10-15, results in /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57334; 55/55 colonies GRCh38</t>
+          <t>submitted ~2026-10-13 (job IDs not recorded); done 2026-10-15, results in /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57334; 55/55 colonies GRCh38; results copied 2026-10-15 to ~/Documents/hsc_results/PD57334; tree_fit: 328 private, 2093 informative shared, 7410 germline</t>
         </is>
       </c>
     </row>
@@ -4205,7 +4221,7 @@
         <v>9</v>
       </c>
       <c r="C5" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D5" t="n">
         <v>8</v>
@@ -4281,7 +4297,7 @@
         <v>50</v>
       </c>
       <c r="C9" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D9" t="n">
         <v>12</v>
@@ -6388,11 +6404,19 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J31" t="inlineStr"/>
-      <c r="K31" t="inlineStr"/>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD43975/PD43975</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L31" t="inlineStr">
         <is>
           <t>no</t>
@@ -6411,7 +6435,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips)</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-16 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43975; 38/38 colonies</t>
         </is>
       </c>
     </row>
@@ -7172,11 +7196,19 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J42" t="inlineStr"/>
-      <c r="K42" t="inlineStr"/>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD54832/PD54832</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L42" t="inlineStr">
         <is>
           <t>no</t>
@@ -7195,7 +7227,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); tips renamed lo00NN -&gt; PD54832b_lo00NN; tissue folder (peripheral_blood) not verified</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); tips renamed lo00NN -&gt; PD54832b_lo00NN; tissue folder (peripheral_blood) not verified; submitted 2026-10-16 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD54832; 49/49 colonies</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7782,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>done (results not yet copied)</t>
+          <t>done</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
@@ -7799,7 +7831,7 @@
       </c>
       <c r="T49" t="inlineStr">
         <is>
-          <t>submitted ~2026-10-13 (job IDs not recorded); done 2026-10-15, results in /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57333; 75/75 colonies GRCh38</t>
+          <t>submitted ~2026-10-13 (job IDs not recorded); done 2026-10-15, results in /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57333; 75/75 colonies GRCh38; results copied 2026-10-16 to ~/Documents/hsc_results/PD57333; tree_fit: 234 private, 2010 informative shared, 8077 germline</t>
         </is>
       </c>
     </row>
@@ -7836,7 +7868,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>done (results not yet copied)</t>
+          <t>done</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
@@ -7885,7 +7917,7 @@
       </c>
       <c r="T50" t="inlineStr">
         <is>
-          <t>submitted ~2026-10-13 (job IDs not recorded); done 2026-10-15, results in /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57334; 55/55 colonies GRCh38</t>
+          <t>submitted ~2026-10-13 (job IDs not recorded); done 2026-10-15, results in /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57334; 55/55 colonies GRCh38; results copied 2026-10-15 to ~/Documents/hsc_results/PD57334; tree_fit: 328 private, 2093 informative shared, 7410 germline</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Run tracker: PD43975 + PD54832 done on farm (not yet local)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -2540,9 +2540,9 @@
       <c r="H31" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="I31" s="6" t="inlineStr">
-        <is>
-          <t>running</t>
+      <c r="I31" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
@@ -2573,7 +2573,7 @@
       </c>
       <c r="T31" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-16 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43975; 38/38 colonies</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-16 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43975; 38/38 colonies; done on farm 2026-10-17</t>
         </is>
       </c>
     </row>
@@ -3332,9 +3332,9 @@
       <c r="H42" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="I42" s="6" t="inlineStr">
-        <is>
-          <t>running</t>
+      <c r="I42" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="J42" s="2" t="inlineStr">
@@ -3365,7 +3365,7 @@
       </c>
       <c r="T42" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); tips renamed lo00NN -&gt; PD54832b_lo00NN; tissue folder (peripheral_blood) not verified; submitted 2026-10-16 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD54832; 49/49 colonies</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); tips renamed lo00NN -&gt; PD54832b_lo00NN; tissue folder (peripheral_blood) not verified; submitted 2026-10-16 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD54832; 49/49 colonies; done on farm 2026-10-17</t>
         </is>
       </c>
     </row>
@@ -3783,11 +3783,11 @@
         <v>32</v>
       </c>
       <c r="Q47" s="2" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="R47" s="2" t="inlineStr">
         <is>
-          <t>80 %</t>
+          <t>95 %</t>
         </is>
       </c>
       <c r="S47" s="5" t="inlineStr">
@@ -3869,11 +3869,11 @@
         <v>9</v>
       </c>
       <c r="Q48" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="R48" s="2" t="inlineStr">
-        <is>
-          <t>40 %</t>
+        <v>10</v>
+      </c>
+      <c r="R48" s="4" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="S48" s="5" t="inlineStr">
@@ -3955,11 +3955,11 @@
         <v>115</v>
       </c>
       <c r="Q49" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R49" s="5" t="inlineStr">
-        <is>
-          <t>not started</t>
+        <v>46</v>
+      </c>
+      <c r="R49" s="4" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="S49" s="5" t="inlineStr">
@@ -4041,11 +4041,11 @@
         <v>58</v>
       </c>
       <c r="Q50" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R50" s="5" t="inlineStr">
-        <is>
-          <t>not started</t>
+        <v>114</v>
+      </c>
+      <c r="R50" s="4" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="S50" s="5" t="inlineStr">
@@ -4165,7 +4165,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-16 04:58</t>
+          <t>refreshed 2026-10-17 09:26</t>
         </is>
       </c>
     </row>
@@ -4202,7 +4202,7 @@
         <v>18</v>
       </c>
       <c r="C4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D4" t="n">
         <v>5</v>
@@ -4259,7 +4259,7 @@
         <v>11</v>
       </c>
       <c r="C7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D7" t="n">
         <v>2</v>
@@ -4297,7 +4297,7 @@
         <v>50</v>
       </c>
       <c r="C9" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D9" t="n">
         <v>12</v>
@@ -6404,7 +6404,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
@@ -6435,7 +6435,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-16 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43975; 38/38 colonies</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-16 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43975; 38/38 colonies; done on farm 2026-10-17</t>
         </is>
       </c>
     </row>
@@ -7196,7 +7196,7 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
@@ -7227,7 +7227,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); tips renamed lo00NN -&gt; PD54832b_lo00NN; tissue folder (peripheral_blood) not verified; submitted 2026-10-16 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD54832; 49/49 colonies</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); tips renamed lo00NN -&gt; PD54832b_lo00NN; tissue folder (peripheral_blood) not verified; submitted 2026-10-16 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD54832; 49/49 colonies; done on farm 2026-10-17</t>
         </is>
       </c>
     </row>
@@ -7645,11 +7645,11 @@
         <v>32</v>
       </c>
       <c r="Q47" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>80 %</t>
+          <t>95 %</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
@@ -7731,11 +7731,11 @@
         <v>9</v>
       </c>
       <c r="Q48" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>40 %</t>
+          <t>complete</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
@@ -7817,11 +7817,11 @@
         <v>115</v>
       </c>
       <c r="Q49" t="n">
-        <v>0</v>
+        <v>46</v>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>complete</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
@@ -7903,11 +7903,11 @@
         <v>58</v>
       </c>
       <c r="Q50" t="n">
-        <v>0</v>
+        <v>114</v>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>complete</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">

</xml_diff>

<commit_message>
Run tracker: PD43975, PD54832, PD57335 local; PD45887, PD42191, PD43293 (native GRCh37) submitted on 1fcdc92
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -2555,17 +2555,35 @@
           <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
         </is>
       </c>
-      <c r="L31" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M31" s="2" t="inlineStr"/>
-      <c r="N31" s="2" t="inlineStr"/>
-      <c r="O31" s="2" t="inlineStr"/>
-      <c r="P31" s="2" t="inlineStr"/>
-      <c r="Q31" s="2" t="inlineStr"/>
-      <c r="R31" s="2" t="inlineStr"/>
+      <c r="L31" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>PD43975</t>
+        </is>
+      </c>
+      <c r="N31" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>1 / 1 / 23</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q31" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R31" s="5" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S31" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2573,7 +2591,7 @@
       </c>
       <c r="T31" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-16 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43975; 38/38 colonies; done on farm 2026-10-17</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-16 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43975; 38/38 colonies; done on farm 2026-10-17; results copied 2026-10-17 to ~/Documents/hsc_results/PD43975</t>
         </is>
       </c>
     </row>
@@ -2616,13 +2634,21 @@
       <c r="H32" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="I32" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J32" s="2" t="inlineStr"/>
-      <c r="K32" s="2" t="inlineStr"/>
+      <c r="I32" s="6" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD43293/PD43293</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L32" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2641,7 +2667,7 @@
       </c>
       <c r="T32" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips)</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43293</t>
         </is>
       </c>
     </row>
@@ -2820,13 +2846,21 @@
       <c r="H35" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="I35" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J35" s="2" t="inlineStr"/>
-      <c r="K35" s="2" t="inlineStr"/>
+      <c r="I35" s="6" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD45887/PD45887</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L35" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2845,7 +2879,7 @@
       </c>
       <c r="T35" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips)</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD45887</t>
         </is>
       </c>
     </row>
@@ -2982,13 +3016,21 @@
       <c r="H37" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="I37" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J37" s="2" t="inlineStr"/>
-      <c r="K37" s="2" t="inlineStr"/>
+      <c r="I37" s="6" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD42191/PD42191</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L37" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -3007,7 +3049,7 @@
       </c>
       <c r="T37" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips)</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD42191</t>
         </is>
       </c>
     </row>
@@ -3347,17 +3389,35 @@
           <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
         </is>
       </c>
-      <c r="L42" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M42" s="2" t="inlineStr"/>
-      <c r="N42" s="2" t="inlineStr"/>
-      <c r="O42" s="2" t="inlineStr"/>
-      <c r="P42" s="2" t="inlineStr"/>
-      <c r="Q42" s="2" t="inlineStr"/>
-      <c r="R42" s="2" t="inlineStr"/>
+      <c r="L42" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M42" s="2" t="inlineStr">
+        <is>
+          <t>PD54832</t>
+        </is>
+      </c>
+      <c r="N42" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>0 / 0 / 19</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q42" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R42" s="5" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S42" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -3365,7 +3425,7 @@
       </c>
       <c r="T42" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); tips renamed lo00NN -&gt; PD54832b_lo00NN; tissue folder (peripheral_blood) not verified; submitted 2026-10-16 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD54832; 49/49 colonies; done on farm 2026-10-17</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); tips renamed lo00NN -&gt; PD54832b_lo00NN; tissue folder (peripheral_blood) not verified; submitted 2026-10-16 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD54832; 49/49 colonies; done on farm 2026-10-17; results copied 2026-10-17 to ~/Documents/hsc_results/PD54832</t>
         </is>
       </c>
     </row>
@@ -4090,9 +4150,9 @@
       <c r="H51" s="2" t="n">
         <v>102</v>
       </c>
-      <c r="I51" s="6" t="inlineStr">
-        <is>
-          <t>running</t>
+      <c r="I51" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr">
@@ -4105,17 +4165,35 @@
           <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
         </is>
       </c>
-      <c r="L51" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M51" s="2" t="inlineStr"/>
-      <c r="N51" s="2" t="inlineStr"/>
-      <c r="O51" s="2" t="inlineStr"/>
-      <c r="P51" s="2" t="inlineStr"/>
-      <c r="Q51" s="2" t="inlineStr"/>
-      <c r="R51" s="2" t="inlineStr"/>
+      <c r="L51" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M51" s="2" t="inlineStr">
+        <is>
+          <t>PD57335</t>
+        </is>
+      </c>
+      <c r="N51" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="O51" s="2" t="inlineStr">
+        <is>
+          <t>1 / 1 / 28</t>
+        </is>
+      </c>
+      <c r="P51" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="Q51" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R51" s="5" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S51" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -4123,7 +4201,7 @@
       </c>
       <c r="T51" s="3" t="inlineStr">
         <is>
-          <t>submitted 2026-10-15 05:24, LSF jobs 699021-699042, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57335; 102/102 colonies GRCh38</t>
+          <t>submitted 2026-10-15 05:24, LSF jobs 699021-699042, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57335; 102/102 colonies GRCh38; results copied 2026-10-17 to ~/Documents/hsc_results/PD57335</t>
         </is>
       </c>
     </row>
@@ -4165,7 +4243,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-17 09:26</t>
+          <t>refreshed 2026-10-17 09:29</t>
         </is>
       </c>
     </row>
@@ -4205,7 +4283,7 @@
         <v>6</v>
       </c>
       <c r="D4" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -4221,10 +4299,10 @@
         <v>9</v>
       </c>
       <c r="C5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -4262,7 +4340,7 @@
         <v>3</v>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
@@ -4297,10 +4375,10 @@
         <v>50</v>
       </c>
       <c r="C9" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D9" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -6419,15 +6497,33 @@
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M31" t="inlineStr"/>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
-      <c r="P31" t="inlineStr"/>
-      <c r="Q31" t="inlineStr"/>
-      <c r="R31" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>PD43975</t>
+        </is>
+      </c>
+      <c r="N31" t="n">
+        <v>25</v>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>1 / 1 / 23</t>
+        </is>
+      </c>
+      <c r="P31" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q31" t="n">
+        <v>0</v>
+      </c>
+      <c r="R31" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S31" t="inlineStr">
         <is>
           <t>no</t>
@@ -6435,7 +6531,7 @@
       </c>
       <c r="T31" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-16 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43975; 38/38 colonies; done on farm 2026-10-17</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-16 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43975; 38/38 colonies; done on farm 2026-10-17; results copied 2026-10-17 to ~/Documents/hsc_results/PD43975</t>
         </is>
       </c>
     </row>
@@ -6480,11 +6576,19 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J32" t="inlineStr"/>
-      <c r="K32" t="inlineStr"/>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD43293/PD43293</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L32" t="inlineStr">
         <is>
           <t>no</t>
@@ -6503,7 +6607,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips)</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43293</t>
         </is>
       </c>
     </row>
@@ -6684,11 +6788,19 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr"/>
-      <c r="K35" t="inlineStr"/>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD45887/PD45887</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L35" t="inlineStr">
         <is>
           <t>no</t>
@@ -6707,7 +6819,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips)</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD45887</t>
         </is>
       </c>
     </row>
@@ -6846,11 +6958,19 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr"/>
-      <c r="K37" t="inlineStr"/>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD42191/PD42191</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L37" t="inlineStr">
         <is>
           <t>no</t>
@@ -6869,7 +6989,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips)</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD42191</t>
         </is>
       </c>
     </row>
@@ -7211,15 +7331,33 @@
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M42" t="inlineStr"/>
-      <c r="N42" t="inlineStr"/>
-      <c r="O42" t="inlineStr"/>
-      <c r="P42" t="inlineStr"/>
-      <c r="Q42" t="inlineStr"/>
-      <c r="R42" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>PD54832</t>
+        </is>
+      </c>
+      <c r="N42" t="n">
+        <v>19</v>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>0 / 0 / 19</t>
+        </is>
+      </c>
+      <c r="P42" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>0</v>
+      </c>
+      <c r="R42" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S42" t="inlineStr">
         <is>
           <t>no</t>
@@ -7227,7 +7365,7 @@
       </c>
       <c r="T42" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); tips renamed lo00NN -&gt; PD54832b_lo00NN; tissue folder (peripheral_blood) not verified; submitted 2026-10-16 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD54832; 49/49 colonies; done on farm 2026-10-17</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); tips renamed lo00NN -&gt; PD54832b_lo00NN; tissue folder (peripheral_blood) not verified; submitted 2026-10-16 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD54832; 49/49 colonies; done on farm 2026-10-17; results copied 2026-10-17 to ~/Documents/hsc_results/PD54832</t>
         </is>
       </c>
     </row>
@@ -7954,7 +8092,7 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
@@ -7969,15 +8107,33 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M51" t="inlineStr"/>
-      <c r="N51" t="inlineStr"/>
-      <c r="O51" t="inlineStr"/>
-      <c r="P51" t="inlineStr"/>
-      <c r="Q51" t="inlineStr"/>
-      <c r="R51" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>PD57335</t>
+        </is>
+      </c>
+      <c r="N51" t="n">
+        <v>30</v>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>1 / 1 / 28</t>
+        </is>
+      </c>
+      <c r="P51" t="n">
+        <v>24</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>0</v>
+      </c>
+      <c r="R51" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S51" t="inlineStr">
         <is>
           <t>no</t>
@@ -7985,7 +8141,7 @@
       </c>
       <c r="T51" t="inlineStr">
         <is>
-          <t>submitted 2026-10-15 05:24, LSF jobs 699021-699042, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57335; 102/102 colonies GRCh38</t>
+          <t>submitted 2026-10-15 05:24, LSF jobs 699021-699042, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD57335; 102/102 colonies GRCh38; results copied 2026-10-17 to ~/Documents/hsc_results/PD57335</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Run tracker: 16 units chain-submitted via hsc_chain.sh (sd/cleanup job IDs); PD43294/PD43295 running
Pair21/24/25 held back (hs37d5+hg19 mixed projects 2679/2693 would lose their hg19
colonies at the GRCh37 header gate); PD49229 rerun not scheduled.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -726,13 +726,21 @@
       <c r="H3" s="2" t="n">
         <v>259</v>
       </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr"/>
-      <c r="K3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD47703/PD47703</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L3" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -751,7 +759,7 @@
       </c>
       <c r="T3" s="3" t="inlineStr">
         <is>
-          <t>old-pipeline results only (~/Documents/retrotransposons_sanger/results/PD47703)</t>
+          <t>old-pipeline results only (~/Documents/retrotransposons_sanger/results/PD47703); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344581, cleanup 344588, stage+discover waits on ended(344578), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD47703</t>
         </is>
       </c>
     </row>
@@ -794,13 +802,21 @@
       <c r="H4" s="2" t="n">
         <v>922</v>
       </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="inlineStr"/>
-      <c r="K4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD45534/PD45534</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L4" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -819,7 +835,7 @@
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>SETTLED 2026-10-10: repopulated preferring GRCh38 -&gt; all 922 colonies GRCh38 (450 proj 2450, 472 proj 3819; old mixed file kept as colonies.tsv.bak.20261010040433). Old-pipeline results in ~/Documents/retrotransposons_sanger/results/PD45534</t>
+          <t>SETTLED 2026-10-10: repopulated preferring GRCh38 -&gt; all 922 colonies GRCh38 (450 proj 2450, 472 proj 3819; old mixed file kept as colonies.tsv.bak.20261010040433). Old-pipeline results in ~/Documents/retrotransposons_sanger/results/PD45534; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh38, sd 344703, cleanup 344711, stage+discover waits on ended(344700), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD45534</t>
         </is>
       </c>
     </row>
@@ -862,13 +878,21 @@
       <c r="H5" s="2" t="n">
         <v>179</v>
       </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr"/>
-      <c r="K5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair11_PD45792_PD45793/Pair11_PD45792_PD45793</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L5" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -885,7 +909,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T5" s="3" t="inlineStr"/>
+      <c r="T5" s="3" t="inlineStr">
+        <is>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344646, cleanup 344654, stage+discover waits on ended(344642), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair11_PD45792_PD45793</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -922,13 +950,21 @@
       <c r="H6" s="2" t="n">
         <v>146</v>
       </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="inlineStr"/>
-      <c r="K6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair11_PD45792_PD45793/Pair11_PD45792_PD45793</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L6" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -945,7 +981,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T6" s="3" t="inlineStr"/>
+      <c r="T6" s="3" t="inlineStr">
+        <is>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344646, cleanup 344654, stage+discover waits on ended(344642), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair11_PD45792_PD45793</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -986,13 +1026,21 @@
       <c r="H7" s="2" t="n">
         <v>104</v>
       </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="inlineStr"/>
-      <c r="K7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair13_PD45794_PD45795/Pair13_PD45794_PD45795</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L7" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -1009,7 +1057,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T7" s="3" t="inlineStr"/>
+      <c r="T7" s="3" t="inlineStr">
+        <is>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344632, cleanup 344642, stage+discover waits on ended(344627), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair13_PD45794_PD45795</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -1046,13 +1098,21 @@
       <c r="H8" s="2" t="n">
         <v>194</v>
       </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr"/>
-      <c r="K8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair13_PD45794_PD45795/Pair13_PD45794_PD45795</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L8" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -1069,7 +1129,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T8" s="3" t="inlineStr"/>
+      <c r="T8" s="3" t="inlineStr">
+        <is>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344632, cleanup 344642, stage+discover waits on ended(344627), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair13_PD45794_PD45795</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1106,13 +1170,21 @@
       <c r="H9" s="2" t="n">
         <v>143</v>
       </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr"/>
-      <c r="K9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair38_PD45808_PD45809/Pair38_PD45808_PD45809</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -1129,7 +1201,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T9" s="3" t="inlineStr"/>
+      <c r="T9" s="3" t="inlineStr">
+        <is>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1170,13 +1246,21 @@
       <c r="H10" s="2" t="n">
         <v>109</v>
       </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="inlineStr"/>
-      <c r="K10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair38_PD45808_PD45809/Pair38_PD45808_PD45809</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L10" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -1193,7 +1277,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T10" s="3" t="inlineStr"/>
+      <c r="T10" s="3" t="inlineStr">
+        <is>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1230,13 +1318,21 @@
       <c r="H11" s="2" t="n">
         <v>143</v>
       </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="inlineStr"/>
-      <c r="K11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair40_PD45810_PD45811/Pair40_PD45810_PD45811</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L11" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -1253,7 +1349,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T11" s="3" t="inlineStr"/>
+      <c r="T11" s="3" t="inlineStr">
+        <is>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344592, cleanup 344598, stage+discover waits on ended(344588), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair40_PD45810_PD45811</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1294,13 +1394,21 @@
       <c r="H12" s="2" t="n">
         <v>136</v>
       </c>
-      <c r="I12" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="inlineStr"/>
-      <c r="K12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair40_PD45810_PD45811/Pair40_PD45810_PD45811</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L12" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -1317,7 +1425,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T12" s="3" t="inlineStr"/>
+      <c r="T12" s="3" t="inlineStr">
+        <is>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344592, cleanup 344598, stage+discover waits on ended(344588), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair40_PD45810_PD45811</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1738,13 +1850,21 @@
       <c r="H19" s="2" t="n">
         <v>66</v>
       </c>
-      <c r="I19" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J19" s="2" t="inlineStr"/>
-      <c r="K19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair28_PD45804_PD45805/Pair28_PD45804_PD45805</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L19" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -1763,7 +1883,7 @@
       </c>
       <c r="T19" s="3" t="inlineStr">
         <is>
-          <t>published Pair_10; added 2026-10-15 (whole transplant cohort)</t>
+          <t>published Pair_10; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805</t>
         </is>
       </c>
     </row>
@@ -1802,13 +1922,21 @@
       <c r="H20" s="2" t="n">
         <v>174</v>
       </c>
-      <c r="I20" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J20" s="2" t="inlineStr"/>
-      <c r="K20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair28_PD45804_PD45805/Pair28_PD45804_PD45805</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L20" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -1827,7 +1955,7 @@
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>published Pair_10; recipient is a CML patient (BCR::ABL1 pre-HSCT), Flu-Bu-ATG; added 2026-10-15 (whole transplant cohort)</t>
+          <t>published Pair_10; recipient is a CML patient (BCR::ABL1 pre-HSCT), Flu-Bu-ATG; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805</t>
         </is>
       </c>
     </row>
@@ -1866,13 +1994,21 @@
       <c r="H21" s="2" t="n">
         <v>67</v>
       </c>
-      <c r="I21" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J21" s="2" t="inlineStr"/>
-      <c r="K21" s="2" t="inlineStr"/>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair31_PD45806_PD45807/Pair31_PD45806_PD45807</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L21" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -1891,7 +2027,7 @@
       </c>
       <c r="T21" s="3" t="inlineStr">
         <is>
-          <t>published Pair_6; added 2026-10-15 (whole transplant cohort)</t>
+          <t>published Pair_6; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807</t>
         </is>
       </c>
     </row>
@@ -1930,13 +2066,21 @@
       <c r="H22" s="2" t="n">
         <v>125</v>
       </c>
-      <c r="I22" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J22" s="2" t="inlineStr"/>
-      <c r="K22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair31_PD45806_PD45807/Pair31_PD45806_PD45807</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L22" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -1955,7 +2099,7 @@
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>published Pair_6; recipient: cisplatin for oesophageal cancer after HSCT; added 2026-10-15 (whole transplant cohort)</t>
+          <t>published Pair_6; recipient: cisplatin for oesophageal cancer after HSCT; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807</t>
         </is>
       </c>
     </row>
@@ -1994,13 +2138,21 @@
       <c r="H23" s="2" t="n">
         <v>119</v>
       </c>
-      <c r="I23" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J23" s="2" t="inlineStr"/>
-      <c r="K23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair41_PD45812_PD45813/Pair41_PD45812_PD45813</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L23" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2019,7 +2171,7 @@
       </c>
       <c r="T23" s="3" t="inlineStr">
         <is>
-          <t>published Pair_2; added 2026-10-15 (whole transplant cohort)</t>
+          <t>published Pair_2; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344601, cleanup 344613, stage+discover waits on ended(344598), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair41_PD45812_PD45813</t>
         </is>
       </c>
     </row>
@@ -2058,13 +2210,21 @@
       <c r="H24" s="2" t="n">
         <v>160</v>
       </c>
-      <c r="I24" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J24" s="2" t="inlineStr"/>
-      <c r="K24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J24" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair41_PD45812_PD45813/Pair41_PD45812_PD45813</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L24" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2083,7 +2243,7 @@
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>published Pair_2; sex-mismatched pair (F donor -&gt; M recipient); added 2026-10-15 (whole transplant cohort)</t>
+          <t>published Pair_2; sex-mismatched pair (F donor -&gt; M recipient); added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344601, cleanup 344613, stage+discover waits on ended(344598), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair41_PD45812_PD45813</t>
         </is>
       </c>
     </row>
@@ -2216,13 +2376,21 @@
       <c r="H26" s="2" t="n">
         <v>344</v>
       </c>
-      <c r="I26" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J26" s="2" t="inlineStr"/>
-      <c r="K26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD49226/PD49226</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L26" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2241,7 +2409,7 @@
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort)</t>
+          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344657, cleanup 344664, stage+discover waits on ended(344654), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD49226</t>
         </is>
       </c>
     </row>
@@ -2280,13 +2448,21 @@
       <c r="H27" s="2" t="n">
         <v>423</v>
       </c>
-      <c r="I27" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J27" s="2" t="inlineStr"/>
-      <c r="K27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD49227/PD49227</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L27" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2305,7 +2481,7 @@
       </c>
       <c r="T27" s="3" t="inlineStr">
         <is>
-          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort)</t>
+          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344667, cleanup 344676, stage+discover waits on ended(344664), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD49227</t>
         </is>
       </c>
     </row>
@@ -2344,13 +2520,21 @@
       <c r="H28" s="2" t="n">
         <v>486</v>
       </c>
-      <c r="I28" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J28" s="2" t="inlineStr"/>
-      <c r="K28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD49228/PD49228</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L28" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2369,7 +2553,7 @@
       </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort)</t>
+          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344680, cleanup 344686, stage+discover waits on ended(344676), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD49228</t>
         </is>
       </c>
     </row>
@@ -2408,13 +2592,21 @@
       <c r="H29" s="2" t="n">
         <v>535</v>
       </c>
-      <c r="I29" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J29" s="2" t="inlineStr"/>
-      <c r="K29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD53373/PD53373</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L29" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2433,7 +2625,7 @@
       </c>
       <c r="T29" s="3" t="inlineStr">
         <is>
-          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort)</t>
+          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344692, cleanup 344700, stage+discover waits on ended(344686), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD53373</t>
         </is>
       </c>
     </row>
@@ -2472,13 +2664,21 @@
       <c r="H30" s="2" t="n">
         <v>297</v>
       </c>
-      <c r="I30" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J30" s="2" t="inlineStr"/>
-      <c r="K30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD53374/PD53374</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L30" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2497,7 +2697,7 @@
       </c>
       <c r="T30" s="3" t="inlineStr">
         <is>
-          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort)</t>
+          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344620, cleanup 344627, stage+discover waits on ended(344613), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD53374</t>
         </is>
       </c>
     </row>
@@ -2649,17 +2849,25 @@
           <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
         </is>
       </c>
-      <c r="L32" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M32" s="2" t="inlineStr"/>
+      <c r="L32" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>PD43293</t>
+        </is>
+      </c>
       <c r="N32" s="2" t="inlineStr"/>
       <c r="O32" s="2" t="inlineStr"/>
       <c r="P32" s="2" t="inlineStr"/>
       <c r="Q32" s="2" t="inlineStr"/>
-      <c r="R32" s="2" t="inlineStr"/>
+      <c r="R32" s="2" t="inlineStr">
+        <is>
+          <t>no somatic table</t>
+        </is>
+      </c>
       <c r="S32" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2710,13 +2918,21 @@
       <c r="H33" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="I33" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J33" s="2" t="inlineStr"/>
-      <c r="K33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/SDS5_PD42190_PD45888/SDS5_PD42190_PD45888</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L33" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2735,7 +2951,7 @@
       </c>
       <c r="T33" s="3" t="inlineStr">
         <is>
-          <t>one tree with PD45888; colonies.tsv populated 2026-10-10 (100/100)</t>
+          <t>one tree with PD45888; colonies.tsv populated 2026-10-10 (100/100); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344533, cleanup 344539, stage+discover waits on ended(344527), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/SDS5_PD42190_PD45888</t>
         </is>
       </c>
     </row>
@@ -2778,13 +2994,21 @@
       <c r="H34" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="I34" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J34" s="2" t="inlineStr"/>
-      <c r="K34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/SDS5_PD42190_PD45888/SDS5_PD42190_PD45888</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L34" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2803,7 +3027,7 @@
       </c>
       <c r="T34" s="3" t="inlineStr">
         <is>
-          <t>one tree with PD42190; colonies.tsv populated 2026-10-10 (100/100)</t>
+          <t>one tree with PD42190; colonies.tsv populated 2026-10-10 (100/100); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344533, cleanup 344539, stage+discover waits on ended(344527), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/SDS5_PD42190_PD45888</t>
         </is>
       </c>
     </row>
@@ -2861,17 +3085,25 @@
           <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
         </is>
       </c>
-      <c r="L35" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M35" s="2" t="inlineStr"/>
+      <c r="L35" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="M35" s="2" t="inlineStr">
+        <is>
+          <t>PD45887</t>
+        </is>
+      </c>
       <c r="N35" s="2" t="inlineStr"/>
       <c r="O35" s="2" t="inlineStr"/>
       <c r="P35" s="2" t="inlineStr"/>
       <c r="Q35" s="2" t="inlineStr"/>
-      <c r="R35" s="2" t="inlineStr"/>
+      <c r="R35" s="2" t="inlineStr">
+        <is>
+          <t>no somatic table</t>
+        </is>
+      </c>
       <c r="S35" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -3031,17 +3263,25 @@
           <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
         </is>
       </c>
-      <c r="L37" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M37" s="2" t="inlineStr"/>
+      <c r="L37" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="M37" s="2" t="inlineStr">
+        <is>
+          <t>PD42191</t>
+        </is>
+      </c>
       <c r="N37" s="2" t="inlineStr"/>
       <c r="O37" s="2" t="inlineStr"/>
       <c r="P37" s="2" t="inlineStr"/>
       <c r="Q37" s="2" t="inlineStr"/>
-      <c r="R37" s="2" t="inlineStr"/>
+      <c r="R37" s="2" t="inlineStr">
+        <is>
+          <t>no somatic table</t>
+        </is>
+      </c>
       <c r="S37" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -3182,13 +3422,21 @@
       <c r="H39" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="I39" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J39" s="2" t="inlineStr"/>
-      <c r="K39" s="2" t="inlineStr"/>
+      <c r="I39" s="6" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD43294/PD43294</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L39" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -3207,7 +3455,7 @@
       </c>
       <c r="T39" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 18/18 tips, all proj 2045; ready to submit</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 18/18 tips, all proj 2045; ready to submit; submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43294</t>
         </is>
       </c>
     </row>
@@ -3246,13 +3494,21 @@
       <c r="H40" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="I40" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J40" s="2" t="inlineStr"/>
-      <c r="K40" s="2" t="inlineStr"/>
+      <c r="I40" s="6" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD43295/PD43295</t>
+        </is>
+      </c>
+      <c r="K40" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L40" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -3271,7 +3527,7 @@
       </c>
       <c r="T40" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 23/23 tips, all proj 2045; ready to submit</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 23/23 tips, all proj 2045; ready to submit; submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43295</t>
         </is>
       </c>
     </row>
@@ -3310,13 +3566,21 @@
       <c r="H41" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="I41" s="5" t="inlineStr">
-        <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J41" s="2" t="inlineStr"/>
-      <c r="K41" s="2" t="inlineStr"/>
+      <c r="I41" s="6" t="inlineStr">
+        <is>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD45889/PD45889</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L41" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -3335,7 +3599,7 @@
       </c>
       <c r="T41" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 27/27 tips, all proj 2045; ready to submit</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 27/27 tips, all proj 2045; ready to submit; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344519, cleanup 344527, stage+discover starts immediately, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD45889</t>
         </is>
       </c>
     </row>
@@ -4243,7 +4507,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-17 09:29</t>
+          <t>refreshed 2026-10-18 07:04</t>
         </is>
       </c>
     </row>
@@ -4668,11 +4932,19 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD47703/PD47703</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L3" t="inlineStr">
         <is>
           <t>no</t>
@@ -4691,7 +4963,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>old-pipeline results only (~/Documents/retrotransposons_sanger/results/PD47703)</t>
+          <t>old-pipeline results only (~/Documents/retrotransposons_sanger/results/PD47703); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344581, cleanup 344588, stage+discover waits on ended(344578), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD47703</t>
         </is>
       </c>
     </row>
@@ -4736,11 +5008,19 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD45534/PD45534</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L4" t="inlineStr">
         <is>
           <t>no</t>
@@ -4759,7 +5039,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>SETTLED 2026-10-10: repopulated preferring GRCh38 -&gt; all 922 colonies GRCh38 (450 proj 2450, 472 proj 3819; old mixed file kept as colonies.tsv.bak.20261010040433). Old-pipeline results in ~/Documents/retrotransposons_sanger/results/PD45534</t>
+          <t>SETTLED 2026-10-10: repopulated preferring GRCh38 -&gt; all 922 colonies GRCh38 (450 proj 2450, 472 proj 3819; old mixed file kept as colonies.tsv.bak.20261010040433). Old-pipeline results in ~/Documents/retrotransposons_sanger/results/PD45534; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh38, sd 344703, cleanup 344711, stage+discover waits on ended(344700), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD45534</t>
         </is>
       </c>
     </row>
@@ -4804,11 +5084,19 @@
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair11_PD45792_PD45793/Pair11_PD45792_PD45793</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L5" t="inlineStr">
         <is>
           <t>no</t>
@@ -4825,7 +5113,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T5" t="inlineStr"/>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344646, cleanup 344654, stage+discover waits on ended(344642), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair11_PD45792_PD45793</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -4864,11 +5156,19 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair11_PD45792_PD45793/Pair11_PD45792_PD45793</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L6" t="inlineStr">
         <is>
           <t>no</t>
@@ -4885,7 +5185,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr"/>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344646, cleanup 344654, stage+discover waits on ended(344642), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair11_PD45792_PD45793</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -4928,11 +5232,19 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair13_PD45794_PD45795/Pair13_PD45794_PD45795</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L7" t="inlineStr">
         <is>
           <t>no</t>
@@ -4949,7 +5261,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr"/>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344632, cleanup 344642, stage+discover waits on ended(344627), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair13_PD45794_PD45795</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -4988,11 +5304,19 @@
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair13_PD45794_PD45795/Pair13_PD45794_PD45795</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L8" t="inlineStr">
         <is>
           <t>no</t>
@@ -5009,7 +5333,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T8" t="inlineStr"/>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344632, cleanup 344642, stage+discover waits on ended(344627), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair13_PD45794_PD45795</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -5048,11 +5376,19 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair38_PD45808_PD45809/Pair38_PD45808_PD45809</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L9" t="inlineStr">
         <is>
           <t>no</t>
@@ -5069,7 +5405,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T9" t="inlineStr"/>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -5112,11 +5452,19 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair38_PD45808_PD45809/Pair38_PD45808_PD45809</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L10" t="inlineStr">
         <is>
           <t>no</t>
@@ -5133,7 +5481,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T10" t="inlineStr"/>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -5172,11 +5524,19 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair40_PD45810_PD45811/Pair40_PD45810_PD45811</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L11" t="inlineStr">
         <is>
           <t>no</t>
@@ -5193,7 +5553,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T11" t="inlineStr"/>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344592, cleanup 344598, stage+discover waits on ended(344588), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair40_PD45810_PD45811</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -5236,11 +5600,19 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair40_PD45810_PD45811/Pair40_PD45810_PD45811</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L12" t="inlineStr">
         <is>
           <t>no</t>
@@ -5257,7 +5629,11 @@
           <t>no</t>
         </is>
       </c>
-      <c r="T12" t="inlineStr"/>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344592, cleanup 344598, stage+discover waits on ended(344588), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair40_PD45810_PD45811</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -5680,11 +6056,19 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr"/>
-      <c r="K19" t="inlineStr"/>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair28_PD45804_PD45805/Pair28_PD45804_PD45805</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L19" t="inlineStr">
         <is>
           <t>no</t>
@@ -5703,7 +6087,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>published Pair_10; added 2026-10-15 (whole transplant cohort)</t>
+          <t>published Pair_10; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805</t>
         </is>
       </c>
     </row>
@@ -5744,11 +6128,19 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr"/>
-      <c r="K20" t="inlineStr"/>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair28_PD45804_PD45805/Pair28_PD45804_PD45805</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L20" t="inlineStr">
         <is>
           <t>no</t>
@@ -5767,7 +6159,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>published Pair_10; recipient is a CML patient (BCR::ABL1 pre-HSCT), Flu-Bu-ATG; added 2026-10-15 (whole transplant cohort)</t>
+          <t>published Pair_10; recipient is a CML patient (BCR::ABL1 pre-HSCT), Flu-Bu-ATG; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805</t>
         </is>
       </c>
     </row>
@@ -5808,11 +6200,19 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr"/>
-      <c r="K21" t="inlineStr"/>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair31_PD45806_PD45807/Pair31_PD45806_PD45807</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L21" t="inlineStr">
         <is>
           <t>no</t>
@@ -5831,7 +6231,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>published Pair_6; added 2026-10-15 (whole transplant cohort)</t>
+          <t>published Pair_6; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807</t>
         </is>
       </c>
     </row>
@@ -5872,11 +6272,19 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr"/>
-      <c r="K22" t="inlineStr"/>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair31_PD45806_PD45807/Pair31_PD45806_PD45807</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L22" t="inlineStr">
         <is>
           <t>no</t>
@@ -5895,7 +6303,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>published Pair_6; recipient: cisplatin for oesophageal cancer after HSCT; added 2026-10-15 (whole transplant cohort)</t>
+          <t>published Pair_6; recipient: cisplatin for oesophageal cancer after HSCT; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807</t>
         </is>
       </c>
     </row>
@@ -5936,11 +6344,19 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr"/>
-      <c r="K23" t="inlineStr"/>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair41_PD45812_PD45813/Pair41_PD45812_PD45813</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L23" t="inlineStr">
         <is>
           <t>no</t>
@@ -5959,7 +6375,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>published Pair_2; added 2026-10-15 (whole transplant cohort)</t>
+          <t>published Pair_2; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344601, cleanup 344613, stage+discover waits on ended(344598), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair41_PD45812_PD45813</t>
         </is>
       </c>
     </row>
@@ -6000,11 +6416,19 @@
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr"/>
-      <c r="K24" t="inlineStr"/>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair41_PD45812_PD45813/Pair41_PD45812_PD45813</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L24" t="inlineStr">
         <is>
           <t>no</t>
@@ -6023,7 +6447,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>published Pair_2; sex-mismatched pair (F donor -&gt; M recipient); added 2026-10-15 (whole transplant cohort)</t>
+          <t>published Pair_2; sex-mismatched pair (F donor -&gt; M recipient); added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344601, cleanup 344613, stage+discover waits on ended(344598), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair41_PD45812_PD45813</t>
         </is>
       </c>
     </row>
@@ -6158,11 +6582,19 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr"/>
-      <c r="K26" t="inlineStr"/>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD49226/PD49226</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L26" t="inlineStr">
         <is>
           <t>no</t>
@@ -6181,7 +6613,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort)</t>
+          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344657, cleanup 344664, stage+discover waits on ended(344654), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD49226</t>
         </is>
       </c>
     </row>
@@ -6222,11 +6654,19 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr"/>
-      <c r="K27" t="inlineStr"/>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD49227/PD49227</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L27" t="inlineStr">
         <is>
           <t>no</t>
@@ -6245,7 +6685,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort)</t>
+          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344667, cleanup 344676, stage+discover waits on ended(344664), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD49227</t>
         </is>
       </c>
     </row>
@@ -6286,11 +6726,19 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr"/>
-      <c r="K28" t="inlineStr"/>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD49228/PD49228</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L28" t="inlineStr">
         <is>
           <t>no</t>
@@ -6309,7 +6757,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort)</t>
+          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344680, cleanup 344686, stage+discover waits on ended(344676), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD49228</t>
         </is>
       </c>
     </row>
@@ -6350,11 +6798,19 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr"/>
-      <c r="K29" t="inlineStr"/>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD53373/PD53373</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L29" t="inlineStr">
         <is>
           <t>no</t>
@@ -6373,7 +6829,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort)</t>
+          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344692, cleanup 344700, stage+discover waits on ended(344686), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD53373</t>
         </is>
       </c>
     </row>
@@ -6414,11 +6870,19 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J30" t="inlineStr"/>
-      <c r="K30" t="inlineStr"/>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD53374/PD53374</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L30" t="inlineStr">
         <is>
           <t>no</t>
@@ -6437,7 +6901,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort)</t>
+          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344620, cleanup 344627, stage+discover waits on ended(344613), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD53374</t>
         </is>
       </c>
     </row>
@@ -6591,15 +7055,23 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M32" t="inlineStr"/>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>PD43293</t>
+        </is>
+      </c>
       <c r="N32" t="inlineStr"/>
       <c r="O32" t="inlineStr"/>
       <c r="P32" t="inlineStr"/>
       <c r="Q32" t="inlineStr"/>
-      <c r="R32" t="inlineStr"/>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>no somatic table</t>
+        </is>
+      </c>
       <c r="S32" t="inlineStr">
         <is>
           <t>no</t>
@@ -6652,11 +7124,19 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J33" t="inlineStr"/>
-      <c r="K33" t="inlineStr"/>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/SDS5_PD42190_PD45888/SDS5_PD42190_PD45888</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L33" t="inlineStr">
         <is>
           <t>no</t>
@@ -6675,7 +7155,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>one tree with PD45888; colonies.tsv populated 2026-10-10 (100/100)</t>
+          <t>one tree with PD45888; colonies.tsv populated 2026-10-10 (100/100); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344533, cleanup 344539, stage+discover waits on ended(344527), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/SDS5_PD42190_PD45888</t>
         </is>
       </c>
     </row>
@@ -6720,11 +7200,19 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J34" t="inlineStr"/>
-      <c r="K34" t="inlineStr"/>
+          <t>queued</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/SDS5_PD42190_PD45888/SDS5_PD42190_PD45888</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L34" t="inlineStr">
         <is>
           <t>no</t>
@@ -6743,7 +7231,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>one tree with PD42190; colonies.tsv populated 2026-10-10 (100/100)</t>
+          <t>one tree with PD42190; colonies.tsv populated 2026-10-10 (100/100); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344533, cleanup 344539, stage+discover waits on ended(344527), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/SDS5_PD42190_PD45888</t>
         </is>
       </c>
     </row>
@@ -6803,15 +7291,23 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M35" t="inlineStr"/>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>PD45887</t>
+        </is>
+      </c>
       <c r="N35" t="inlineStr"/>
       <c r="O35" t="inlineStr"/>
       <c r="P35" t="inlineStr"/>
       <c r="Q35" t="inlineStr"/>
-      <c r="R35" t="inlineStr"/>
+      <c r="R35" t="inlineStr">
+        <is>
+          <t>no somatic table</t>
+        </is>
+      </c>
       <c r="S35" t="inlineStr">
         <is>
           <t>no</t>
@@ -6973,15 +7469,23 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M37" t="inlineStr"/>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>PD42191</t>
+        </is>
+      </c>
       <c r="N37" t="inlineStr"/>
       <c r="O37" t="inlineStr"/>
       <c r="P37" t="inlineStr"/>
       <c r="Q37" t="inlineStr"/>
-      <c r="R37" t="inlineStr"/>
+      <c r="R37" t="inlineStr">
+        <is>
+          <t>no somatic table</t>
+        </is>
+      </c>
       <c r="S37" t="inlineStr">
         <is>
           <t>no</t>
@@ -7124,11 +7628,19 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J39" t="inlineStr"/>
-      <c r="K39" t="inlineStr"/>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD43294/PD43294</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L39" t="inlineStr">
         <is>
           <t>no</t>
@@ -7147,7 +7659,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 18/18 tips, all proj 2045; ready to submit</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 18/18 tips, all proj 2045; ready to submit; submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43294</t>
         </is>
       </c>
     </row>
@@ -7188,11 +7700,19 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J40" t="inlineStr"/>
-      <c r="K40" t="inlineStr"/>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD43295/PD43295</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
+        </is>
+      </c>
       <c r="L40" t="inlineStr">
         <is>
           <t>no</t>
@@ -7211,7 +7731,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 23/23 tips, all proj 2045; ready to submit</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 23/23 tips, all proj 2045; ready to submit; submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43295</t>
         </is>
       </c>
     </row>
@@ -7252,11 +7772,19 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>not run</t>
-        </is>
-      </c>
-      <c r="J41" t="inlineStr"/>
-      <c r="K41" t="inlineStr"/>
+          <t>running</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/PD45889/PD45889</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
+        </is>
+      </c>
       <c r="L41" t="inlineStr">
         <is>
           <t>no</t>
@@ -7275,7 +7803,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 27/27 tips, all proj 2045; ready to submit</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 27/27 tips, all proj 2045; ready to submit; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344519, cleanup 344527, stage+discover starts immediately, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD45889</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Run tracker: PD42191 local (155 rows); PD45887, PD43293 done on farm, copy in progress
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -2834,9 +2834,9 @@
       <c r="H32" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="I32" s="6" t="inlineStr">
-        <is>
-          <t>running</t>
+      <c r="I32" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -2849,9 +2849,9 @@
           <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
         </is>
       </c>
-      <c r="L32" s="6" t="inlineStr">
-        <is>
-          <t>partial</t>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr">
@@ -2859,13 +2859,23 @@
           <t>PD43293</t>
         </is>
       </c>
-      <c r="N32" s="2" t="inlineStr"/>
-      <c r="O32" s="2" t="inlineStr"/>
-      <c r="P32" s="2" t="inlineStr"/>
-      <c r="Q32" s="2" t="inlineStr"/>
-      <c r="R32" s="2" t="inlineStr">
-        <is>
-          <t>no somatic table</t>
+      <c r="N32" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>10 / 11 / 27</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q32" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R32" s="5" t="inlineStr">
+        <is>
+          <t>not started</t>
         </is>
       </c>
       <c r="S32" s="5" t="inlineStr">
@@ -2875,7 +2885,7 @@
       </c>
       <c r="T32" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43293</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43293; done 2026-10-17</t>
         </is>
       </c>
     </row>
@@ -3070,9 +3080,9 @@
       <c r="H35" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="I35" s="6" t="inlineStr">
-        <is>
-          <t>running</t>
+      <c r="I35" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="J35" s="2" t="inlineStr">
@@ -3085,9 +3095,9 @@
           <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
         </is>
       </c>
-      <c r="L35" s="6" t="inlineStr">
-        <is>
-          <t>partial</t>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="M35" s="2" t="inlineStr">
@@ -3095,13 +3105,23 @@
           <t>PD45887</t>
         </is>
       </c>
-      <c r="N35" s="2" t="inlineStr"/>
-      <c r="O35" s="2" t="inlineStr"/>
-      <c r="P35" s="2" t="inlineStr"/>
-      <c r="Q35" s="2" t="inlineStr"/>
-      <c r="R35" s="2" t="inlineStr">
-        <is>
-          <t>no somatic table</t>
+      <c r="N35" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>1 / 4 / 41</t>
+        </is>
+      </c>
+      <c r="P35" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q35" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R35" s="5" t="inlineStr">
+        <is>
+          <t>not started</t>
         </is>
       </c>
       <c r="S35" s="5" t="inlineStr">
@@ -3111,7 +3131,7 @@
       </c>
       <c r="T35" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD45887</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD45887; done 2026-10-17</t>
         </is>
       </c>
     </row>
@@ -3248,9 +3268,9 @@
       <c r="H37" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="I37" s="6" t="inlineStr">
-        <is>
-          <t>running</t>
+      <c r="I37" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="J37" s="2" t="inlineStr">
@@ -3263,9 +3283,9 @@
           <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
         </is>
       </c>
-      <c r="L37" s="6" t="inlineStr">
-        <is>
-          <t>partial</t>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="M37" s="2" t="inlineStr">
@@ -3273,13 +3293,23 @@
           <t>PD42191</t>
         </is>
       </c>
-      <c r="N37" s="2" t="inlineStr"/>
-      <c r="O37" s="2" t="inlineStr"/>
-      <c r="P37" s="2" t="inlineStr"/>
-      <c r="Q37" s="2" t="inlineStr"/>
-      <c r="R37" s="2" t="inlineStr">
-        <is>
-          <t>no somatic table</t>
+      <c r="N37" s="2" t="n">
+        <v>155</v>
+      </c>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>21 / 46 / 88</t>
+        </is>
+      </c>
+      <c r="P37" s="2" t="n">
+        <v>603</v>
+      </c>
+      <c r="Q37" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R37" s="5" t="inlineStr">
+        <is>
+          <t>not started</t>
         </is>
       </c>
       <c r="S37" s="5" t="inlineStr">
@@ -3289,7 +3319,7 @@
       </c>
       <c r="T37" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD42191</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD42191; done 2026-10-17, results copied 2026-10-18 to ~/Documents/hsc_results/PD42191</t>
         </is>
       </c>
     </row>
@@ -4507,7 +4537,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-18 07:04</t>
+          <t>refreshed 2026-10-18 07:05</t>
         </is>
       </c>
     </row>
@@ -4544,10 +4574,10 @@
         <v>18</v>
       </c>
       <c r="C4" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="D4" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -4601,10 +4631,10 @@
         <v>11</v>
       </c>
       <c r="C7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
@@ -4639,10 +4669,10 @@
         <v>50</v>
       </c>
       <c r="C9" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="D9" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -7040,7 +7070,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
@@ -7055,7 +7085,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
@@ -7063,13 +7093,23 @@
           <t>PD43293</t>
         </is>
       </c>
-      <c r="N32" t="inlineStr"/>
-      <c r="O32" t="inlineStr"/>
-      <c r="P32" t="inlineStr"/>
-      <c r="Q32" t="inlineStr"/>
+      <c r="N32" t="n">
+        <v>48</v>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>10 / 11 / 27</t>
+        </is>
+      </c>
+      <c r="P32" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>0</v>
+      </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>no somatic table</t>
+          <t>not started</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -7079,7 +7119,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43293</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43293; done 2026-10-17</t>
         </is>
       </c>
     </row>
@@ -7276,7 +7316,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
@@ -7291,7 +7331,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
@@ -7299,13 +7339,23 @@
           <t>PD45887</t>
         </is>
       </c>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
-      <c r="P35" t="inlineStr"/>
-      <c r="Q35" t="inlineStr"/>
+      <c r="N35" t="n">
+        <v>46</v>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>1 / 4 / 41</t>
+        </is>
+      </c>
+      <c r="P35" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q35" t="n">
+        <v>0</v>
+      </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>no somatic table</t>
+          <t>not started</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -7315,7 +7365,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD45887</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD45887; done 2026-10-17</t>
         </is>
       </c>
     </row>
@@ -7454,7 +7504,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -7469,7 +7519,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -7477,13 +7527,23 @@
           <t>PD42191</t>
         </is>
       </c>
-      <c r="N37" t="inlineStr"/>
-      <c r="O37" t="inlineStr"/>
-      <c r="P37" t="inlineStr"/>
-      <c r="Q37" t="inlineStr"/>
+      <c r="N37" t="n">
+        <v>155</v>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>21 / 46 / 88</t>
+        </is>
+      </c>
+      <c r="P37" t="n">
+        <v>603</v>
+      </c>
+      <c r="Q37" t="n">
+        <v>0</v>
+      </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>no somatic table</t>
+          <t>not started</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -7493,7 +7553,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD42191</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD42191; done 2026-10-17, results copied 2026-10-18 to ~/Documents/hsc_results/PD42191</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Run tracker: PD43294/PD43295 state unknown (pre-existing jobids.tsv, not submitted by Jeremy)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -3452,9 +3452,9 @@
       <c r="H39" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="I39" s="6" t="inlineStr">
-        <is>
-          <t>running</t>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
@@ -3485,7 +3485,7 @@
       </c>
       <c r="T39" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 18/18 tips, all proj 2045; ready to submit; submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43294</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 18/18 tips, all proj 2045; ready to submit; 2026-10-18 hsc_chain.sh SKIPPED it: hsc_foldback2/PD43294/jobids.tsv already exists (submitted by someone else, not Jeremy) -- state unverified</t>
         </is>
       </c>
     </row>
@@ -3524,9 +3524,9 @@
       <c r="H40" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="I40" s="6" t="inlineStr">
-        <is>
-          <t>running</t>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -3557,7 +3557,7 @@
       </c>
       <c r="T40" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 23/23 tips, all proj 2045; ready to submit; submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43295</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 23/23 tips, all proj 2045; ready to submit; 2026-10-18 hsc_chain.sh SKIPPED it: hsc_foldback2/PD43295/jobids.tsv already exists (submitted by someone else, not Jeremy) -- state unverified</t>
         </is>
       </c>
     </row>
@@ -7688,7 +7688,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -7719,7 +7719,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 18/18 tips, all proj 2045; ready to submit; submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43294</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 18/18 tips, all proj 2045; ready to submit; 2026-10-18 hsc_chain.sh SKIPPED it: hsc_foldback2/PD43294/jobids.tsv already exists (submitted by someone else, not Jeremy) -- state unverified</t>
         </is>
       </c>
     </row>
@@ -7760,7 +7760,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -7791,7 +7791,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 23/23 tips, all proj 2045; ready to submit; submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43295</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 23/23 tips, all proj 2045; ready to submit; 2026-10-18 hsc_chain.sh SKIPPED it: hsc_foldback2/PD43295/jobids.tsv already exists (submitted by someone else, not Jeremy) -- state unverified</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Run tracker: PD43294/PD43295 done on farm (submitted 2026-10-17 08:32, jobs recorded)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -3452,9 +3452,9 @@
       <c r="H39" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="I39" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="I39" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr">
@@ -3485,7 +3485,7 @@
       </c>
       <c r="T39" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 18/18 tips, all proj 2045; ready to submit; 2026-10-18 hsc_chain.sh SKIPPED it: hsc_foldback2/PD43294/jobids.tsv already exists (submitted by someone else, not Jeremy) -- state unverified</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 18/18 tips, all proj 2045; ready to submit; submitted 2026-10-17 08:32 (not by Jeremy; LSF jobs 239587-239603), native GRCh37; status 2026-10-18: all colonies discovered+genotyped, contract+calls yes; results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43294</t>
         </is>
       </c>
     </row>
@@ -3524,9 +3524,9 @@
       <c r="H40" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
+      <c r="I40" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr">
@@ -3557,7 +3557,7 @@
       </c>
       <c r="T40" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 23/23 tips, all proj 2045; ready to submit; 2026-10-18 hsc_chain.sh SKIPPED it: hsc_foldback2/PD43295/jobids.tsv already exists (submitted by someone else, not Jeremy) -- state unverified</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 23/23 tips, all proj 2045; ready to submit; submitted 2026-10-17 08:32 (not by Jeremy; LSF jobs 239608-239631), native GRCh37; status 2026-10-18: all colonies discovered+genotyped, contract+calls yes; results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43295</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4537,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-18 07:05</t>
+          <t>refreshed 2026-10-18 07:06</t>
         </is>
       </c>
     </row>
@@ -4631,7 +4631,7 @@
         <v>11</v>
       </c>
       <c r="C7" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="D7" t="n">
         <v>6</v>
@@ -4669,7 +4669,7 @@
         <v>50</v>
       </c>
       <c r="C9" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D9" t="n">
         <v>18</v>
@@ -7688,7 +7688,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>done</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
@@ -7719,7 +7719,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 18/18 tips, all proj 2045; ready to submit; 2026-10-18 hsc_chain.sh SKIPPED it: hsc_foldback2/PD43294/jobids.tsv already exists (submitted by someone else, not Jeremy) -- state unverified</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 18/18 tips, all proj 2045; ready to submit; submitted 2026-10-17 08:32 (not by Jeremy; LSF jobs 239587-239603), native GRCh37; status 2026-10-18: all colonies discovered+genotyped, contract+calls yes; results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43294</t>
         </is>
       </c>
     </row>
@@ -7760,7 +7760,7 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>done</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
@@ -7791,7 +7791,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 23/23 tips, all proj 2045; ready to submit; 2026-10-18 hsc_chain.sh SKIPPED it: hsc_foldback2/PD43295/jobids.tsv already exists (submitted by someone else, not Jeremy) -- state unverified</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 23/23 tips, all proj 2045; ready to submit; submitted 2026-10-17 08:32 (not by Jeremy; LSF jobs 239608-239631), native GRCh37; status 2026-10-18: all colonies discovered+genotyped, contract+calls yes; results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43295</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Run tracker: PD45887, PD43293, PD43294, PD43295 results local
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -2885,7 +2885,7 @@
       </c>
       <c r="T32" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43293; done 2026-10-17</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43293; done 2026-10-17; results copied 2026-10-18 to ~/Documents/hsc_results/PD43293</t>
         </is>
       </c>
     </row>
@@ -3131,7 +3131,7 @@
       </c>
       <c r="T35" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD45887; done 2026-10-17</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD45887; done 2026-10-17; results copied 2026-10-18 to ~/Documents/hsc_results/PD45887</t>
         </is>
       </c>
     </row>
@@ -3467,17 +3467,35 @@
           <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
         </is>
       </c>
-      <c r="L39" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M39" s="2" t="inlineStr"/>
-      <c r="N39" s="2" t="inlineStr"/>
-      <c r="O39" s="2" t="inlineStr"/>
-      <c r="P39" s="2" t="inlineStr"/>
-      <c r="Q39" s="2" t="inlineStr"/>
-      <c r="R39" s="2" t="inlineStr"/>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="inlineStr">
+        <is>
+          <t>PD43294</t>
+        </is>
+      </c>
+      <c r="N39" s="2" t="n">
+        <v>22</v>
+      </c>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>2 / 5 / 15</t>
+        </is>
+      </c>
+      <c r="P39" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q39" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R39" s="5" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S39" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -3485,7 +3503,7 @@
       </c>
       <c r="T39" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 18/18 tips, all proj 2045; ready to submit; submitted 2026-10-17 08:32 (not by Jeremy; LSF jobs 239587-239603), native GRCh37; status 2026-10-18: all colonies discovered+genotyped, contract+calls yes; results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43294</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 18/18 tips, all proj 2045; ready to submit; submitted 2026-10-17 08:32 (not by Jeremy; LSF jobs 239587-239603), native GRCh37; status 2026-10-18: all colonies discovered+genotyped, contract+calls yes; results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43294; results copied 2026-10-18 to ~/Documents/hsc_results/PD43294</t>
         </is>
       </c>
     </row>
@@ -3539,17 +3557,35 @@
           <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate)</t>
         </is>
       </c>
-      <c r="L40" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M40" s="2" t="inlineStr"/>
-      <c r="N40" s="2" t="inlineStr"/>
-      <c r="O40" s="2" t="inlineStr"/>
-      <c r="P40" s="2" t="inlineStr"/>
-      <c r="Q40" s="2" t="inlineStr"/>
-      <c r="R40" s="2" t="inlineStr"/>
+      <c r="L40" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M40" s="2" t="inlineStr">
+        <is>
+          <t>PD43295</t>
+        </is>
+      </c>
+      <c r="N40" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>1 / 4 / 40</t>
+        </is>
+      </c>
+      <c r="P40" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q40" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R40" s="5" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S40" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -3557,7 +3593,7 @@
       </c>
       <c r="T40" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 23/23 tips, all proj 2045; ready to submit; submitted 2026-10-17 08:32 (not by Jeremy; LSF jobs 239608-239631), native GRCh37; status 2026-10-18: all colonies discovered+genotyped, contract+calls yes; results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43295</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 23/23 tips, all proj 2045; ready to submit; submitted 2026-10-17 08:32 (not by Jeremy; LSF jobs 239608-239631), native GRCh37; status 2026-10-18: all colonies discovered+genotyped, contract+calls yes; results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43295; results copied 2026-10-18 to ~/Documents/hsc_results/PD43295</t>
         </is>
       </c>
     </row>
@@ -4537,7 +4573,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-18 07:06</t>
+          <t>refreshed 2026-10-18 07:07</t>
         </is>
       </c>
     </row>
@@ -4634,7 +4670,7 @@
         <v>8</v>
       </c>
       <c r="D7" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
@@ -4672,7 +4708,7 @@
         <v>19</v>
       </c>
       <c r="D9" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -7119,7 +7155,7 @@
       </c>
       <c r="T32" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43293; done 2026-10-17</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43293; done 2026-10-17; results copied 2026-10-18 to ~/Documents/hsc_results/PD43293</t>
         </is>
       </c>
     </row>
@@ -7365,7 +7401,7 @@
       </c>
       <c r="T35" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD45887; done 2026-10-17</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD45887; done 2026-10-17; results copied 2026-10-18 to ~/Documents/hsc_results/PD45887</t>
         </is>
       </c>
     </row>
@@ -7703,15 +7739,33 @@
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M39" t="inlineStr"/>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
-      <c r="P39" t="inlineStr"/>
-      <c r="Q39" t="inlineStr"/>
-      <c r="R39" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>PD43294</t>
+        </is>
+      </c>
+      <c r="N39" t="n">
+        <v>22</v>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>2 / 5 / 15</t>
+        </is>
+      </c>
+      <c r="P39" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q39" t="n">
+        <v>0</v>
+      </c>
+      <c r="R39" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S39" t="inlineStr">
         <is>
           <t>no</t>
@@ -7719,7 +7773,7 @@
       </c>
       <c r="T39" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 18/18 tips, all proj 2045; ready to submit; submitted 2026-10-17 08:32 (not by Jeremy; LSF jobs 239587-239603), native GRCh37; status 2026-10-18: all colonies discovered+genotyped, contract+calls yes; results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43294</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 18/18 tips, all proj 2045; ready to submit; submitted 2026-10-17 08:32 (not by Jeremy; LSF jobs 239587-239603), native GRCh37; status 2026-10-18: all colonies discovered+genotyped, contract+calls yes; results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43294; results copied 2026-10-18 to ~/Documents/hsc_results/PD43294</t>
         </is>
       </c>
     </row>
@@ -7775,15 +7829,33 @@
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M40" t="inlineStr"/>
-      <c r="N40" t="inlineStr"/>
-      <c r="O40" t="inlineStr"/>
-      <c r="P40" t="inlineStr"/>
-      <c r="Q40" t="inlineStr"/>
-      <c r="R40" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>PD43295</t>
+        </is>
+      </c>
+      <c r="N40" t="n">
+        <v>45</v>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>1 / 4 / 40</t>
+        </is>
+      </c>
+      <c r="P40" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>0</v>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S40" t="inlineStr">
         <is>
           <t>no</t>
@@ -7791,7 +7863,7 @@
       </c>
       <c r="T40" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 23/23 tips, all proj 2045; ready to submit; submitted 2026-10-17 08:32 (not by Jeremy; LSF jobs 239608-239631), native GRCh37; status 2026-10-18: all colonies discovered+genotyped, contract+calls yes; results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43295</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 23/23 tips, all proj 2045; ready to submit; submitted 2026-10-17 08:32 (not by Jeremy; LSF jobs 239608-239631), native GRCh37; status 2026-10-18: all colonies discovered+genotyped, contract+calls yes; results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD43295; results copied 2026-10-18 to ~/Documents/hsc_results/PD43295</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Run tracker: Pair31 chain stall diagnosed and recovered (sdr 6992, ci rewired)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -669,11 +669,11 @@
       </c>
       <c r="P2" s="2" t="inlineStr"/>
       <c r="Q2" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="R2" s="2" t="inlineStr">
-        <is>
-          <t>30 %</t>
+        <v>20</v>
+      </c>
+      <c r="R2" s="4" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="S2" s="5" t="inlineStr">
@@ -2027,7 +2027,7 @@
       </c>
       <c r="T21" s="3" t="inlineStr">
         <is>
-          <t>published Pair_6; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807</t>
+          <t>published Pair_6; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058)</t>
         </is>
       </c>
     </row>
@@ -2099,7 +2099,7 @@
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>published Pair_6; recipient: cisplatin for oesophageal cancer after HSCT; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807</t>
+          <t>published Pair_6; recipient: cisplatin for oesophageal cancer after HSCT; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058)</t>
         </is>
       </c>
     </row>
@@ -2777,11 +2777,11 @@
         <v>7</v>
       </c>
       <c r="Q31" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R31" s="5" t="inlineStr">
-        <is>
-          <t>not started</t>
+        <v>25</v>
+      </c>
+      <c r="R31" s="4" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="S31" s="5" t="inlineStr">
@@ -2871,11 +2871,11 @@
         <v>6</v>
       </c>
       <c r="Q32" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R32" s="5" t="inlineStr">
-        <is>
-          <t>not started</t>
+        <v>48</v>
+      </c>
+      <c r="R32" s="4" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="S32" s="5" t="inlineStr">
@@ -3305,11 +3305,11 @@
         <v>603</v>
       </c>
       <c r="Q37" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R37" s="5" t="inlineStr">
-        <is>
-          <t>not started</t>
+        <v>36</v>
+      </c>
+      <c r="R37" s="2" t="inlineStr">
+        <is>
+          <t>23 %</t>
         </is>
       </c>
       <c r="S37" s="5" t="inlineStr">
@@ -3489,11 +3489,11 @@
         <v>3</v>
       </c>
       <c r="Q39" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R39" s="5" t="inlineStr">
-        <is>
-          <t>not started</t>
+        <v>22</v>
+      </c>
+      <c r="R39" s="4" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="S39" s="5" t="inlineStr">
@@ -3579,11 +3579,11 @@
         <v>18</v>
       </c>
       <c r="Q40" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R40" s="5" t="inlineStr">
-        <is>
-          <t>not started</t>
+        <v>45</v>
+      </c>
+      <c r="R40" s="4" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="S40" s="5" t="inlineStr">
@@ -3741,11 +3741,11 @@
         <v>13</v>
       </c>
       <c r="Q42" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R42" s="5" t="inlineStr">
-        <is>
-          <t>not started</t>
+        <v>19</v>
+      </c>
+      <c r="R42" s="4" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="S42" s="5" t="inlineStr">
@@ -4573,7 +4573,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-18 07:07</t>
+          <t>refreshed 2026-10-20 04:05</t>
         </is>
       </c>
     </row>
@@ -4939,11 +4939,11 @@
       </c>
       <c r="P2" t="inlineStr"/>
       <c r="Q2" t="n">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>30 %</t>
+          <t>complete</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
@@ -6297,7 +6297,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>published Pair_6; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807</t>
+          <t>published Pair_6; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058)</t>
         </is>
       </c>
     </row>
@@ -6369,7 +6369,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>published Pair_6; recipient: cisplatin for oesophageal cancer after HSCT; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807</t>
+          <t>published Pair_6; recipient: cisplatin for oesophageal cancer after HSCT; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058)</t>
         </is>
       </c>
     </row>
@@ -7047,11 +7047,11 @@
         <v>7</v>
       </c>
       <c r="Q31" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>complete</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -7141,11 +7141,11 @@
         <v>6</v>
       </c>
       <c r="Q32" t="n">
-        <v>0</v>
+        <v>48</v>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>complete</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -7575,11 +7575,11 @@
         <v>603</v>
       </c>
       <c r="Q37" t="n">
-        <v>0</v>
+        <v>36</v>
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>23 %</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -7759,11 +7759,11 @@
         <v>3</v>
       </c>
       <c r="Q39" t="n">
-        <v>0</v>
+        <v>22</v>
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>complete</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
@@ -7849,11 +7849,11 @@
         <v>18</v>
       </c>
       <c r="Q40" t="n">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>complete</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -8011,11 +8011,11 @@
         <v>13</v>
       </c>
       <c r="Q42" t="n">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>complete</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">

</xml_diff>

<commit_message>
Run tracker: PD45889 + SDS5_PD42190_PD45888 done on farm, results local
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -2928,9 +2928,9 @@
       <c r="H33" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>queued</t>
+      <c r="I33" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
@@ -2943,17 +2943,35 @@
           <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
         </is>
       </c>
-      <c r="L33" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M33" s="2" t="inlineStr"/>
-      <c r="N33" s="2" t="inlineStr"/>
-      <c r="O33" s="2" t="inlineStr"/>
-      <c r="P33" s="2" t="inlineStr"/>
-      <c r="Q33" s="2" t="inlineStr"/>
-      <c r="R33" s="2" t="inlineStr"/>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="inlineStr">
+        <is>
+          <t>SDS5_PD42190_PD45888</t>
+        </is>
+      </c>
+      <c r="N33" s="2" t="n">
+        <v>117</v>
+      </c>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>2 / 4 / 111</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="n">
+        <v>93</v>
+      </c>
+      <c r="Q33" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R33" s="5" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S33" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2961,7 +2979,7 @@
       </c>
       <c r="T33" s="3" t="inlineStr">
         <is>
-          <t>one tree with PD45888; colonies.tsv populated 2026-10-10 (100/100); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344533, cleanup 344539, stage+discover waits on ended(344527), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/SDS5_PD42190_PD45888</t>
+          <t>one tree with PD45888; colonies.tsv populated 2026-10-10 (100/100); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344533, cleanup 344539, stage+discover waits on ended(344527), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/SDS5_PD42190_PD45888; done on farm 2026-10-19 (somatic.xlsx 06:26); results copied 2026-10-20 to ~/Documents/hsc_results/SDS5_PD42190_PD45888; copy-number rule applied locally (apply_copy_number.py): 0 rows moved</t>
         </is>
       </c>
     </row>
@@ -3004,9 +3022,9 @@
       <c r="H34" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>queued</t>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -3019,17 +3037,35 @@
           <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
         </is>
       </c>
-      <c r="L34" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M34" s="2" t="inlineStr"/>
-      <c r="N34" s="2" t="inlineStr"/>
-      <c r="O34" s="2" t="inlineStr"/>
-      <c r="P34" s="2" t="inlineStr"/>
-      <c r="Q34" s="2" t="inlineStr"/>
-      <c r="R34" s="2" t="inlineStr"/>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>SDS5_PD42190_PD45888</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="n">
+        <v>117</v>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>2 / 4 / 111</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="n">
+        <v>93</v>
+      </c>
+      <c r="Q34" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R34" s="5" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S34" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -3037,7 +3073,7 @@
       </c>
       <c r="T34" s="3" t="inlineStr">
         <is>
-          <t>one tree with PD42190; colonies.tsv populated 2026-10-10 (100/100); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344533, cleanup 344539, stage+discover waits on ended(344527), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/SDS5_PD42190_PD45888</t>
+          <t>one tree with PD42190; colonies.tsv populated 2026-10-10 (100/100); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344533, cleanup 344539, stage+discover waits on ended(344527), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/SDS5_PD42190_PD45888; done on farm 2026-10-19 (somatic.xlsx 06:26); results copied 2026-10-20 to ~/Documents/hsc_results/SDS5_PD42190_PD45888; copy-number rule applied locally (apply_copy_number.py): 0 rows moved</t>
         </is>
       </c>
     </row>
@@ -3632,9 +3668,9 @@
       <c r="H41" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="I41" s="6" t="inlineStr">
-        <is>
-          <t>running</t>
+      <c r="I41" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
@@ -3647,17 +3683,35 @@
           <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
         </is>
       </c>
-      <c r="L41" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M41" s="2" t="inlineStr"/>
-      <c r="N41" s="2" t="inlineStr"/>
-      <c r="O41" s="2" t="inlineStr"/>
-      <c r="P41" s="2" t="inlineStr"/>
-      <c r="Q41" s="2" t="inlineStr"/>
-      <c r="R41" s="2" t="inlineStr"/>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>PD45889</t>
+        </is>
+      </c>
+      <c r="N41" s="2" t="n">
+        <v>62</v>
+      </c>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>5 / 8 / 49</t>
+        </is>
+      </c>
+      <c r="P41" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q41" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R41" s="5" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S41" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -3665,7 +3719,7 @@
       </c>
       <c r="T41" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 27/27 tips, all proj 2045; ready to submit; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344519, cleanup 344527, stage+discover starts immediately, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD45889</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 27/27 tips, all proj 2045; ready to submit; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344519, cleanup 344527, stage+discover starts immediately, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD45889; done on farm 2026-10-18 (somatic.xlsx 14:11); results copied 2026-10-20 to ~/Documents/hsc_results/PD45889</t>
         </is>
       </c>
     </row>
@@ -4573,7 +4627,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-20 04:05</t>
+          <t>refreshed 2026-10-20 04:09</t>
         </is>
       </c>
     </row>
@@ -4610,10 +4664,10 @@
         <v>18</v>
       </c>
       <c r="C4" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="D4" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -4667,10 +4721,10 @@
         <v>11</v>
       </c>
       <c r="C7" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="D7" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="E7" t="n">
         <v>0</v>
@@ -4705,10 +4759,10 @@
         <v>50</v>
       </c>
       <c r="C9" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="D9" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -7200,7 +7254,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>done</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
@@ -7215,15 +7269,33 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M33" t="inlineStr"/>
-      <c r="N33" t="inlineStr"/>
-      <c r="O33" t="inlineStr"/>
-      <c r="P33" t="inlineStr"/>
-      <c r="Q33" t="inlineStr"/>
-      <c r="R33" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>SDS5_PD42190_PD45888</t>
+        </is>
+      </c>
+      <c r="N33" t="n">
+        <v>117</v>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>2 / 4 / 111</t>
+        </is>
+      </c>
+      <c r="P33" t="n">
+        <v>93</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>0</v>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S33" t="inlineStr">
         <is>
           <t>no</t>
@@ -7231,7 +7303,7 @@
       </c>
       <c r="T33" t="inlineStr">
         <is>
-          <t>one tree with PD45888; colonies.tsv populated 2026-10-10 (100/100); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344533, cleanup 344539, stage+discover waits on ended(344527), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/SDS5_PD42190_PD45888</t>
+          <t>one tree with PD45888; colonies.tsv populated 2026-10-10 (100/100); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344533, cleanup 344539, stage+discover waits on ended(344527), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/SDS5_PD42190_PD45888; done on farm 2026-10-19 (somatic.xlsx 06:26); results copied 2026-10-20 to ~/Documents/hsc_results/SDS5_PD42190_PD45888; copy-number rule applied locally (apply_copy_number.py): 0 rows moved</t>
         </is>
       </c>
     </row>
@@ -7276,7 +7348,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>done</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
@@ -7291,15 +7363,33 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M34" t="inlineStr"/>
-      <c r="N34" t="inlineStr"/>
-      <c r="O34" t="inlineStr"/>
-      <c r="P34" t="inlineStr"/>
-      <c r="Q34" t="inlineStr"/>
-      <c r="R34" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>SDS5_PD42190_PD45888</t>
+        </is>
+      </c>
+      <c r="N34" t="n">
+        <v>117</v>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>2 / 4 / 111</t>
+        </is>
+      </c>
+      <c r="P34" t="n">
+        <v>93</v>
+      </c>
+      <c r="Q34" t="n">
+        <v>0</v>
+      </c>
+      <c r="R34" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S34" t="inlineStr">
         <is>
           <t>no</t>
@@ -7307,7 +7397,7 @@
       </c>
       <c r="T34" t="inlineStr">
         <is>
-          <t>one tree with PD42190; colonies.tsv populated 2026-10-10 (100/100); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344533, cleanup 344539, stage+discover waits on ended(344527), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/SDS5_PD42190_PD45888</t>
+          <t>one tree with PD42190; colonies.tsv populated 2026-10-10 (100/100); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344533, cleanup 344539, stage+discover waits on ended(344527), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/SDS5_PD42190_PD45888; done on farm 2026-10-19 (somatic.xlsx 06:26); results copied 2026-10-20 to ~/Documents/hsc_results/SDS5_PD42190_PD45888; copy-number rule applied locally (apply_copy_number.py): 0 rows moved</t>
         </is>
       </c>
     </row>
@@ -7904,7 +7994,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>done</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
@@ -7919,15 +8009,33 @@
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M41" t="inlineStr"/>
-      <c r="N41" t="inlineStr"/>
-      <c r="O41" t="inlineStr"/>
-      <c r="P41" t="inlineStr"/>
-      <c r="Q41" t="inlineStr"/>
-      <c r="R41" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>PD45889</t>
+        </is>
+      </c>
+      <c r="N41" t="n">
+        <v>62</v>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>5 / 8 / 49</t>
+        </is>
+      </c>
+      <c r="P41" t="n">
+        <v>11</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>0</v>
+      </c>
+      <c r="R41" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S41" t="inlineStr">
         <is>
           <t>no</t>
@@ -7935,7 +8043,7 @@
       </c>
       <c r="T41" t="inlineStr">
         <is>
-          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 27/27 tips, all proj 2045; ready to submit; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344519, cleanup 344527, stage+discover starts immediately, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD45889</t>
+          <t>tree added 2026-10-15 from nangalialab/SchwachmanDiamond cache/PDD.RDS (zeros outgroup dropped); colonies.tsv populated 2026-10-16 (iRODS, HSC_ASSEMBLY=GRCh37): 27/27 tips, all proj 2045; ready to submit; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344519, cleanup 344527, stage+discover starts immediately, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD45889; done on farm 2026-10-18 (somatic.xlsx 14:11); results copied 2026-10-20 to ~/Documents/hsc_results/PD45889</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Run tracker: PD45886 results = foldback2 run only; superseded runs archived
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -2965,11 +2965,11 @@
         <v>93</v>
       </c>
       <c r="Q33" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R33" s="5" t="inlineStr">
-        <is>
-          <t>not started</t>
+        <v>4</v>
+      </c>
+      <c r="R33" s="2" t="inlineStr">
+        <is>
+          <t>3 %</t>
         </is>
       </c>
       <c r="S33" s="5" t="inlineStr">
@@ -3059,11 +3059,11 @@
         <v>93</v>
       </c>
       <c r="Q34" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R34" s="5" t="inlineStr">
-        <is>
-          <t>not started</t>
+        <v>4</v>
+      </c>
+      <c r="R34" s="2" t="inlineStr">
+        <is>
+          <t>3 %</t>
         </is>
       </c>
       <c r="S34" s="5" t="inlineStr">
@@ -3153,11 +3153,11 @@
         <v>2</v>
       </c>
       <c r="Q35" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R35" s="5" t="inlineStr">
-        <is>
-          <t>not started</t>
+        <v>9</v>
+      </c>
+      <c r="R35" s="2" t="inlineStr">
+        <is>
+          <t>19 %</t>
         </is>
       </c>
       <c r="S35" s="5" t="inlineStr">
@@ -3247,11 +3247,11 @@
         <v>30</v>
       </c>
       <c r="Q36" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R36" s="5" t="inlineStr">
-        <is>
-          <t>not started</t>
+        <v>60</v>
+      </c>
+      <c r="R36" s="4" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="S36" s="5" t="inlineStr">
@@ -3341,11 +3341,11 @@
         <v>603</v>
       </c>
       <c r="Q37" s="2" t="n">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="R37" s="2" t="inlineStr">
         <is>
-          <t>23 %</t>
+          <t>37 %</t>
         </is>
       </c>
       <c r="S37" s="5" t="inlineStr">
@@ -3420,7 +3420,7 @@
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>PD45886_foldback2/PD45886</t>
+          <t>PD45886</t>
         </is>
       </c>
       <c r="N38" s="2" t="n">
@@ -3449,7 +3449,7 @@
       </c>
       <c r="T38" s="3" t="inlineStr">
         <is>
-          <t>27 colonies, proj 2045; 73 private calls (B 7, C 10), 2570 germline MEIs; first run (489 = cruciform artefacts) in ~/Documents/hsc_results/PD45886; hsc_foldback lost 217 germline (strand bug)</t>
+          <t>27 colonies, proj 2045; 73 private calls (B 7, C 10), 2570 germline MEIs; superseded runs (first run: 489 cruciform artefacts; hsc_foldback: lost 217 germline, strand bug) moved to ~/Documents/hsc_results_superseded</t>
         </is>
       </c>
     </row>
@@ -3705,11 +3705,11 @@
         <v>11</v>
       </c>
       <c r="Q41" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R41" s="5" t="inlineStr">
-        <is>
-          <t>not started</t>
+        <v>9</v>
+      </c>
+      <c r="R41" s="2" t="inlineStr">
+        <is>
+          <t>14 %</t>
         </is>
       </c>
       <c r="S41" s="5" t="inlineStr">
@@ -4571,11 +4571,11 @@
         <v>24</v>
       </c>
       <c r="Q51" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R51" s="5" t="inlineStr">
-        <is>
-          <t>not started</t>
+        <v>30</v>
+      </c>
+      <c r="R51" s="4" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="S51" s="5" t="inlineStr">
@@ -4627,7 +4627,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-20 04:09</t>
+          <t>refreshed 2026-10-20 05:34</t>
         </is>
       </c>
     </row>
@@ -7289,11 +7289,11 @@
         <v>93</v>
       </c>
       <c r="Q33" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>3 %</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -7383,11 +7383,11 @@
         <v>93</v>
       </c>
       <c r="Q34" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>3 %</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -7477,11 +7477,11 @@
         <v>2</v>
       </c>
       <c r="Q35" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>19 %</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -7571,11 +7571,11 @@
         <v>30</v>
       </c>
       <c r="Q36" t="n">
-        <v>0</v>
+        <v>60</v>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>complete</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -7665,11 +7665,11 @@
         <v>603</v>
       </c>
       <c r="Q37" t="n">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>23 %</t>
+          <t>37 %</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -7744,7 +7744,7 @@
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>PD45886_foldback2/PD45886</t>
+          <t>PD45886</t>
         </is>
       </c>
       <c r="N38" t="n">
@@ -7773,7 +7773,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>27 colonies, proj 2045; 73 private calls (B 7, C 10), 2570 germline MEIs; first run (489 = cruciform artefacts) in ~/Documents/hsc_results/PD45886; hsc_foldback lost 217 germline (strand bug)</t>
+          <t>27 colonies, proj 2045; 73 private calls (B 7, C 10), 2570 germline MEIs; superseded runs (first run: 489 cruciform artefacts; hsc_foldback: lost 217 germline, strand bug) moved to ~/Documents/hsc_results_superseded</t>
         </is>
       </c>
     </row>
@@ -8029,11 +8029,11 @@
         <v>11</v>
       </c>
       <c r="Q41" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>14 %</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -8895,11 +8895,11 @@
         <v>24</v>
       </c>
       <c r="Q51" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>not started</t>
+          <t>complete</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">

</xml_diff>

<commit_message>
Run tracker: PD45886 superseded runs deleted
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -3153,11 +3153,11 @@
         <v>2</v>
       </c>
       <c r="Q35" s="2" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="R35" s="2" t="inlineStr">
         <is>
-          <t>19 %</t>
+          <t>36 %</t>
         </is>
       </c>
       <c r="S35" s="5" t="inlineStr">
@@ -3449,7 +3449,7 @@
       </c>
       <c r="T38" s="3" t="inlineStr">
         <is>
-          <t>27 colonies, proj 2045; 73 private calls (B 7, C 10), 2570 germline MEIs; superseded runs (first run: 489 cruciform artefacts; hsc_foldback: lost 217 germline, strand bug) moved to ~/Documents/hsc_results_superseded</t>
+          <t>27 colonies, proj 2045; 73 private calls (B 7, C 10), 2570 germline MEIs; superseded runs (first run: 489 cruciform artefacts; hsc_foldback: lost 217 germline, strand bug) deleted 2026-10-20</t>
         </is>
       </c>
     </row>
@@ -7477,11 +7477,11 @@
         <v>2</v>
       </c>
       <c r="Q35" t="n">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>19 %</t>
+          <t>36 %</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -7773,7 +7773,7 @@
       </c>
       <c r="T38" t="inlineStr">
         <is>
-          <t>27 colonies, proj 2045; 73 private calls (B 7, C 10), 2570 germline MEIs; superseded runs (first run: 489 cruciform artefacts; hsc_foldback: lost 217 germline, strand bug) moved to ~/Documents/hsc_results_superseded</t>
+          <t>27 colonies, proj 2045; 73 private calls (B 7, C 10), 2570 germline MEIs; superseded runs (first run: 489 cruciform artefacts; hsc_foldback: lost 217 germline, strand bug) deleted 2026-10-20</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Run tracker: PD42191 matched normal PD42191m genotyped, trunk candidates
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -3153,11 +3153,11 @@
         <v>2</v>
       </c>
       <c r="Q35" s="2" t="n">
-        <v>17</v>
-      </c>
-      <c r="R35" s="2" t="inlineStr">
-        <is>
-          <t>36 %</t>
+        <v>46</v>
+      </c>
+      <c r="R35" s="4" t="inlineStr">
+        <is>
+          <t>complete</t>
         </is>
       </c>
       <c r="S35" s="5" t="inlineStr">
@@ -3334,11 +3334,11 @@
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
-          <t>21 / 46 / 88</t>
+          <t>16 / 50 / 89</t>
         </is>
       </c>
       <c r="P37" s="2" t="n">
-        <v>603</v>
+        <v>634</v>
       </c>
       <c r="Q37" s="2" t="n">
         <v>58</v>
@@ -3355,7 +3355,7 @@
       </c>
       <c r="T37" s="3" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD42191; done 2026-10-17, results copied 2026-10-18 to ~/Documents/hsc_results/PD42191</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD42191; done 2026-10-17, results copied 2026-10-18 to ~/Documents/hsc_results/PD42191; 2026-10-21 matched normal PD42191m (buccal WGS, proj 2045) genotyped (job 10898, a4662c4): 30 candidates excluded as germline (28 = joint N2/N15 8-colony clade, normal VAF 0.33 pooled), 29 ROOT loci absent from normal -&gt; trunk candidates (B 5 / C 9 / D 15); best: 3:191993028 + 5:179182535 + 9:138098950 Alu TPRT; PD42191o = TARGETED (proj 3163), unusable</t>
         </is>
       </c>
     </row>
@@ -4627,7 +4627,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-20 05:34</t>
+          <t>refreshed 2026-10-20 05:42</t>
         </is>
       </c>
     </row>
@@ -7477,11 +7477,11 @@
         <v>2</v>
       </c>
       <c r="Q35" t="n">
-        <v>17</v>
+        <v>46</v>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>36 %</t>
+          <t>complete</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -7658,11 +7658,11 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>21 / 46 / 88</t>
+          <t>16 / 50 / 89</t>
         </is>
       </c>
       <c r="P37" t="n">
-        <v>603</v>
+        <v>634</v>
       </c>
       <c r="Q37" t="n">
         <v>58</v>
@@ -7679,7 +7679,7 @@
       </c>
       <c r="T37" t="inlineStr">
         <is>
-          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD42191; done 2026-10-17, results copied 2026-10-18 to ~/Documents/hsc_results/PD42191</t>
+          <t>tree added 2026-10-10 (zeros outgroup dropped); colonies.tsv populated 2026-10-10 (iRODS, all tips); submitted 2026-10-17 (job IDs not recorded), native GRCh37, results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD42191; done 2026-10-17, results copied 2026-10-18 to ~/Documents/hsc_results/PD42191; 2026-10-21 matched normal PD42191m (buccal WGS, proj 2045) genotyped (job 10898, a4662c4): 30 candidates excluded as germline (28 = joint N2/N15 8-colony clade, normal VAF 0.33 pooled), 29 ROOT loci absent from normal -&gt; trunk candidates (B 5 / C 9 / D 15); best: 3:191993028 + 5:179182535 + 9:138098950 Alu TPRT; PD42191o = TARGETED (proj 3163), unusable</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Run tracker: Pair31 done; Pair28 combine_gt memory kill blocks the hsc_foldback2 chain
Chain order (chain.*.tsv): PD45889, SDS5, Pair31, Pair28, Pair38, PD47703, ...; each unit's
stage+discover waits on ended(previous cleanup). Pair28's combine_gt (344560) died on the 8 GB
cap with 240 colonies, so its cleanup (344561) is 'never satisfied' and the 12 units behind it
sit in PEND (9485 jobs). Fix: resubmit combine-genotypes at 32 GB and bmod the cleanup/annotate
dependencies onto the new job.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -1852,7 +1852,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>combine_gt failed</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="T19" s="3" t="inlineStr">
         <is>
-          <t>published Pair_10; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805</t>
+          <t>published Pair_10; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed</t>
         </is>
       </c>
     </row>
@@ -1924,7 +1924,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>combine_gt failed</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -1955,7 +1955,7 @@
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>published Pair_10; recipient is a CML patient (BCR::ABL1 pre-HSCT), Flu-Bu-ATG; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805</t>
+          <t>published Pair_10; recipient is a CML patient (BCR::ABL1 pre-HSCT), Flu-Bu-ATG; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed</t>
         </is>
       </c>
     </row>
@@ -1994,9 +1994,9 @@
       <c r="H21" s="2" t="n">
         <v>67</v>
       </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>queued</t>
+      <c r="I21" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
@@ -2027,7 +2027,7 @@
       </c>
       <c r="T21" s="3" t="inlineStr">
         <is>
-          <t>published Pair_6; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058)</t>
+          <t>published Pair_6; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058); chain finished 2026-10-21 (Pair31.somatic.xlsx on NFS), not yet copied to ~/Documents/hsc_results</t>
         </is>
       </c>
     </row>
@@ -2066,9 +2066,9 @@
       <c r="H22" s="2" t="n">
         <v>125</v>
       </c>
-      <c r="I22" s="2" t="inlineStr">
-        <is>
-          <t>queued</t>
+      <c r="I22" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -2099,7 +2099,7 @@
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>published Pair_6; recipient: cisplatin for oesophageal cancer after HSCT; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058)</t>
+          <t>published Pair_6; recipient: cisplatin for oesophageal cancer after HSCT; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058); chain finished 2026-10-21 (Pair31.somatic.xlsx on NFS), not yet copied to ~/Documents/hsc_results</t>
         </is>
       </c>
     </row>
@@ -4627,7 +4627,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-20 05:42</t>
+          <t>refreshed 2026-10-22 06:32</t>
         </is>
       </c>
     </row>
@@ -4702,7 +4702,7 @@
         <v>20</v>
       </c>
       <c r="C6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="D6" t="n">
         <v>0</v>
@@ -4759,7 +4759,7 @@
         <v>50</v>
       </c>
       <c r="C9" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D9" t="n">
         <v>23</v>
@@ -6176,7 +6176,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>combine_gt failed</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -6207,7 +6207,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>published Pair_10; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805</t>
+          <t>published Pair_10; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed</t>
         </is>
       </c>
     </row>
@@ -6248,7 +6248,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>combine_gt failed</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -6279,7 +6279,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>published Pair_10; recipient is a CML patient (BCR::ABL1 pre-HSCT), Flu-Bu-ATG; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805</t>
+          <t>published Pair_10; recipient is a CML patient (BCR::ABL1 pre-HSCT), Flu-Bu-ATG; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed</t>
         </is>
       </c>
     </row>
@@ -6320,7 +6320,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>done</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -6351,7 +6351,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>published Pair_6; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058)</t>
+          <t>published Pair_6; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058); chain finished 2026-10-21 (Pair31.somatic.xlsx on NFS), not yet copied to ~/Documents/hsc_results</t>
         </is>
       </c>
     </row>
@@ -6392,7 +6392,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>done</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -6423,7 +6423,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>published Pair_6; recipient: cisplatin for oesophageal cancer after HSCT; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058)</t>
+          <t>published Pair_6; recipient: cisplatin for oesophageal cancer after HSCT; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058); chain finished 2026-10-21 (Pair31.somatic.xlsx on NFS), not yet copied to ~/Documents/hsc_results</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Run tracker: Pair28 combine_gt resubmitted (511647, 32 GB), chain unblocked; 12 queued units regrouped to team273 and cg raised to 48 GB
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -759,7 +759,7 @@
       </c>
       <c r="T3" s="3" t="inlineStr">
         <is>
-          <t>old-pipeline results only (~/Documents/retrotransposons_sanger/results/PD47703); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344581, cleanup 344588, stage+discover waits on ended(344578), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD47703</t>
+          <t>old-pipeline results only (~/Documents/retrotransposons_sanger/results/PD47703); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344581, cleanup 344588, stage+discover waits on ended(344578), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD47703; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -835,7 +835,7 @@
       </c>
       <c r="T4" s="3" t="inlineStr">
         <is>
-          <t>SETTLED 2026-10-10: repopulated preferring GRCh38 -&gt; all 922 colonies GRCh38 (450 proj 2450, 472 proj 3819; old mixed file kept as colonies.tsv.bak.20261010040433). Old-pipeline results in ~/Documents/retrotransposons_sanger/results/PD45534; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh38, sd 344703, cleanup 344711, stage+discover waits on ended(344700), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD45534</t>
+          <t>SETTLED 2026-10-10: repopulated preferring GRCh38 -&gt; all 922 colonies GRCh38 (450 proj 2450, 472 proj 3819; old mixed file kept as colonies.tsv.bak.20261010040433). Old-pipeline results in ~/Documents/retrotransposons_sanger/results/PD45534; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh38, sd 344703, cleanup 344711, stage+discover waits on ended(344700), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD45534; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -911,7 +911,7 @@
       </c>
       <c r="T5" s="3" t="inlineStr">
         <is>
-          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344646, cleanup 344654, stage+discover waits on ended(344642), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair11_PD45792_PD45793</t>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344646, cleanup 344654, stage+discover waits on ended(344642), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair11_PD45792_PD45793; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -983,7 +983,7 @@
       </c>
       <c r="T6" s="3" t="inlineStr">
         <is>
-          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344646, cleanup 344654, stage+discover waits on ended(344642), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair11_PD45792_PD45793</t>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344646, cleanup 344654, stage+discover waits on ended(344642), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair11_PD45792_PD45793; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -1059,7 +1059,7 @@
       </c>
       <c r="T7" s="3" t="inlineStr">
         <is>
-          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344632, cleanup 344642, stage+discover waits on ended(344627), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair13_PD45794_PD45795</t>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344632, cleanup 344642, stage+discover waits on ended(344627), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair13_PD45794_PD45795; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -1131,7 +1131,7 @@
       </c>
       <c r="T8" s="3" t="inlineStr">
         <is>
-          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344632, cleanup 344642, stage+discover waits on ended(344627), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair13_PD45794_PD45795</t>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344632, cleanup 344642, stage+discover waits on ended(344627), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair13_PD45794_PD45795; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -1203,7 +1203,7 @@
       </c>
       <c r="T9" s="3" t="inlineStr">
         <is>
-          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809</t>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -1279,7 +1279,7 @@
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809</t>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -1351,7 +1351,7 @@
       </c>
       <c r="T11" s="3" t="inlineStr">
         <is>
-          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344592, cleanup 344598, stage+discover waits on ended(344588), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair40_PD45810_PD45811</t>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344592, cleanup 344598, stage+discover waits on ended(344588), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair40_PD45810_PD45811; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -1427,7 +1427,7 @@
       </c>
       <c r="T12" s="3" t="inlineStr">
         <is>
-          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344592, cleanup 344598, stage+discover waits on ended(344588), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair40_PD45810_PD45811</t>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344592, cleanup 344598, stage+discover waits on ended(344588), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair40_PD45810_PD45811; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -1852,7 +1852,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>combine_gt failed</t>
+          <t>combine_gt resubmitted</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -1883,7 +1883,7 @@
       </c>
       <c r="T19" s="3" t="inlineStr">
         <is>
-          <t>published Pair_10; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed</t>
+          <t>published Pair_10; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed; 2026-10-22 FIXED: combine-genotypes resubmitted as job 511647 at 32 GB (jobids.tsv cg2), cleanup 344561 + annotate 344562 bmod -w done(511647), report 344564 re-armed; chain resumes on its own</t>
         </is>
       </c>
     </row>
@@ -1924,7 +1924,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>combine_gt failed</t>
+          <t>combine_gt resubmitted</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -1955,7 +1955,7 @@
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>published Pair_10; recipient is a CML patient (BCR::ABL1 pre-HSCT), Flu-Bu-ATG; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed</t>
+          <t>published Pair_10; recipient is a CML patient (BCR::ABL1 pre-HSCT), Flu-Bu-ATG; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed; 2026-10-22 FIXED: combine-genotypes resubmitted as job 511647 at 32 GB (jobids.tsv cg2), cleanup 344561 + annotate 344562 bmod -w done(511647), report 344564 re-armed; chain resumes on its own</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2171,7 @@
       </c>
       <c r="T23" s="3" t="inlineStr">
         <is>
-          <t>published Pair_2; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344601, cleanup 344613, stage+discover waits on ended(344598), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair41_PD45812_PD45813</t>
+          <t>published Pair_2; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344601, cleanup 344613, stage+discover waits on ended(344598), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair41_PD45812_PD45813; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -2243,7 +2243,7 @@
       </c>
       <c r="T24" s="3" t="inlineStr">
         <is>
-          <t>published Pair_2; sex-mismatched pair (F donor -&gt; M recipient); added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344601, cleanup 344613, stage+discover waits on ended(344598), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair41_PD45812_PD45813</t>
+          <t>published Pair_2; sex-mismatched pair (F donor -&gt; M recipient); added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344601, cleanup 344613, stage+discover waits on ended(344598), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair41_PD45812_PD45813; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -2409,7 +2409,7 @@
       </c>
       <c r="T26" s="3" t="inlineStr">
         <is>
-          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344657, cleanup 344664, stage+discover waits on ended(344654), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD49226</t>
+          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344657, cleanup 344664, stage+discover waits on ended(344654), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD49226; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -2481,7 +2481,7 @@
       </c>
       <c r="T27" s="3" t="inlineStr">
         <is>
-          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344667, cleanup 344676, stage+discover waits on ended(344664), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD49227</t>
+          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344667, cleanup 344676, stage+discover waits on ended(344664), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD49227; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -2553,7 +2553,7 @@
       </c>
       <c r="T28" s="3" t="inlineStr">
         <is>
-          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344680, cleanup 344686, stage+discover waits on ended(344676), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD49228</t>
+          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344680, cleanup 344686, stage+discover waits on ended(344676), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD49228; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -2625,7 +2625,7 @@
       </c>
       <c r="T29" s="3" t="inlineStr">
         <is>
-          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344692, cleanup 344700, stage+discover waits on ended(344686), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD53373</t>
+          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344692, cleanup 344700, stage+discover waits on ended(344686), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD53373; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -2697,7 +2697,7 @@
       </c>
       <c r="T30" s="3" t="inlineStr">
         <is>
-          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344620, cleanup 344627, stage+discover waits on ended(344613), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD53374</t>
+          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344620, cleanup 344627, stage+discover waits on ended(344613), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD53374; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -4627,7 +4627,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-22 06:32</t>
+          <t>refreshed 2026-10-22 07:00</t>
         </is>
       </c>
     </row>
@@ -5083,7 +5083,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>old-pipeline results only (~/Documents/retrotransposons_sanger/results/PD47703); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344581, cleanup 344588, stage+discover waits on ended(344578), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD47703</t>
+          <t>old-pipeline results only (~/Documents/retrotransposons_sanger/results/PD47703); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344581, cleanup 344588, stage+discover waits on ended(344578), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD47703; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -5159,7 +5159,7 @@
       </c>
       <c r="T4" t="inlineStr">
         <is>
-          <t>SETTLED 2026-10-10: repopulated preferring GRCh38 -&gt; all 922 colonies GRCh38 (450 proj 2450, 472 proj 3819; old mixed file kept as colonies.tsv.bak.20261010040433). Old-pipeline results in ~/Documents/retrotransposons_sanger/results/PD45534; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh38, sd 344703, cleanup 344711, stage+discover waits on ended(344700), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD45534</t>
+          <t>SETTLED 2026-10-10: repopulated preferring GRCh38 -&gt; all 922 colonies GRCh38 (450 proj 2450, 472 proj 3819; old mixed file kept as colonies.tsv.bak.20261010040433). Old-pipeline results in ~/Documents/retrotransposons_sanger/results/PD45534; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh38, sd 344703, cleanup 344711, stage+discover waits on ended(344700), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD45534; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -5235,7 +5235,7 @@
       </c>
       <c r="T5" t="inlineStr">
         <is>
-          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344646, cleanup 344654, stage+discover waits on ended(344642), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair11_PD45792_PD45793</t>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344646, cleanup 344654, stage+discover waits on ended(344642), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair11_PD45792_PD45793; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -5307,7 +5307,7 @@
       </c>
       <c r="T6" t="inlineStr">
         <is>
-          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344646, cleanup 344654, stage+discover waits on ended(344642), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair11_PD45792_PD45793</t>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344646, cleanup 344654, stage+discover waits on ended(344642), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair11_PD45792_PD45793; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -5383,7 +5383,7 @@
       </c>
       <c r="T7" t="inlineStr">
         <is>
-          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344632, cleanup 344642, stage+discover waits on ended(344627), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair13_PD45794_PD45795</t>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344632, cleanup 344642, stage+discover waits on ended(344627), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair13_PD45794_PD45795; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -5455,7 +5455,7 @@
       </c>
       <c r="T8" t="inlineStr">
         <is>
-          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344632, cleanup 344642, stage+discover waits on ended(344627), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair13_PD45794_PD45795</t>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344632, cleanup 344642, stage+discover waits on ended(344627), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair13_PD45794_PD45795; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -5527,7 +5527,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809</t>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -5603,7 +5603,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809</t>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -5675,7 +5675,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344592, cleanup 344598, stage+discover waits on ended(344588), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair40_PD45810_PD45811</t>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344592, cleanup 344598, stage+discover waits on ended(344588), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair40_PD45810_PD45811; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -5751,7 +5751,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344592, cleanup 344598, stage+discover waits on ended(344588), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair40_PD45810_PD45811</t>
+          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344592, cleanup 344598, stage+discover waits on ended(344588), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair40_PD45810_PD45811; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -6176,7 +6176,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>combine_gt failed</t>
+          <t>combine_gt resubmitted</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -6207,7 +6207,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>published Pair_10; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed</t>
+          <t>published Pair_10; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed; 2026-10-22 FIXED: combine-genotypes resubmitted as job 511647 at 32 GB (jobids.tsv cg2), cleanup 344561 + annotate 344562 bmod -w done(511647), report 344564 re-armed; chain resumes on its own</t>
         </is>
       </c>
     </row>
@@ -6248,7 +6248,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>combine_gt failed</t>
+          <t>combine_gt resubmitted</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -6279,7 +6279,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>published Pair_10; recipient is a CML patient (BCR::ABL1 pre-HSCT), Flu-Bu-ATG; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed</t>
+          <t>published Pair_10; recipient is a CML patient (BCR::ABL1 pre-HSCT), Flu-Bu-ATG; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed; 2026-10-22 FIXED: combine-genotypes resubmitted as job 511647 at 32 GB (jobids.tsv cg2), cleanup 344561 + annotate 344562 bmod -w done(511647), report 344564 re-armed; chain resumes on its own</t>
         </is>
       </c>
     </row>
@@ -6495,7 +6495,7 @@
       </c>
       <c r="T23" t="inlineStr">
         <is>
-          <t>published Pair_2; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344601, cleanup 344613, stage+discover waits on ended(344598), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair41_PD45812_PD45813</t>
+          <t>published Pair_2; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344601, cleanup 344613, stage+discover waits on ended(344598), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair41_PD45812_PD45813; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -6567,7 +6567,7 @@
       </c>
       <c r="T24" t="inlineStr">
         <is>
-          <t>published Pair_2; sex-mismatched pair (F donor -&gt; M recipient); added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344601, cleanup 344613, stage+discover waits on ended(344598), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair41_PD45812_PD45813</t>
+          <t>published Pair_2; sex-mismatched pair (F donor -&gt; M recipient); added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344601, cleanup 344613, stage+discover waits on ended(344598), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair41_PD45812_PD45813; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -6733,7 +6733,7 @@
       </c>
       <c r="T26" t="inlineStr">
         <is>
-          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344657, cleanup 344664, stage+discover waits on ended(344654), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD49226</t>
+          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344657, cleanup 344664, stage+discover waits on ended(344654), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD49226; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -6805,7 +6805,7 @@
       </c>
       <c r="T27" t="inlineStr">
         <is>
-          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344667, cleanup 344676, stage+discover waits on ended(344664), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD49227</t>
+          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344667, cleanup 344676, stage+discover waits on ended(344664), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD49227; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -6877,7 +6877,7 @@
       </c>
       <c r="T28" t="inlineStr">
         <is>
-          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344680, cleanup 344686, stage+discover waits on ended(344676), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD49228</t>
+          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344680, cleanup 344686, stage+discover waits on ended(344676), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD49228; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -6949,7 +6949,7 @@
       </c>
       <c r="T29" t="inlineStr">
         <is>
-          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344692, cleanup 344700, stage+discover waits on ended(344686), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD53373</t>
+          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344692, cleanup 344700, stage+discover waits on ended(344686), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD53373; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>
@@ -7021,7 +7021,7 @@
       </c>
       <c r="T30" t="inlineStr">
         <is>
-          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344620, cleanup 344627, stage+discover waits on ended(344613), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD53374</t>
+          <t>colonies.tsv populated 2026-07-18 (nst_links), all hs37d5; folder still patients/unknown_tissue_bcl (should be re-filed as blood); added 2026-10-15 (whole SCD cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344620, cleanup 344627, stage+discover waits on ended(344613), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD53374; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Run tracker: Pair38 restarted (sd 381006 / sdr 381008) after stageBam's inner bsub died on the stale LSF group; gates armed on all 12 queued units
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -60,12 +60,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F2F2F2"/>
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -95,10 +95,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -1170,9 +1170,9 @@
       <c r="H9" s="2" t="n">
         <v>143</v>
       </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>queued</t>
+      <c r="I9" s="6" t="inlineStr">
+        <is>
+          <t>running</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1246,9 +1246,9 @@
       <c r="H10" s="2" t="n">
         <v>109</v>
       </c>
-      <c r="I10" s="2" t="inlineStr">
-        <is>
-          <t>queued</t>
+      <c r="I10" s="6" t="inlineStr">
+        <is>
+          <t>running</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -2009,17 +2009,35 @@
           <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
         </is>
       </c>
-      <c r="L21" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M21" s="2" t="inlineStr"/>
-      <c r="N21" s="2" t="inlineStr"/>
-      <c r="O21" s="2" t="inlineStr"/>
-      <c r="P21" s="2" t="inlineStr"/>
-      <c r="Q21" s="2" t="inlineStr"/>
-      <c r="R21" s="2" t="inlineStr"/>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>Pair31_PD45806_PD45807</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="n">
+        <v>187</v>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>10 / 13 / 164</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="n">
+        <v>149</v>
+      </c>
+      <c r="Q21" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" s="5" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S21" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -2081,17 +2099,35 @@
           <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
         </is>
       </c>
-      <c r="L22" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="inlineStr"/>
-      <c r="N22" s="2" t="inlineStr"/>
-      <c r="O22" s="2" t="inlineStr"/>
-      <c r="P22" s="2" t="inlineStr"/>
-      <c r="Q22" s="2" t="inlineStr"/>
-      <c r="R22" s="2" t="inlineStr"/>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>Pair31_PD45806_PD45807</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="n">
+        <v>187</v>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>10 / 13 / 164</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="n">
+        <v>149</v>
+      </c>
+      <c r="Q22" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" s="5" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S22" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -4627,7 +4663,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-22 07:00</t>
+          <t>refreshed 2026-10-25 09:07</t>
         </is>
       </c>
     </row>
@@ -4705,7 +4741,7 @@
         <v>2</v>
       </c>
       <c r="D6" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -4762,7 +4798,7 @@
         <v>24</v>
       </c>
       <c r="D9" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -5496,7 +5532,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>running</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -5572,7 +5608,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>running</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -6335,15 +6371,33 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr"/>
-      <c r="N21" t="inlineStr"/>
-      <c r="O21" t="inlineStr"/>
-      <c r="P21" t="inlineStr"/>
-      <c r="Q21" t="inlineStr"/>
-      <c r="R21" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Pair31_PD45806_PD45807</t>
+        </is>
+      </c>
+      <c r="N21" t="n">
+        <v>187</v>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>10 / 13 / 164</t>
+        </is>
+      </c>
+      <c r="P21" t="n">
+        <v>149</v>
+      </c>
+      <c r="Q21" t="n">
+        <v>0</v>
+      </c>
+      <c r="R21" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S21" t="inlineStr">
         <is>
           <t>no</t>
@@ -6407,15 +6461,33 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr"/>
-      <c r="N22" t="inlineStr"/>
-      <c r="O22" t="inlineStr"/>
-      <c r="P22" t="inlineStr"/>
-      <c r="Q22" t="inlineStr"/>
-      <c r="R22" t="inlineStr"/>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Pair31_PD45806_PD45807</t>
+        </is>
+      </c>
+      <c r="N22" t="n">
+        <v>187</v>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>10 / 13 / 164</t>
+        </is>
+      </c>
+      <c r="P22" t="n">
+        <v>149</v>
+      </c>
+      <c r="Q22" t="n">
+        <v>0</v>
+      </c>
+      <c r="R22" t="inlineStr">
+        <is>
+          <t>not started</t>
+        </is>
+      </c>
       <c r="S22" t="inlineStr">
         <is>
           <t>no</t>

</xml_diff>

<commit_message>
Run tracker: Pair28/Pair31 discovery half OOM-excluded, Pair38 failed at combine, PD47703 done, Pair40 running; fetch also reads hsc_rediscover
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -660,14 +660,16 @@
         </is>
       </c>
       <c r="N2" s="2" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>1 / 2 / 17</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr"/>
+          <t>0 / 2 / 12</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="n">
+        <v>6</v>
+      </c>
       <c r="Q2" s="2" t="n">
         <v>20</v>
       </c>
@@ -726,9 +728,9 @@
       <c r="H3" s="2" t="n">
         <v>259</v>
       </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>queued</t>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>done</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -741,17 +743,25 @@
           <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
         </is>
       </c>
-      <c r="L3" s="5" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="inlineStr"/>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>PD47703</t>
+        </is>
+      </c>
       <c r="N3" s="2" t="inlineStr"/>
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
-      <c r="R3" s="2" t="inlineStr"/>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>no somatic table</t>
+        </is>
+      </c>
       <c r="S3" s="5" t="inlineStr">
         <is>
           <t>no</t>
@@ -759,7 +769,7 @@
       </c>
       <c r="T3" s="3" t="inlineStr">
         <is>
-          <t>old-pipeline results only (~/Documents/retrotransposons_sanger/results/PD47703); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344581, cleanup 344588, stage+discover waits on ended(344578), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD47703; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
+          <t>old-pipeline results only (~/Documents/retrotransposons_sanger/results/PD47703); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344581, cleanup 344588, stage+discover waits on ended(344578), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD47703; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 259/259 discovered + genotyped, calls present (report status: see fetch)</t>
         </is>
       </c>
     </row>
@@ -1170,9 +1180,9 @@
       <c r="H9" s="2" t="n">
         <v>143</v>
       </c>
-      <c r="I9" s="6" t="inlineStr">
-        <is>
-          <t>running</t>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>failed (combine)</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
@@ -1203,7 +1213,7 @@
       </c>
       <c r="T9" s="3" t="inlineStr">
         <is>
-          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
+          <t>chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 64 GB rediscovery (sd 549176/sdr 549178) finished 2026-10-27 21:45, then combine 344574 apparently died ~22:16 (log under investigation); gate 549226 logged "unknown" (EXIT purged before it ran), killed the unit and deleted its staged BAMs, released PD47703-&gt;Pair40</t>
         </is>
       </c>
     </row>
@@ -1246,9 +1256,9 @@
       <c r="H10" s="2" t="n">
         <v>109</v>
       </c>
-      <c r="I10" s="6" t="inlineStr">
-        <is>
-          <t>running</t>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>failed (combine)</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
@@ -1279,7 +1289,7 @@
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
+          <t>chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 64 GB rediscovery (sd 549176/sdr 549178) finished 2026-10-27 21:45, then combine 344574 apparently died ~22:16 (log under investigation); gate 549226 logged "unknown" (EXIT purged before it ran), killed the unit and deleted its staged BAMs, released PD47703-&gt;Pair40</t>
         </is>
       </c>
     </row>
@@ -1318,9 +1328,9 @@
       <c r="H11" s="2" t="n">
         <v>143</v>
       </c>
-      <c r="I11" s="2" t="inlineStr">
-        <is>
-          <t>queued</t>
+      <c r="I11" s="6" t="inlineStr">
+        <is>
+          <t>running</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
@@ -1351,7 +1361,7 @@
       </c>
       <c r="T11" s="3" t="inlineStr">
         <is>
-          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344592, cleanup 344598, stage+discover waits on ended(344588), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair40_PD45810_PD45811; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
+          <t>chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344592, cleanup 344598, stage+discover waits on ended(344588), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair40_PD45810_PD45811; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: stage+discover running (chain released by the Pair38 gate 2026-10-27)</t>
         </is>
       </c>
     </row>
@@ -1394,9 +1404,9 @@
       <c r="H12" s="2" t="n">
         <v>136</v>
       </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>queued</t>
+      <c r="I12" s="6" t="inlineStr">
+        <is>
+          <t>running</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
@@ -1427,7 +1437,7 @@
       </c>
       <c r="T12" s="3" t="inlineStr">
         <is>
-          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344592, cleanup 344598, stage+discover waits on ended(344588), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair40_PD45810_PD45811; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
+          <t>chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344592, cleanup 344598, stage+discover waits on ended(344588), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair40_PD45810_PD45811; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: stage+discover running (chain released by the Pair38 gate 2026-10-27)</t>
         </is>
       </c>
     </row>
@@ -1852,7 +1862,7 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>combine_gt resubmitted</t>
+          <t>INCOMPLETE: discovery OOM</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
@@ -1883,7 +1893,7 @@
       </c>
       <c r="T19" s="3" t="inlineStr">
         <is>
-          <t>published Pair_10; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed; 2026-10-22 FIXED: combine-genotypes resubmitted as job 511647 at 32 GB (jobids.tsv cg2), cleanup 344561 + annotate 344562 bmod -w done(511647), report 344564 re-armed; chain resumes on its own</t>
+          <t>published Pair_10; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed; 2026-10-22 FIXED: combine-genotypes resubmitted as job 511647 at 32 GB (jobids.tsv cg2), cleanup 344561 + annotate 344562 bmod -w done(511647), report 344564 re-armed; chain resumes on its own; 2026-10-31: calls exist but discover_excluded = 119/240 colonies OOM at the old 32 GB tier2 (48 PD45804 + 71 PD45805); rerun of the 119 at 64 GB in hsc_rediscover</t>
         </is>
       </c>
     </row>
@@ -1924,7 +1934,7 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>combine_gt resubmitted</t>
+          <t>INCOMPLETE: discovery OOM</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
@@ -1955,7 +1965,7 @@
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>published Pair_10; recipient is a CML patient (BCR::ABL1 pre-HSCT), Flu-Bu-ATG; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed; 2026-10-22 FIXED: combine-genotypes resubmitted as job 511647 at 32 GB (jobids.tsv cg2), cleanup 344561 + annotate 344562 bmod -w done(511647), report 344564 re-armed; chain resumes on its own</t>
+          <t>published Pair_10; recipient is a CML patient (BCR::ABL1 pre-HSCT), Flu-Bu-ATG; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed; 2026-10-22 FIXED: combine-genotypes resubmitted as job 511647 at 32 GB (jobids.tsv cg2), cleanup 344561 + annotate 344562 bmod -w done(511647), report 344564 re-armed; chain resumes on its own; 2026-10-31: calls exist but discover_excluded = 119/240 colonies OOM at the old 32 GB tier2 (48 PD45804 + 71 PD45805); rerun of the 119 at 64 GB in hsc_rediscover</t>
         </is>
       </c>
     </row>
@@ -1994,9 +2004,9 @@
       <c r="H21" s="2" t="n">
         <v>67</v>
       </c>
-      <c r="I21" s="4" t="inlineStr">
-        <is>
-          <t>done</t>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>INCOMPLETE: discovery OOM</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
@@ -2045,7 +2055,7 @@
       </c>
       <c r="T21" s="3" t="inlineStr">
         <is>
-          <t>published Pair_6; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058); chain finished 2026-10-21 (Pair31.somatic.xlsx on NFS), not yet copied to ~/Documents/hsc_results</t>
+          <t>published Pair_6; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058); chain finished 2026-10-21 (Pair31.somatic.xlsx on NFS), not yet copied to ~/Documents/hsc_results; 2026-10-31: discover_excluded = 142/192 colonies OOM at the old 32 GB tier2 (64 PD45806 + 78 PD45807) -&gt; local results cover discovery in only 50 colonies; rerun of the 142 at 64 GB in hsc_rediscover (old discovery hard-linked)</t>
         </is>
       </c>
     </row>
@@ -2084,9 +2094,9 @@
       <c r="H22" s="2" t="n">
         <v>125</v>
       </c>
-      <c r="I22" s="4" t="inlineStr">
-        <is>
-          <t>done</t>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>INCOMPLETE: discovery OOM</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
@@ -2135,7 +2145,7 @@
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>published Pair_6; recipient: cisplatin for oesophageal cancer after HSCT; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058); chain finished 2026-10-21 (Pair31.somatic.xlsx on NFS), not yet copied to ~/Documents/hsc_results</t>
+          <t>published Pair_6; recipient: cisplatin for oesophageal cancer after HSCT; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058); chain finished 2026-10-21 (Pair31.somatic.xlsx on NFS), not yet copied to ~/Documents/hsc_results; 2026-10-31: discover_excluded = 142/192 colonies OOM at the old 32 GB tier2 (64 PD45806 + 78 PD45807) -&gt; local results cover discovery in only 50 colonies; rerun of the 142 at 64 GB in hsc_rediscover (old discovery hard-linked)</t>
         </is>
       </c>
     </row>
@@ -4663,7 +4673,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-25 09:07</t>
+          <t>refreshed 2026-10-31 07:08</t>
         </is>
       </c>
     </row>
@@ -4700,7 +4710,7 @@
         <v>18</v>
       </c>
       <c r="C4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D4" t="n">
         <v>12</v>
@@ -4738,7 +4748,7 @@
         <v>20</v>
       </c>
       <c r="C6" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D6" t="n">
         <v>2</v>
@@ -4795,7 +4805,7 @@
         <v>50</v>
       </c>
       <c r="C9" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D9" t="n">
         <v>25</v>
@@ -5020,14 +5030,16 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>1 / 2 / 17</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr"/>
+          <t>0 / 2 / 12</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
+        <v>6</v>
+      </c>
       <c r="Q2" t="n">
         <v>20</v>
       </c>
@@ -5088,7 +5100,7 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>done</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -5103,15 +5115,23 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr"/>
+          <t>partial</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>PD47703</t>
+        </is>
+      </c>
       <c r="N3" t="inlineStr"/>
       <c r="O3" t="inlineStr"/>
       <c r="P3" t="inlineStr"/>
       <c r="Q3" t="inlineStr"/>
-      <c r="R3" t="inlineStr"/>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>no somatic table</t>
+        </is>
+      </c>
       <c r="S3" t="inlineStr">
         <is>
           <t>no</t>
@@ -5119,7 +5139,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>old-pipeline results only (~/Documents/retrotransposons_sanger/results/PD47703); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344581, cleanup 344588, stage+discover waits on ended(344578), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD47703; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
+          <t>old-pipeline results only (~/Documents/retrotransposons_sanger/results/PD47703); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344581, cleanup 344588, stage+discover waits on ended(344578), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD47703; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 259/259 discovered + genotyped, calls present (report status: see fetch)</t>
         </is>
       </c>
     </row>
@@ -5532,7 +5552,7 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>failed (combine)</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -5563,7 +5583,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
+          <t>chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 64 GB rediscovery (sd 549176/sdr 549178) finished 2026-10-27 21:45, then combine 344574 apparently died ~22:16 (log under investigation); gate 549226 logged "unknown" (EXIT purged before it ran), killed the unit and deleted its staged BAMs, released PD47703-&gt;Pair40</t>
         </is>
       </c>
     </row>
@@ -5608,7 +5628,7 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>running</t>
+          <t>failed (combine)</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -5639,7 +5659,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
+          <t>chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 64 GB rediscovery (sd 549176/sdr 549178) finished 2026-10-27 21:45, then combine 344574 apparently died ~22:16 (log under investigation); gate 549226 logged "unknown" (EXIT purged before it ran), killed the unit and deleted its staged BAMs, released PD47703-&gt;Pair40</t>
         </is>
       </c>
     </row>
@@ -5680,7 +5700,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>running</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -5711,7 +5731,7 @@
       </c>
       <c r="T11" t="inlineStr">
         <is>
-          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344592, cleanup 344598, stage+discover waits on ended(344588), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair40_PD45810_PD45811; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
+          <t>chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344592, cleanup 344598, stage+discover waits on ended(344588), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair40_PD45810_PD45811; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: stage+discover running (chain released by the Pair38 gate 2026-10-27)</t>
         </is>
       </c>
     </row>
@@ -5756,7 +5776,7 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>queued</t>
+          <t>running</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -5787,7 +5807,7 @@
       </c>
       <c r="T12" t="inlineStr">
         <is>
-          <t>; chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344592, cleanup 344598, stage+discover waits on ended(344588), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair40_PD45810_PD45811; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M)</t>
+          <t>chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344592, cleanup 344598, stage+discover waits on ended(344588), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair40_PD45810_PD45811; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: stage+discover running (chain released by the Pair38 gate 2026-10-27)</t>
         </is>
       </c>
     </row>
@@ -6212,7 +6232,7 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>combine_gt resubmitted</t>
+          <t>INCOMPLETE: discovery OOM</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -6243,7 +6263,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>published Pair_10; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed; 2026-10-22 FIXED: combine-genotypes resubmitted as job 511647 at 32 GB (jobids.tsv cg2), cleanup 344561 + annotate 344562 bmod -w done(511647), report 344564 re-armed; chain resumes on its own</t>
+          <t>published Pair_10; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed; 2026-10-22 FIXED: combine-genotypes resubmitted as job 511647 at 32 GB (jobids.tsv cg2), cleanup 344561 + annotate 344562 bmod -w done(511647), report 344564 re-armed; chain resumes on its own; 2026-10-31: calls exist but discover_excluded = 119/240 colonies OOM at the old 32 GB tier2 (48 PD45804 + 71 PD45805); rerun of the 119 at 64 GB in hsc_rediscover</t>
         </is>
       </c>
     </row>
@@ -6284,7 +6304,7 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>combine_gt resubmitted</t>
+          <t>INCOMPLETE: discovery OOM</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -6315,7 +6335,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>published Pair_10; recipient is a CML patient (BCR::ABL1 pre-HSCT), Flu-Bu-ATG; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed; 2026-10-22 FIXED: combine-genotypes resubmitted as job 511647 at 32 GB (jobids.tsv cg2), cleanup 344561 + annotate 344562 bmod -w done(511647), report 344564 re-armed; chain resumes on its own</t>
+          <t>published Pair_10; recipient is a CML patient (BCR::ABL1 pre-HSCT), Flu-Bu-ATG; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed; 2026-10-22 FIXED: combine-genotypes resubmitted as job 511647 at 32 GB (jobids.tsv cg2), cleanup 344561 + annotate 344562 bmod -w done(511647), report 344564 re-armed; chain resumes on its own; 2026-10-31: calls exist but discover_excluded = 119/240 colonies OOM at the old 32 GB tier2 (48 PD45804 + 71 PD45805); rerun of the 119 at 64 GB in hsc_rediscover</t>
         </is>
       </c>
     </row>
@@ -6356,7 +6376,7 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>INCOMPLETE: discovery OOM</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -6405,7 +6425,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>published Pair_6; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058); chain finished 2026-10-21 (Pair31.somatic.xlsx on NFS), not yet copied to ~/Documents/hsc_results</t>
+          <t>published Pair_6; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058); chain finished 2026-10-21 (Pair31.somatic.xlsx on NFS), not yet copied to ~/Documents/hsc_results; 2026-10-31: discover_excluded = 142/192 colonies OOM at the old 32 GB tier2 (64 PD45806 + 78 PD45807) -&gt; local results cover discovery in only 50 colonies; rerun of the 142 at 64 GB in hsc_rediscover (old discovery hard-linked)</t>
         </is>
       </c>
     </row>
@@ -6446,7 +6466,7 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>done</t>
+          <t>INCOMPLETE: discovery OOM</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -6495,7 +6515,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>published Pair_6; recipient: cisplatin for oesophageal cancer after HSCT; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058); chain finished 2026-10-21 (Pair31.somatic.xlsx on NFS), not yet copied to ~/Documents/hsc_results</t>
+          <t>published Pair_6; recipient: cisplatin for oesophageal cancer after HSCT; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058); chain finished 2026-10-21 (Pair31.somatic.xlsx on NFS), not yet copied to ~/Documents/hsc_results; 2026-10-31: discover_excluded = 142/192 colonies OOM at the old 32 GB tier2 (64 PD45806 + 78 PD45807) -&gt; local results cover discovery in only 50 colonies; rerun of the 142 at 64 GB in hsc_rediscover (old discovery hard-linked)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Run tracker: Pair38 failure = combine OOM at 16 GB
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -743,9 +743,9 @@
           <t>1fcdc92 (annotate SV lift + PROVIRUS_LTR, somatic_table beta-binomial het gate); checkout f01828e (+ hsc_chain.sh, no pipeline change)</t>
         </is>
       </c>
-      <c r="L3" s="6" t="inlineStr">
-        <is>
-          <t>partial</t>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>yes</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
@@ -753,13 +753,23 @@
           <t>PD47703</t>
         </is>
       </c>
-      <c r="N3" s="2" t="inlineStr"/>
-      <c r="O3" s="2" t="inlineStr"/>
-      <c r="P3" s="2" t="inlineStr"/>
-      <c r="Q3" s="2" t="inlineStr"/>
-      <c r="R3" s="2" t="inlineStr">
-        <is>
-          <t>no somatic table</t>
+      <c r="N3" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>15 / 8 / 19</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="Q3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" s="5" t="inlineStr">
+        <is>
+          <t>not started</t>
         </is>
       </c>
       <c r="S3" s="5" t="inlineStr">
@@ -1213,7 +1223,7 @@
       </c>
       <c r="T9" s="3" t="inlineStr">
         <is>
-          <t>chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 64 GB rediscovery (sd 549176/sdr 549178) finished 2026-10-27 21:45, then combine 344574 apparently died ~22:16 (log under investigation); gate 549226 logged "unknown" (EXIT purged before it ran), killed the unit and deleted its staged BAMs, released PD47703-&gt;Pair40</t>
+          <t>chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 64 GB rediscovery (sd 549176/sdr 549178) finished 2026-10-27 21:45, then combine 344574 TERM_MEMLIMIT at 16 GB (6.46M insertions) 2026-10-27 22:16; 3 colonies discovery "error"; rerun in hsc_rediscover with CI_MEM 128 GB; gate 549226 logged "unknown" (EXIT purged before it ran), killed the unit and deleted its staged BAMs, released PD47703-&gt;Pair40</t>
         </is>
       </c>
     </row>
@@ -1289,7 +1299,7 @@
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 64 GB rediscovery (sd 549176/sdr 549178) finished 2026-10-27 21:45, then combine 344574 apparently died ~22:16 (log under investigation); gate 549226 logged "unknown" (EXIT purged before it ran), killed the unit and deleted its staged BAMs, released PD47703-&gt;Pair40</t>
+          <t>chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 64 GB rediscovery (sd 549176/sdr 549178) finished 2026-10-27 21:45, then combine 344574 TERM_MEMLIMIT at 16 GB (6.46M insertions) 2026-10-27 22:16; 3 colonies discovery "error"; rerun in hsc_rediscover with CI_MEM 128 GB; gate 549226 logged "unknown" (EXIT purged before it ran), killed the unit and deleted its staged BAMs, released PD47703-&gt;Pair40</t>
         </is>
       </c>
     </row>
@@ -4673,7 +4683,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-31 07:08</t>
+          <t>refreshed 2026-10-31 07:10</t>
         </is>
       </c>
     </row>
@@ -4713,7 +4723,7 @@
         <v>12</v>
       </c>
       <c r="D4" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
@@ -4808,7 +4818,7 @@
         <v>23</v>
       </c>
       <c r="D9" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E9" t="n">
         <v>0</v>
@@ -5115,7 +5125,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>partial</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -5123,13 +5133,23 @@
           <t>PD47703</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
-      <c r="P3" t="inlineStr"/>
-      <c r="Q3" t="inlineStr"/>
+      <c r="N3" t="n">
+        <v>42</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>15 / 8 / 19</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>38</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>no somatic table</t>
+          <t>not started</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -5583,7 +5603,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 64 GB rediscovery (sd 549176/sdr 549178) finished 2026-10-27 21:45, then combine 344574 apparently died ~22:16 (log under investigation); gate 549226 logged "unknown" (EXIT purged before it ran), killed the unit and deleted its staged BAMs, released PD47703-&gt;Pair40</t>
+          <t>chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 64 GB rediscovery (sd 549176/sdr 549178) finished 2026-10-27 21:45, then combine 344574 TERM_MEMLIMIT at 16 GB (6.46M insertions) 2026-10-27 22:16; 3 colonies discovery "error"; rerun in hsc_rediscover with CI_MEM 128 GB; gate 549226 logged "unknown" (EXIT purged before it ran), killed the unit and deleted its staged BAMs, released PD47703-&gt;Pair40</t>
         </is>
       </c>
     </row>
@@ -5659,7 +5679,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 64 GB rediscovery (sd 549176/sdr 549178) finished 2026-10-27 21:45, then combine 344574 apparently died ~22:16 (log under investigation); gate 549226 logged "unknown" (EXIT purged before it ran), killed the unit and deleted its staged BAMs, released PD47703-&gt;Pair40</t>
+          <t>chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 64 GB rediscovery (sd 549176/sdr 549178) finished 2026-10-27 21:45, then combine 344574 TERM_MEMLIMIT at 16 GB (6.46M insertions) 2026-10-27 22:16; 3 colonies discovery "error"; rerun in hsc_rediscover with CI_MEM 128 GB; gate 549226 logged "unknown" (EXIT purged before it ran), killed the unit and deleted its staged BAMs, released PD47703-&gt;Pair40</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Run tracker: Pair28 + Pair31 rerun submitted in hsc_rediscover
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -1872,12 +1872,12 @@
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE: discovery OOM</t>
+          <t>rerun running</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair28_PD45804_PD45805/Pair28_PD45804_PD45805</t>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_rediscover/Pair28_PD45804_PD45805/Pair28_PD45804_PD45805</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1903,7 +1903,7 @@
       </c>
       <c r="T19" s="3" t="inlineStr">
         <is>
-          <t>published Pair_10; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed; 2026-10-22 FIXED: combine-genotypes resubmitted as job 511647 at 32 GB (jobids.tsv cg2), cleanup 344561 + annotate 344562 bmod -w done(511647), report 344564 re-armed; chain resumes on its own; 2026-10-31: calls exist but discover_excluded = 119/240 colonies OOM at the old 32 GB tier2 (48 PD45804 + 71 PD45805); rerun of the 119 at 64 GB in hsc_rediscover</t>
+          <t>published Pair_10; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed; 2026-10-22 FIXED: combine-genotypes resubmitted as job 511647 at 32 GB (jobids.tsv cg2), cleanup 344561 + annotate 344562 bmod -w done(511647), report 344564 re-armed; chain resumes on its own; 2026-10-31: calls exist but discover_excluded = 119/240 colonies OOM at the old 32 GB tier2 (48 PD45804 + 71 PD45805); rerun of the 119 at 64 GB in hsc_rediscover; rerun submitted 2026-10-31 06:11 in hsc_rediscover (121 discovery files reused, PT_RESTAGE=1, CI 64 GB): sd 498556, sdr 498558, ci 498563, gt 498565, gtr 498568, cg 498573, cu 498579, an 498585, rp 498587; results -&gt; /nfs/users/nfs_j/jd43/results/hsc_rediscover/Pair28_PD45804_PD45805</t>
         </is>
       </c>
     </row>
@@ -1944,12 +1944,12 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE: discovery OOM</t>
+          <t>rerun running</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair28_PD45804_PD45805/Pair28_PD45804_PD45805</t>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_rediscover/Pair28_PD45804_PD45805/Pair28_PD45804_PD45805</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1975,7 +1975,7 @@
       </c>
       <c r="T20" s="3" t="inlineStr">
         <is>
-          <t>published Pair_10; recipient is a CML patient (BCR::ABL1 pre-HSCT), Flu-Bu-ATG; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed; 2026-10-22 FIXED: combine-genotypes resubmitted as job 511647 at 32 GB (jobids.tsv cg2), cleanup 344561 + annotate 344562 bmod -w done(511647), report 344564 re-armed; chain resumes on its own; 2026-10-31: calls exist but discover_excluded = 119/240 colonies OOM at the old 32 GB tier2 (48 PD45804 + 71 PD45805); rerun of the 119 at 64 GB in hsc_rediscover</t>
+          <t>published Pair_10; recipient is a CML patient (BCR::ABL1 pre-HSCT), Flu-Bu-ATG; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed; 2026-10-22 FIXED: combine-genotypes resubmitted as job 511647 at 32 GB (jobids.tsv cg2), cleanup 344561 + annotate 344562 bmod -w done(511647), report 344564 re-armed; chain resumes on its own; 2026-10-31: calls exist but discover_excluded = 119/240 colonies OOM at the old 32 GB tier2 (48 PD45804 + 71 PD45805); rerun of the 119 at 64 GB in hsc_rediscover; rerun submitted 2026-10-31 06:11 in hsc_rediscover (121 discovery files reused, PT_RESTAGE=1, CI 64 GB): sd 498556, sdr 498558, ci 498563, gt 498565, gtr 498568, cg 498573, cu 498579, an 498585, rp 498587; results -&gt; /nfs/users/nfs_j/jd43/results/hsc_rediscover/Pair28_PD45804_PD45805</t>
         </is>
       </c>
     </row>
@@ -2016,12 +2016,12 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE: discovery OOM</t>
+          <t>rerun running</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair31_PD45806_PD45807/Pair31_PD45806_PD45807</t>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_rediscover/Pair31_PD45806_PD45807/Pair31_PD45806_PD45807</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -2065,7 +2065,7 @@
       </c>
       <c r="T21" s="3" t="inlineStr">
         <is>
-          <t>published Pair_6; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058); chain finished 2026-10-21 (Pair31.somatic.xlsx on NFS), not yet copied to ~/Documents/hsc_results; 2026-10-31: discover_excluded = 142/192 colonies OOM at the old 32 GB tier2 (64 PD45806 + 78 PD45807) -&gt; local results cover discovery in only 50 colonies; rerun of the 142 at 64 GB in hsc_rediscover (old discovery hard-linked)</t>
+          <t>published Pair_6; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058); chain finished 2026-10-21 (Pair31.somatic.xlsx on NFS), not yet copied to ~/Documents/hsc_results; 2026-10-31: discover_excluded = 142/192 colonies OOM at the old 32 GB tier2 (64 PD45806 + 78 PD45807) -&gt; local results cover discovery in only 50 colonies; rerun of the 142 at 64 GB in hsc_rediscover (old discovery hard-linked); rerun submitted 2026-10-31 06:10 in hsc_rediscover (50 discovery files reused, PT_RESTAGE=1, CI 64 GB): sd 498515, sdr 498526, ci 498530, gt 498533, gtr 498536, cg 498539, cu 498541, an 498545, rp 498548; results -&gt; /nfs/users/nfs_j/jd43/results/hsc_rediscover/Pair31_PD45806_PD45807</t>
         </is>
       </c>
     </row>
@@ -2106,12 +2106,12 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>INCOMPLETE: discovery OOM</t>
+          <t>rerun running</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair31_PD45806_PD45807/Pair31_PD45806_PD45807</t>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_rediscover/Pair31_PD45806_PD45807/Pair31_PD45806_PD45807</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -2155,7 +2155,7 @@
       </c>
       <c r="T22" s="3" t="inlineStr">
         <is>
-          <t>published Pair_6; recipient: cisplatin for oesophageal cancer after HSCT; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058); chain finished 2026-10-21 (Pair31.somatic.xlsx on NFS), not yet copied to ~/Documents/hsc_results; 2026-10-31: discover_excluded = 142/192 colonies OOM at the old 32 GB tier2 (64 PD45806 + 78 PD45807) -&gt; local results cover discovery in only 50 colonies; rerun of the 142 at 64 GB in hsc_rediscover (old discovery hard-linked)</t>
+          <t>published Pair_6; recipient: cisplatin for oesophageal cancer after HSCT; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058); chain finished 2026-10-21 (Pair31.somatic.xlsx on NFS), not yet copied to ~/Documents/hsc_results; 2026-10-31: discover_excluded = 142/192 colonies OOM at the old 32 GB tier2 (64 PD45806 + 78 PD45807) -&gt; local results cover discovery in only 50 colonies; rerun of the 142 at 64 GB in hsc_rediscover (old discovery hard-linked); rerun submitted 2026-10-31 06:10 in hsc_rediscover (50 discovery files reused, PT_RESTAGE=1, CI 64 GB): sd 498515, sdr 498526, ci 498530, gt 498533, gtr 498536, cg 498539, cu 498541, an 498545, rp 498548; results -&gt; /nfs/users/nfs_j/jd43/results/hsc_rediscover/Pair31_PD45806_PD45807</t>
         </is>
       </c>
     </row>
@@ -4683,7 +4683,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-31 07:10</t>
+          <t>refreshed 2026-10-31 07:11</t>
         </is>
       </c>
     </row>
@@ -6252,12 +6252,12 @@
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>INCOMPLETE: discovery OOM</t>
+          <t>rerun running</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair28_PD45804_PD45805/Pair28_PD45804_PD45805</t>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_rediscover/Pair28_PD45804_PD45805/Pair28_PD45804_PD45805</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -6283,7 +6283,7 @@
       </c>
       <c r="T19" t="inlineStr">
         <is>
-          <t>published Pair_10; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed; 2026-10-22 FIXED: combine-genotypes resubmitted as job 511647 at 32 GB (jobids.tsv cg2), cleanup 344561 + annotate 344562 bmod -w done(511647), report 344564 re-armed; chain resumes on its own; 2026-10-31: calls exist but discover_excluded = 119/240 colonies OOM at the old 32 GB tier2 (48 PD45804 + 71 PD45805); rerun of the 119 at 64 GB in hsc_rediscover</t>
+          <t>published Pair_10; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed; 2026-10-22 FIXED: combine-genotypes resubmitted as job 511647 at 32 GB (jobids.tsv cg2), cleanup 344561 + annotate 344562 bmod -w done(511647), report 344564 re-armed; chain resumes on its own; 2026-10-31: calls exist but discover_excluded = 119/240 colonies OOM at the old 32 GB tier2 (48 PD45804 + 71 PD45805); rerun of the 119 at 64 GB in hsc_rediscover; rerun submitted 2026-10-31 06:11 in hsc_rediscover (121 discovery files reused, PT_RESTAGE=1, CI 64 GB): sd 498556, sdr 498558, ci 498563, gt 498565, gtr 498568, cg 498573, cu 498579, an 498585, rp 498587; results -&gt; /nfs/users/nfs_j/jd43/results/hsc_rediscover/Pair28_PD45804_PD45805</t>
         </is>
       </c>
     </row>
@@ -6324,12 +6324,12 @@
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>INCOMPLETE: discovery OOM</t>
+          <t>rerun running</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair28_PD45804_PD45805/Pair28_PD45804_PD45805</t>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_rediscover/Pair28_PD45804_PD45805/Pair28_PD45804_PD45805</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -6355,7 +6355,7 @@
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>published Pair_10; recipient is a CML patient (BCR::ABL1 pre-HSCT), Flu-Bu-ATG; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed; 2026-10-22 FIXED: combine-genotypes resubmitted as job 511647 at 32 GB (jobids.tsv cg2), cleanup 344561 + annotate 344562 bmod -w done(511647), report 344564 re-armed; chain resumes on its own; 2026-10-31: calls exist but discover_excluded = 119/240 colonies OOM at the old 32 GB tier2 (48 PD45804 + 71 PD45805); rerun of the 119 at 64 GB in hsc_rediscover</t>
+          <t>published Pair_10; recipient is a CML patient (BCR::ABL1 pre-HSCT), Flu-Bu-ATG; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344555, cleanup 344561, stage+discover waits on ended(344552), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair28_PD45804_PD45805; 2026-10-22: combine_gt job 344560 died 2026-10-21 (240 colonies, 8 GB cap, Delta Memory negative = memory kill), no calls; cleanup 344561 unsatisfiable -&gt; Pair38 and the 11 units behind it blocked (9485 PEND); fix = resubmit combine-genotypes at 32 GB + bmod 344561/344562 to done(new), 344564 re-armed; 2026-10-22 FIXED: combine-genotypes resubmitted as job 511647 at 32 GB (jobids.tsv cg2), cleanup 344561 + annotate 344562 bmod -w done(511647), report 344564 re-armed; chain resumes on its own; 2026-10-31: calls exist but discover_excluded = 119/240 colonies OOM at the old 32 GB tier2 (48 PD45804 + 71 PD45805); rerun of the 119 at 64 GB in hsc_rediscover; rerun submitted 2026-10-31 06:11 in hsc_rediscover (121 discovery files reused, PT_RESTAGE=1, CI 64 GB): sd 498556, sdr 498558, ci 498563, gt 498565, gtr 498568, cg 498573, cu 498579, an 498585, rp 498587; results -&gt; /nfs/users/nfs_j/jd43/results/hsc_rediscover/Pair28_PD45804_PD45805</t>
         </is>
       </c>
     </row>
@@ -6396,12 +6396,12 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>INCOMPLETE: discovery OOM</t>
+          <t>rerun running</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair31_PD45806_PD45807/Pair31_PD45806_PD45807</t>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_rediscover/Pair31_PD45806_PD45807/Pair31_PD45806_PD45807</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -6445,7 +6445,7 @@
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>published Pair_6; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058); chain finished 2026-10-21 (Pair31.somatic.xlsx on NFS), not yet copied to ~/Documents/hsc_results; 2026-10-31: discover_excluded = 142/192 colonies OOM at the old 32 GB tier2 (64 PD45806 + 78 PD45807) -&gt; local results cover discovery in only 50 colonies; rerun of the 142 at 64 GB in hsc_rediscover (old discovery hard-linked)</t>
+          <t>published Pair_6; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058); chain finished 2026-10-21 (Pair31.somatic.xlsx on NFS), not yet copied to ~/Documents/hsc_results; 2026-10-31: discover_excluded = 142/192 colonies OOM at the old 32 GB tier2 (64 PD45806 + 78 PD45807) -&gt; local results cover discovery in only 50 colonies; rerun of the 142 at 64 GB in hsc_rediscover (old discovery hard-linked); rerun submitted 2026-10-31 06:10 in hsc_rediscover (50 discovery files reused, PT_RESTAGE=1, CI 64 GB): sd 498515, sdr 498526, ci 498530, gt 498533, gtr 498536, cg 498539, cu 498541, an 498545, rp 498548; results -&gt; /nfs/users/nfs_j/jd43/results/hsc_rediscover/Pair31_PD45806_PD45807</t>
         </is>
       </c>
     </row>
@@ -6486,12 +6486,12 @@
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>INCOMPLETE: discovery OOM</t>
+          <t>rerun running</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair31_PD45806_PD45807/Pair31_PD45806_PD45807</t>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_rediscover/Pair31_PD45806_PD45807/Pair31_PD45806_PD45807</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -6535,7 +6535,7 @@
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>published Pair_6; recipient: cisplatin for oesophageal cancer after HSCT; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058); chain finished 2026-10-21 (Pair31.somatic.xlsx on NFS), not yet copied to ~/Documents/hsc_results; 2026-10-31: discover_excluded = 142/192 colonies OOM at the old 32 GB tier2 (64 PD45806 + 78 PD45807) -&gt; local results cover discovery in only 50 colonies; rerun of the 142 at 64 GB in hsc_rediscover (old discovery hard-linked)</t>
+          <t>published Pair_6; recipient: cisplatin for oesophageal cancer after HSCT; added 2026-10-15 (whole transplant cohort); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344542, cleanup 344552, stage+discover waits on ended(344539), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair31_PD45806_PD45807; 2026-10-20: chain STALLED here -- 188/192 sd OOM at 4000 MB (peak 5.1 GB), sdr 344543 died on 'Bad job name' (long tier2 index list; fixed e0f23ac); resubmitted sdr as 6992, ci 344545 bmod'ed to done(6992); pending sd arrays of all later units bmod'ed to 8000 MB (hsc_run default now 8000, 4f9f058); chain finished 2026-10-21 (Pair31.somatic.xlsx on NFS), not yet copied to ~/Documents/hsc_results; 2026-10-31: discover_excluded = 142/192 colonies OOM at the old 32 GB tier2 (64 PD45806 + 78 PD45807) -&gt; local results cover discovery in only 50 colonies; rerun of the 142 at 64 GB in hsc_rediscover (old discovery hard-linked); rerun submitted 2026-10-31 06:10 in hsc_rediscover (50 discovery files reused, PT_RESTAGE=1, CI 64 GB): sd 498515, sdr 498526, ci 498530, gt 498533, gtr 498536, cg 498539, cu 498541, an 498545, rp 498548; results -&gt; /nfs/users/nfs_j/jd43/results/hsc_rediscover/Pair31_PD45806_PD45807</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Run tracker: PD47703 results local
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -779,7 +779,7 @@
       </c>
       <c r="T3" s="3" t="inlineStr">
         <is>
-          <t>old-pipeline results only (~/Documents/retrotransposons_sanger/results/PD47703); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344581, cleanup 344588, stage+discover waits on ended(344578), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD47703; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 259/259 discovered + genotyped, calls present (report status: see fetch)</t>
+          <t>old-pipeline results only (~/Documents/retrotransposons_sanger/results/PD47703); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344581, cleanup 344588, stage+discover waits on ended(344578), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD47703; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 259/259 discovered + genotyped, no discovery exclusions; results copied 2026-10-31 to ~/Documents/hsc_results/PD47703</t>
         </is>
       </c>
     </row>
@@ -4683,7 +4683,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-31 07:11</t>
+          <t>refreshed 2026-10-31 07:12</t>
         </is>
       </c>
     </row>
@@ -5159,7 +5159,7 @@
       </c>
       <c r="T3" t="inlineStr">
         <is>
-          <t>old-pipeline results only (~/Documents/retrotransposons_sanger/results/PD47703); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344581, cleanup 344588, stage+discover waits on ended(344578), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD47703; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 259/259 discovered + genotyped, calls present (report status: see fetch)</t>
+          <t>old-pipeline results only (~/Documents/retrotransposons_sanger/results/PD47703); chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344581, cleanup 344588, stage+discover waits on ended(344578), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/PD47703; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 259/259 discovered + genotyped, no discovery exclusions; results copied 2026-10-31 to ~/Documents/hsc_results/PD47703</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Run tracker: Pair38 rerun submitted in hsc_rediscover (CI 128 GB)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/patients/run_tracker.xlsx
+++ b/patients/run_tracker.xlsx
@@ -1192,12 +1192,12 @@
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>failed (combine)</t>
+          <t>rerun running</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair38_PD45808_PD45809/Pair38_PD45808_PD45809</t>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_rediscover/Pair38_PD45808_PD45809/Pair38_PD45808_PD45809</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1223,7 +1223,7 @@
       </c>
       <c r="T9" s="3" t="inlineStr">
         <is>
-          <t>chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 64 GB rediscovery (sd 549176/sdr 549178) finished 2026-10-27 21:45, then combine 344574 TERM_MEMLIMIT at 16 GB (6.46M insertions) 2026-10-27 22:16; 3 colonies discovery "error"; rerun in hsc_rediscover with CI_MEM 128 GB; gate 549226 logged "unknown" (EXIT purged before it ran), killed the unit and deleted its staged BAMs, released PD47703-&gt;Pair40</t>
+          <t>chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 64 GB rediscovery (sd 549176/sdr 549178) finished 2026-10-27 21:45, then combine 344574 TERM_MEMLIMIT at 16 GB (6.46M insertions) 2026-10-27 22:16; 3 colonies discovery "error"; rerun in hsc_rediscover with CI_MEM 128 GB; gate 549226 logged "unknown" (EXIT purged before it ran), killed the unit and deleted its staged BAMs, released PD47703-&gt;Pair40; rerun submitted 2026-10-31 06:12 in hsc_rediscover (249 discovery files reused, PT_RESTAGE=1, CI 128 GB): sd 498671, sdr 498672, ci 498673, gt 498675, gtr 498680, cg 498684, cu 498687, an 498690, rp 498695; results -&gt; /nfs/users/nfs_j/jd43/results/hsc_rediscover/Pair38_PD45808_PD45809</t>
         </is>
       </c>
     </row>
@@ -1268,12 +1268,12 @@
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>failed (combine)</t>
+          <t>rerun running</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair38_PD45808_PD45809/Pair38_PD45808_PD45809</t>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_rediscover/Pair38_PD45808_PD45809/Pair38_PD45808_PD45809</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1299,7 +1299,7 @@
       </c>
       <c r="T10" s="3" t="inlineStr">
         <is>
-          <t>chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 64 GB rediscovery (sd 549176/sdr 549178) finished 2026-10-27 21:45, then combine 344574 TERM_MEMLIMIT at 16 GB (6.46M insertions) 2026-10-27 22:16; 3 colonies discovery "error"; rerun in hsc_rediscover with CI_MEM 128 GB; gate 549226 logged "unknown" (EXIT purged before it ran), killed the unit and deleted its staged BAMs, released PD47703-&gt;Pair40</t>
+          <t>chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 64 GB rediscovery (sd 549176/sdr 549178) finished 2026-10-27 21:45, then combine 344574 TERM_MEMLIMIT at 16 GB (6.46M insertions) 2026-10-27 22:16; 3 colonies discovery "error"; rerun in hsc_rediscover with CI_MEM 128 GB; gate 549226 logged "unknown" (EXIT purged before it ran), killed the unit and deleted its staged BAMs, released PD47703-&gt;Pair40; rerun submitted 2026-10-31 06:12 in hsc_rediscover (249 discovery files reused, PT_RESTAGE=1, CI 128 GB): sd 498671, sdr 498672, ci 498673, gt 498675, gtr 498680, cg 498684, cu 498687, an 498690, rp 498695; results -&gt; /nfs/users/nfs_j/jd43/results/hsc_rediscover/Pair38_PD45808_PD45809</t>
         </is>
       </c>
     </row>
@@ -4683,7 +4683,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>refreshed 2026-10-31 07:12</t>
+          <t>refreshed 2026-10-31 07:14</t>
         </is>
       </c>
     </row>
@@ -5572,12 +5572,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>failed (combine)</t>
+          <t>rerun running</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair38_PD45808_PD45809/Pair38_PD45808_PD45809</t>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_rediscover/Pair38_PD45808_PD45809/Pair38_PD45808_PD45809</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -5603,7 +5603,7 @@
       </c>
       <c r="T9" t="inlineStr">
         <is>
-          <t>chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 64 GB rediscovery (sd 549176/sdr 549178) finished 2026-10-27 21:45, then combine 344574 TERM_MEMLIMIT at 16 GB (6.46M insertions) 2026-10-27 22:16; 3 colonies discovery "error"; rerun in hsc_rediscover with CI_MEM 128 GB; gate 549226 logged "unknown" (EXIT purged before it ran), killed the unit and deleted its staged BAMs, released PD47703-&gt;Pair40</t>
+          <t>chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 64 GB rediscovery (sd 549176/sdr 549178) finished 2026-10-27 21:45, then combine 344574 TERM_MEMLIMIT at 16 GB (6.46M insertions) 2026-10-27 22:16; 3 colonies discovery "error"; rerun in hsc_rediscover with CI_MEM 128 GB; gate 549226 logged "unknown" (EXIT purged before it ran), killed the unit and deleted its staged BAMs, released PD47703-&gt;Pair40; rerun submitted 2026-10-31 06:12 in hsc_rediscover (249 discovery files reused, PT_RESTAGE=1, CI 128 GB): sd 498671, sdr 498672, ci 498673, gt 498675, gtr 498680, cg 498684, cu 498687, an 498690, rp 498695; results -&gt; /nfs/users/nfs_j/jd43/results/hsc_rediscover/Pair38_PD45808_PD45809</t>
         </is>
       </c>
     </row>
@@ -5648,12 +5648,12 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>failed (combine)</t>
+          <t>rerun running</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_foldback2/Pair38_PD45808_PD45809/Pair38_PD45808_PD45809</t>
+          <t>/lustre/scratch126/casm/teams/team273/users/jd43/hsc_rediscover/Pair38_PD45808_PD45809/Pair38_PD45808_PD45809</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -5679,7 +5679,7 @@
       </c>
       <c r="T10" t="inlineStr">
         <is>
-          <t>chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 64 GB rediscovery (sd 549176/sdr 549178) finished 2026-10-27 21:45, then combine 344574 TERM_MEMLIMIT at 16 GB (6.46M insertions) 2026-10-27 22:16; 3 colonies discovery "error"; rerun in hsc_rediscover with CI_MEM 128 GB; gate 549226 logged "unknown" (EXIT purged before it ran), killed the unit and deleted its staged BAMs, released PD47703-&gt;Pair40</t>
+          <t>chain-submitted 2026-10-18 (cluster/hsc_chain.sh), native GRCh37, sd 344569, cleanup 344578, stage+discover waits on ended(344561), results -&gt; /nfs/users/nfs_j/jd43/results/hsc_foldback2/Pair38_PD45808_PD45809; 2026-10-22: was blocked behind Pair28 (cleanup 344561 never satisfied) 10-21..10-22; all pending jobs moved from retired LSF group team273-grp to team273 (bmod -G); cg job raised 8 -&gt; 48 GB in place (bmod -M); 2026-10-31: 64 GB rediscovery (sd 549176/sdr 549178) finished 2026-10-27 21:45, then combine 344574 TERM_MEMLIMIT at 16 GB (6.46M insertions) 2026-10-27 22:16; 3 colonies discovery "error"; rerun in hsc_rediscover with CI_MEM 128 GB; gate 549226 logged "unknown" (EXIT purged before it ran), killed the unit and deleted its staged BAMs, released PD47703-&gt;Pair40; rerun submitted 2026-10-31 06:12 in hsc_rediscover (249 discovery files reused, PT_RESTAGE=1, CI 128 GB): sd 498671, sdr 498672, ci 498673, gt 498675, gtr 498680, cg 498684, cu 498687, an 498690, rp 498695; results -&gt; /nfs/users/nfs_j/jd43/results/hsc_rediscover/Pair38_PD45808_PD45809</t>
         </is>
       </c>
     </row>

</xml_diff>